<commit_message>
AutomaTivio: carteira inclui posições sem data; alocação real volta a ser sobre o PL
- Base Carteira: linhas sem data entram junto com as do mês (eram posições
  atuais: no ALT 90 duas cotas sênior e um caixa; no ALT 180, 11 linhas).
- Alocação real sobre o PL, como a planilha da gestão (ALT Light alavancado,
  126%). Setembro fecha com as tabelas: ALT 180 100,3%, ALT 90 100,7%.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -1483,7 +1483,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>[{'n': 'FIDCs Cota Sênior', 'p': 58.5}, {'n': 'FIDCs Cota Mezanino', 'p': 20.6}, {'n': 'Liquidez', 'p': 10.0}, {'n': 'Crédito Privado', 'p': 4.2}, {'n': 'Fiagro', 'p': 3.9}, {'n': 'Precatório', 'p': 2.7}]</t>
+          <t>[{'n': 'FIDCs Cota Sênior', 'p': 49.3}, {'n': 'FIDCs Cota Mezanino', 'p': 27.0}, {'n': 'Liquidez', 'p': 9.1}, {'n': 'Crédito Estruturado', 'p': 5.5}, {'n': 'Crédito Privado', 'p': 3.4}, {'n': 'Fiagro', 'p': 3.2}, {'n': 'Precatório', 'p': 2.8}]</t>
         </is>
       </c>
     </row>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>[{'n': 'FIDCs Cota Sênior', 'p': 74.2}, {'n': 'Liquidez', 'p': 16.6}, {'n': 'Crédito Privado', 'p': 3.9}, {'n': 'Crédito Estruturado', 'p': 3.1}, {'n': 'Fiagro', 'p': 1.6}, {'n': 'FIDCs Cota Mezanino', 'p': 0.6}]</t>
+          <t>[{'n': 'FIDCs Cota Sênior', 'p': 76.7}, {'n': 'Liquidez', 'p': 15.7}, {'n': 'Crédito Privado', 'p': 3.5}, {'n': 'Crédito Estruturado', 'p': 2.8}, {'n': 'Fiagro', 'p': 1.5}, {'n': 'FIDCs Cota Mezanino', 'p': 0.5}]</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>[{'n': 'Bancário', 'p': 31.4}, {'n': 'Liquidez', 'p': 27.3}, {'n': 'FIDCs Cota Sênior', 'p': 20.5}, {'n': 'Crédito Privado', 'p': 18.9}, {'n': 'FIP', 'p': 1.9}]</t>
+          <t>[{'n': 'Bancário', 'p': 39.6}, {'n': 'Liquidez', 'p': 34.4}, {'n': 'FIDCs Cota Sênior', 'p': 25.9}, {'n': 'Crédito Privado', 'p': 23.8}, {'n': 'FIP', 'p': 2.4}]</t>
         </is>
       </c>
     </row>
@@ -2698,7 +2698,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>{'total': '62', 'top': [{'p': '23%', 'n': 'financeiro'}, {'p': '12%', 'n': 'FIDC'}, {'p': '5%', 'n': 'energia elétrica'}]}</t>
+          <t>{'total': '70', 'top': [{'p': '28%', 'n': 'financeiro'}, {'p': '13%', 'n': 'FIDC'}, {'p': '7%', 'n': 'energia elétrica'}]}</t>
         </is>
       </c>
     </row>
@@ -2725,7 +2725,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>0,83</t>
+          <t>0,91</t>
         </is>
       </c>
     </row>
@@ -2752,7 +2752,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>1,53</t>
+          <t>1,74</t>
         </is>
       </c>
     </row>
@@ -11198,7 +11198,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1966288</v>
+        <v>1966259</v>
       </c>
     </row>
     <row r="6">
@@ -11213,7 +11213,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>838964</v>
+        <v>838981</v>
       </c>
     </row>
     <row r="7">
@@ -11228,7 +11228,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1985741</v>
+        <v>1985711</v>
       </c>
     </row>
     <row r="8">
@@ -11303,7 +11303,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>817919</v>
+        <v>817905</v>
       </c>
     </row>
     <row r="13">
@@ -11318,7 +11318,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1942899</v>
+        <v>1942870</v>
       </c>
     </row>
     <row r="14">
@@ -11333,7 +11333,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>827554</v>
+        <v>827596</v>
       </c>
     </row>
     <row r="15">
@@ -11348,7 +11348,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1956927</v>
+        <v>1956665</v>
       </c>
     </row>
     <row r="16">
@@ -11363,7 +11363,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>618585</v>
+        <v>618935</v>
       </c>
     </row>
     <row r="17">
@@ -11378,7 +11378,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>295700</v>
+        <v>296290</v>
       </c>
     </row>
     <row r="18">
@@ -11393,7 +11393,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>617302</v>
+        <v>617071</v>
       </c>
     </row>
     <row r="19">
@@ -11408,7 +11408,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>290569</v>
+        <v>291161</v>
       </c>
     </row>
     <row r="20">
@@ -11423,7 +11423,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>612955</v>
+        <v>612757</v>
       </c>
     </row>
     <row r="21">
@@ -11438,7 +11438,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>284115</v>
+        <v>284097</v>
       </c>
     </row>
     <row r="22">
@@ -11453,7 +11453,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>830146</v>
+        <v>830104</v>
       </c>
     </row>
     <row r="23">
@@ -11468,7 +11468,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1960127</v>
+        <v>1960267</v>
       </c>
     </row>
     <row r="24">
@@ -11483,7 +11483,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>832464</v>
+        <v>832191</v>
       </c>
     </row>
     <row r="25">
@@ -11498,7 +11498,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1968015</v>
+        <v>1968199</v>
       </c>
     </row>
     <row r="26">
@@ -11513,7 +11513,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>830848</v>
+        <v>830709</v>
       </c>
     </row>
     <row r="27">
@@ -11528,7 +11528,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1959014</v>
+        <v>1958853</v>
       </c>
     </row>
     <row r="28">
@@ -11543,7 +11543,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3222755</v>
+        <v>3222930</v>
       </c>
     </row>
     <row r="29">
@@ -11558,7 +11558,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1060034</v>
+        <v>1060433</v>
       </c>
     </row>
     <row r="30">
@@ -11618,7 +11618,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>114657</v>
+        <v>114693</v>
       </c>
     </row>
     <row r="34">

</xml_diff>

<commit_message>
AutomaTivio: ALT Light fecha 100% tirando a alavancagem só da linha do Caixa
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -1861,7 +1861,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>[{'n': 'Bancário', 'p': 39.6}, {'n': 'Liquidez', 'p': 34.4}, {'n': 'FIDCs Cota Sênior', 'p': 25.9}, {'n': 'Crédito Privado', 'p': 23.8}, {'n': 'FIP', 'p': 2.4}]</t>
+          <t>[{'n': 'Bancário', 'p': 39.6}, {'n': 'FIDCs Cota Sênior', 'p': 25.9}, {'n': 'Crédito Privado', 'p': 23.8}, {'n': 'Liquidez', 'p': 8.2}, {'n': 'FIP', 'p': 2.4}]</t>
         </is>
       </c>
     </row>
@@ -11198,7 +11198,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1966259</v>
+        <v>1966288</v>
       </c>
     </row>
     <row r="6">
@@ -11363,7 +11363,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>618935</v>
+        <v>618771</v>
       </c>
     </row>
     <row r="17">
@@ -11393,7 +11393,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>617071</v>
+        <v>617212</v>
       </c>
     </row>
     <row r="19">
@@ -11408,7 +11408,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>291161</v>
+        <v>290880</v>
       </c>
     </row>
     <row r="20">
@@ -11423,7 +11423,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>612757</v>
+        <v>612974</v>
       </c>
     </row>
     <row r="21">
@@ -11438,7 +11438,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>284097</v>
+        <v>284126</v>
       </c>
     </row>
     <row r="22">
@@ -11453,7 +11453,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>830104</v>
+        <v>830146</v>
       </c>
     </row>
     <row r="23">
@@ -11483,7 +11483,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>832191</v>
+        <v>832464</v>
       </c>
     </row>
     <row r="25">
@@ -11498,7 +11498,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1968199</v>
+        <v>1968015</v>
       </c>
     </row>
     <row r="26">
@@ -11513,7 +11513,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>830709</v>
+        <v>830848</v>
       </c>
     </row>
     <row r="27">
@@ -11528,7 +11528,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1958853</v>
+        <v>1959014</v>
       </c>
     </row>
     <row r="28">
@@ -11558,7 +11558,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1060433</v>
+        <v>1060482</v>
       </c>
     </row>
     <row r="30">
@@ -11618,7 +11618,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>114693</v>
+        <v>114692</v>
       </c>
     </row>
     <row r="34">

</xml_diff>

<commit_message>
AutomaTivio: posts com logos horizontais e Infra Plus CDI; abertura automática dos ALT; post sem casa decimal
- Posts de Crédito Privado e Estruturado: logos horizontais de assets/logos.
- Post de Crédito Privado: card do Infra Plus CDI (página 8); sem 12M, o
  destaque vira "Desde o início".
- Boxes de Rentabilidade dos posts sem casa decimal ("100%"), exceto Infra
  Plus e Infra Plus CDI.
- ALT 180, 90 e Light (`abertura: alt`): o 1º parágrafo do comentário é a
  abertura padrão com os números da tabela; o anualizado é o "%" desde o
  início da tabela (ALT 180 de setembro: 130,15%).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E161"/>
+  <dimension ref="A1:E166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1402,7 +1402,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>123,25%</t>
+          <t>123%</t>
         </is>
       </c>
     </row>
@@ -1419,17 +1419,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>120%</t>
+          <t>[{'n': 'FIDCs Cotas Sênior', 'p': 49.6}, {'n': 'FIDCs Cotas Mezanino', 'p': 27.5}, {'n': 'Liquidez', 'p': 9.3}, {'n': 'Crédito Estruturado', 'p': 5.5}, {'n': 'Crédito Privado', 'p': 3.5}, {'n': 'Precatório', 'p': 2.8}, {'n': 'Fiagro', 'p': 2.0}]</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>120,09%</t>
+          <t>[{'n': 'FIDCs Cota Sênior', 'p': 49.3}, {'n': 'FIDCs Cota Mezanino', 'p': 27.0}, {'n': 'Liquidez', 'p': 9.1}, {'n': 'Crédito Estruturado', 'p': 5.5}, {'n': 'Crédito Privado', 'p': 3.4}, {'n': 'Fiagro', 'p': 3.2}, {'n': 'Precatório', 'p': 2.8}]</t>
         </is>
       </c>
     </row>
@@ -1446,17 +1446,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>119%</t>
+          <t>Taxa de administração e gestão: 1,15% a.a. Taxa de performance: 20% do que exceder do CDI. Resgate: D+180.</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>119,45%</t>
+          <t>Taxa global: 1,15% a.a. Taxa de performance: 20% do que exceder do CDI. Resgate: D+180.</t>
         </is>
       </c>
     </row>
@@ -1468,22 +1468,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>alt180</t>
+          <t>alt90</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>b1val</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>[{'n': 'FIDCs Cotas Sênior', 'p': 49.6}, {'n': 'FIDCs Cotas Mezanino', 'p': 27.5}, {'n': 'Liquidez', 'p': 9.3}, {'n': 'Crédito Estruturado', 'p': 5.5}, {'n': 'Crédito Privado', 'p': 3.5}, {'n': 'Precatório', 'p': 2.8}, {'n': 'Fiagro', 'p': 2.0}]</t>
+          <t>R$ 19.936.394,95</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>[{'n': 'FIDCs Cota Sênior', 'p': 49.3}, {'n': 'FIDCs Cota Mezanino', 'p': 27.0}, {'n': 'Liquidez', 'p': 9.1}, {'n': 'Crédito Estruturado', 'p': 5.5}, {'n': 'Crédito Privado', 'p': 3.4}, {'n': 'Fiagro', 'p': 3.2}, {'n': 'Precatório', 'p': 2.8}]</t>
+          <t>R$ 20.954.147,09</t>
         </is>
       </c>
     </row>
@@ -1495,22 +1495,22 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>alt180</t>
+          <t>alt90</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>b2val</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Taxa de administração e gestão: 1,15% a.a. Taxa de performance: 20% do que exceder do CDI. Resgate: D+180.</t>
+          <t>R$ 14.275.935,66</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Taxa global: 1,15% a.a. Taxa de performance: 20% do que exceder do CDI. Resgate: D+180.</t>
+          <t>R$ 16.917.619,85</t>
         </is>
       </c>
     </row>
@@ -1527,17 +1527,17 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>b1val</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>R$ 19.936.394,95</t>
+          <t>114%</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>R$ 20.954.147,09</t>
+          <t>112%</t>
         </is>
       </c>
     </row>
@@ -1554,17 +1554,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>b2val</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>R$ 14.275.935,66</t>
+          <t>112%</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>R$ 16.917.619,85</t>
+          <t>108%</t>
         </is>
       </c>
     </row>
@@ -1581,17 +1581,17 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>114%</t>
+          <t>[{'n': 'FIDCs Cotas Sênior', 'p': 81.3}, {'n': 'Liquidez', 'p': 11.9}, {'n': 'Crédito Privado', 'p': 3.6}, {'n': 'Crédito Estruturado', 'p': 2.8}, {'n': 'FIDC Mezanino', 'p': 0.6}]</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>112,21%</t>
+          <t>[{'n': 'FIDCs Cota Sênior', 'p': 76.7}, {'n': 'Liquidez', 'p': 15.7}, {'n': 'Crédito Privado', 'p': 3.5}, {'n': 'Crédito Estruturado', 'p': 2.8}, {'n': 'Fiagro', 'p': 1.5}, {'n': 'FIDCs Cota Mezanino', 'p': 0.5}]</t>
         </is>
       </c>
     </row>
@@ -1608,17 +1608,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>111%</t>
+          <t>Taxa de administração e gestão: 1,25% a.a. Taxa de performance: 10% do que exceder do CDI. Resgate: D+90.</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>111,24%</t>
+          <t>Taxa global: 1,25% a.a. Taxa de performance: 10% do que exceder do CDI. Resgate: D+90.</t>
         </is>
       </c>
     </row>
@@ -1630,22 +1630,22 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>alt90</t>
+          <t>altlight</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>b1val</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>112%</t>
+          <t>R$ 26.861.672,93</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>108,27%</t>
+          <t>R$ 20.571.241,16</t>
         </is>
       </c>
     </row>
@@ -1657,22 +1657,22 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>alt90</t>
+          <t>altlight</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>b2val</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>[{'n': 'FIDCs Cotas Sênior', 'p': 81.3}, {'n': 'Liquidez', 'p': 11.9}, {'n': 'Crédito Privado', 'p': 3.6}, {'n': 'Crédito Estruturado', 'p': 2.8}, {'n': 'FIDC Mezanino', 'p': 0.6}]</t>
+          <t>R$ 17.309.791,01</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>[{'n': 'FIDCs Cota Sênior', 'p': 76.7}, {'n': 'Liquidez', 'p': 15.7}, {'n': 'Crédito Privado', 'p': 3.5}, {'n': 'Crédito Estruturado', 'p': 2.8}, {'n': 'Fiagro', 'p': 1.5}, {'n': 'FIDCs Cota Mezanino', 'p': 0.5}]</t>
+          <t>R$ 19.052.692,02</t>
         </is>
       </c>
     </row>
@@ -1684,22 +1684,22 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>alt90</t>
+          <t>altlight</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Taxa de administração e gestão: 1,25% a.a. Taxa de performance: 10% do que exceder do CDI. Resgate: D+90.</t>
+          <t>116%</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Taxa global: 1,25% a.a. Taxa de performance: 10% do que exceder do CDI. Resgate: D+90.</t>
+          <t>109%</t>
         </is>
       </c>
     </row>
@@ -1716,17 +1716,17 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>b1val</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>R$ 26.861.672,93</t>
+          <t>107%</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>R$ 20.571.241,16</t>
+          <t>101%</t>
         </is>
       </c>
     </row>
@@ -1743,17 +1743,17 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>b2val</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>R$ 17.309.791,01</t>
+          <t>101%</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>R$ 19.052.692,02</t>
+          <t>95%</t>
         </is>
       </c>
     </row>
@@ -1770,17 +1770,17 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>116%</t>
+          <t>[{'n': 'Bancário', 'p': 40.8}, {'n': 'Crédito Privado', 'p': 25.6}, {'n': 'FIDCs Cotas Sênior', 'p': 24.0}, {'n': 'Liquidez', 'p': 7.8}, {'n': 'FIP', 'p': 1.9}]</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>109,18%</t>
+          <t>[{'n': 'Bancário', 'p': 39.6}, {'n': 'FIDCs Cota Sênior', 'p': 25.9}, {'n': 'Crédito Privado', 'p': 23.8}, {'n': 'Liquidez', 'p': 8.2}, {'n': 'FIP', 'p': 2.4}]</t>
         </is>
       </c>
     </row>
@@ -1797,17 +1797,17 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>107%</t>
+          <t>Taxa de administração e gestão: 1,15% a.a. Taxa de performance: 15% do retorno que exceder CDI+0,65%.</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>101,22%</t>
+          <t>Taxa global: 1,15% a.a. Taxa de performance: 15% do retorno que exceder CDI+0,65%.</t>
         </is>
       </c>
     </row>
@@ -1819,22 +1819,22 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>altlight</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>101%</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>95,47%</t>
+          <t>30/09/2026</t>
         </is>
       </c>
     </row>
@@ -1846,22 +1846,22 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>altlight</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>[{'n': 'Bancário', 'p': 40.8}, {'n': 'Crédito Privado', 'p': 25.6}, {'n': 'FIDCs Cotas Sênior', 'p': 24.0}, {'n': 'Liquidez', 'p': 7.8}, {'n': 'FIP', 'p': 1.9}]</t>
+          <t>Julho de 2026</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>[{'n': 'Bancário', 'p': 39.6}, {'n': 'FIDCs Cota Sênior', 'p': 25.9}, {'n': 'Crédito Privado', 'p': 23.8}, {'n': 'Liquidez', 'p': 8.2}, {'n': 'FIP', 'p': 2.4}]</t>
+          <t>Setembro de 2026</t>
         </is>
       </c>
     </row>
@@ -1873,22 +1873,22 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>altlight</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Taxa de administração e gestão: 1,15% a.a. Taxa de performance: 15% do retorno que exceder CDI+0,65%.</t>
+          <t>julho de 2026</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Taxa global: 1,15% a.a. Taxa de performance: 15% do retorno que exceder CDI+0,65%.</t>
+          <t>setembro de 2026</t>
         </is>
       </c>
     </row>
@@ -1910,12 +1910,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>31/07/2026</t>
+          <t>JULHO DE 2026</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>SETEMBRO DE 2026</t>
         </is>
       </c>
     </row>
@@ -1937,12 +1937,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Julho de 2026</t>
+          <t>Julho 2026</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Setembro de 2026</t>
+          <t>Setembro 2026</t>
         </is>
       </c>
     </row>
@@ -1964,12 +1964,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>julho de 2026</t>
+          <t>-jul26</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>setembro de 2026</t>
+          <t>-set26</t>
         </is>
       </c>
     </row>
@@ -1991,12 +1991,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>JULHO DE 2026</t>
+          <t>const ATUAL=6;</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>SETEMBRO DE 2026</t>
+          <t>const ATUAL=8;</t>
         </is>
       </c>
     </row>
@@ -2013,98 +2013,98 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>libs de exportação</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Julho 2026</t>
+          <t>CDN</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Setembro 2026</t>
+          <t>4 referências → vendor/ local (CDN como reserva)</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>tivio-post-credito-privado.html</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>banks</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>-jul26</t>
+          <t>101%</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>-set26</t>
+          <t>100%</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>tivio-post-credito-privado.html</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>banks</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>pl</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>const ATUAL=6;</t>
+          <t>R$ 1.698.520.740,05</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>const ATUAL=8;</t>
+          <t>R$ 1.826.931.618,96</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>tivio-post-credito-privado.html</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>banks</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>libs de exportação</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>CDN</t>
+          <t>R$ 1.397.203.402,03</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>4 referências → vendor/ local (CDN como reserva)</t>
+          <t>R$ 1.510.000.753,13</t>
         </is>
       </c>
     </row>
@@ -2121,17 +2121,17 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>{'total': '76', 'top': [{'p': '76,5%', 'n': 'financeiro'}, {'p': '23,7%', 'n': 'caixa'}]}</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>100,35%</t>
+          <t>{'total': '75', 'top': [{'p': '75%', 'n': 'financeiro'}]}</t>
         </is>
       </c>
     </row>
@@ -2148,17 +2148,17 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>0,26</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>100,28%</t>
+          <t>0,25</t>
         </is>
       </c>
     </row>
@@ -2175,17 +2175,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>101%</t>
+          <t>1,12</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>100,04%</t>
+          <t>1,03</t>
         </is>
       </c>
     </row>
@@ -2202,17 +2202,17 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>pl</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>R$ 1.698.520.740,05</t>
+          <t>Taxa de administração: 0,25% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>R$ 1.826.931.618,96</t>
+          <t>Taxa global: 0,25% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
         </is>
       </c>
     </row>
@@ -2224,22 +2224,22 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>R$ 1.397.203.402,03</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>R$ 1.510.000.753,13</t>
+          <t>99%</t>
         </is>
       </c>
     </row>
@@ -2251,22 +2251,22 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>{'total': '76', 'top': [{'p': '76,5%', 'n': 'financeiro'}, {'p': '23,7%', 'n': 'caixa'}]}</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>{'total': '75', 'top': [{'p': '75%', 'n': 'financeiro'}]}</t>
+          <t>99%</t>
         </is>
       </c>
     </row>
@@ -2278,22 +2278,22 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>0,26</t>
+          <t>104%</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>0,25</t>
+          <t>95%</t>
         </is>
       </c>
     </row>
@@ -2305,22 +2305,22 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>pl</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>1,12</t>
+          <t>R$ 1.983.487.947,49</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>1,03</t>
+          <t>R$ 1.627.449.258,92</t>
         </is>
       </c>
     </row>
@@ -2332,22 +2332,22 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Taxa de administração: 0,25% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
+          <t>R$ 2.522.009.705,73</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Taxa global: 0,25% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
+          <t>R$ 2.427.900.811,01</t>
         </is>
       </c>
     </row>
@@ -2364,17 +2364,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>{'total': '69', 'top': [{'p': '52%', 'n': 'financeiro'}, {'p': '4%', 'n': 'energia elétrica'}, {'p': '2%', 'n': 'transporte e logística'}]}</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>99%</t>
+          <t>{'total': '67', 'top': [{'p': '50%', 'n': 'financeiro'}, {'p': '5%', 'n': 'energia elétrica'}, {'p': '2%', 'n': 'FIDC'}]}</t>
         </is>
       </c>
     </row>
@@ -2391,17 +2391,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>0,44</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>99%</t>
+          <t>0,43</t>
         </is>
       </c>
     </row>
@@ -2418,17 +2418,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>104%</t>
+          <t>1,20</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>1,34</t>
         </is>
       </c>
     </row>
@@ -2445,17 +2445,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>pl</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>R$ 1.983.487.947,49</t>
+          <t>Taxa de administração: 0,20% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>R$ 1.627.449.258,92</t>
+          <t>Taxa global: 0,20% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
         </is>
       </c>
     </row>
@@ -2467,22 +2467,22 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>inst15</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>R$ 2.522.009.705,73</t>
+          <t>113%</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>R$ 2.427.900.811,01</t>
+          <t>101%</t>
         </is>
       </c>
     </row>
@@ -2494,22 +2494,22 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>inst15</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>pl</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>{'total': '69', 'top': [{'p': '52%', 'n': 'financeiro'}, {'p': '4%', 'n': 'energia elétrica'}, {'p': '2%', 'n': 'transporte e logística'}]}</t>
+          <t>R$ 161.593.743,98</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>{'total': '67', 'top': [{'p': '50%', 'n': 'financeiro'}, {'p': '5%', 'n': 'energia elétrica'}, {'p': '2%', 'n': 'FIDC'}]}</t>
+          <t>R$ 156.246.478,91</t>
         </is>
       </c>
     </row>
@@ -2521,22 +2521,22 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>inst15</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>0,44</t>
+          <t>R$ 140.997.685,81</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>0,43</t>
+          <t>R$ 151.871.553,37</t>
         </is>
       </c>
     </row>
@@ -2548,22 +2548,22 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>inst15</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>1,20</t>
+          <t>{'total': '74', 'top': [{'p': '29%', 'n': 'financeiro'}, {'p': '13%', 'n': 'FIDC'}, {'p': '7%', 'n': 'energia elétrica'}]}</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>1,34</t>
+          <t>{'total': '70', 'top': [{'p': '28%', 'n': 'financeiro'}, {'p': '13%', 'n': 'FIDC'}, {'p': '7%', 'n': 'energia elétrica'}]}</t>
         </is>
       </c>
     </row>
@@ -2575,22 +2575,22 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>inst15</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Taxa de administração: 0,20% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Taxa global: 0,20% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
+          <t>0,91</t>
         </is>
       </c>
     </row>
@@ -2607,17 +2607,17 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>113%</t>
+          <t>1,97</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>101%</t>
+          <t>1,74</t>
         </is>
       </c>
     </row>
@@ -2634,17 +2634,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>pl</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>R$ 161.593.743,98</t>
+          <t>anos</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>R$ 156.246.478,91</t>
+          <t>ano</t>
         </is>
       </c>
     </row>
@@ -2661,17 +2661,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>R$ 140.997.685,81</t>
+          <t>Taxa de administração: 0,45% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>R$ 151.871.553,37</t>
+          <t>Taxa global: 0,50% a.a. Taxa de performance: 20% do que exceder 102,5% do CDI. Aplicação: D+0 · Resgate: D+0.</t>
         </is>
       </c>
     </row>
@@ -2683,22 +2683,22 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>inst15</t>
+          <t>inst30</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>{'total': '74', 'top': [{'p': '29%', 'n': 'financeiro'}, {'p': '13%', 'n': 'FIDC'}, {'p': '7%', 'n': 'energia elétrica'}]}</t>
+          <t>101%</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>{'total': '70', 'top': [{'p': '28%', 'n': 'financeiro'}, {'p': '13%', 'n': 'FIDC'}, {'p': '7%', 'n': 'energia elétrica'}]}</t>
+          <t>100%</t>
         </is>
       </c>
     </row>
@@ -2710,22 +2710,22 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>inst15</t>
+          <t>inst30</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>113%</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>0,91</t>
+          <t>102%</t>
         </is>
       </c>
     </row>
@@ -2737,22 +2737,22 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>inst15</t>
+          <t>inst30</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>pl</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>1,97</t>
+          <t>R$ 143.232.764,20</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>1,74</t>
+          <t>R$ 138.199.759,13</t>
         </is>
       </c>
     </row>
@@ -2764,22 +2764,22 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>inst15</t>
+          <t>inst30</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>anos</t>
+          <t>R$ 155.004.649,74</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>ano</t>
+          <t>R$ 162.868.029,59</t>
         </is>
       </c>
     </row>
@@ -2791,22 +2791,22 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>inst15</t>
+          <t>inst30</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Taxa de administração: 0,45% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
+          <t>{'total': '84', 'top': [{'p': '33%', 'n': 'financeiro'}, {'p': '15%', 'n': 'FIDC'}, {'p': '8%', 'n': 'energia elétrica'}]}</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Taxa global: 0,50% a.a. Taxa de performance: 20% do que exceder 102,5% do CDI. Aplicação: D+0 · Resgate: D+0.</t>
+          <t>{'total': '79', 'top': [{'p': '31%', 'n': 'financeiro'}, {'p': '15%', 'n': 'FIDC'}, {'p': '8%', 'n': 'energia elétrica'}]}</t>
         </is>
       </c>
     </row>
@@ -2823,17 +2823,17 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>101%</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>1,02</t>
         </is>
       </c>
     </row>
@@ -2850,17 +2850,17 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>113%</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>102%</t>
+          <t>1,79</t>
         </is>
       </c>
     </row>
@@ -2877,17 +2877,17 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>pl</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>R$ 143.232.764,20</t>
+          <t>anos</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>R$ 138.199.759,13</t>
+          <t>ano</t>
         </is>
       </c>
     </row>
@@ -2904,17 +2904,17 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>R$ 155.004.649,74</t>
+          <t>Taxa de administração: 0,63% a.a. Taxa de performance: 20% do que exceder o CDI. Resgate: D+30.</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>R$ 162.868.029,59</t>
+          <t>Taxa global: 0,625% a.a. Taxa de performance: 20% do que exceder 100% do CDI. Resgate: D+30.</t>
         </is>
       </c>
     </row>
@@ -2926,22 +2926,22 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>inst30</t>
+          <t>infraplus</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>{'total': '84', 'top': [{'p': '33%', 'n': 'financeiro'}, {'p': '15%', 'n': 'FIDC'}, {'p': '8%', 'n': 'energia elétrica'}]}</t>
+          <t>12,94%</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>{'total': '79', 'top': [{'p': '31%', 'n': 'financeiro'}, {'p': '15%', 'n': 'FIDC'}, {'p': '8%', 'n': 'energia elétrica'}]}</t>
+          <t>9,10%</t>
         </is>
       </c>
     </row>
@@ -2953,22 +2953,22 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>inst30</t>
+          <t>infraplus</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>a1</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>*Alfa: -2,75%</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>1,02</t>
+          <t>*Alfa: −5,70%</t>
         </is>
       </c>
     </row>
@@ -2980,22 +2980,22 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>inst30</t>
+          <t>infraplus</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7,80%</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>1,79</t>
+          <t>7,05%</t>
         </is>
       </c>
     </row>
@@ -3007,22 +3007,22 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>inst30</t>
+          <t>infraplus</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>a2</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>anos</t>
+          <t>*Alfa: -3,14%</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>ano</t>
+          <t>*Alfa: −4,32%</t>
         </is>
       </c>
     </row>
@@ -3034,22 +3034,22 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>inst30</t>
+          <t>infraplus</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Taxa de administração: 0,63% a.a. Taxa de performance: 20% do que exceder o CDI. Resgate: D+30.</t>
+          <t>1,24%</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Taxa global: 0,625% a.a. Taxa de performance: 20% do que exceder 100% do CDI. Resgate: D+30.</t>
+          <t>1,01%</t>
         </is>
       </c>
     </row>
@@ -3066,17 +3066,17 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>a3</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>12,94%</t>
+          <t>*Alfa: -0,14%</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>9,10%</t>
+          <t>*Alfa: −1,00%</t>
         </is>
       </c>
     </row>
@@ -3093,17 +3093,17 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>a1</t>
+          <t>pl</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>*Alfa: -2,75%</t>
+          <t>R$ 42.983.282,75</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>*Alfa: −5,70%</t>
+          <t>R$ 37.299.076,05</t>
         </is>
       </c>
     </row>
@@ -3120,17 +3120,17 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>7,80%</t>
+          <t>R$ 52.049.593,91</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>7,05%</t>
+          <t>R$ 46.597.018,20</t>
         </is>
       </c>
     </row>
@@ -3147,17 +3147,17 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>a2</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>*Alfa: -3,14%</t>
+          <t>{'total': '95', 'top': [{'p': '55%', 'n': 'energia elétrica'}, {'p': '15%', 'n': 'transporte e logística'}, {'p': '7%', 'n': 'saneamento'}]}</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>*Alfa: −4,32%</t>
+          <t>{'total': '97', 'top': [{'p': '53%', 'n': 'energia elétrica'}, {'p': '14%', 'n': 'transporte e logística'}, {'p': '8%', 'n': 'saneamento'}]}</t>
         </is>
       </c>
     </row>
@@ -3174,17 +3174,17 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>1,24%</t>
+          <t>8,63</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>1,01%</t>
+          <t>8,11</t>
         </is>
       </c>
     </row>
@@ -3201,17 +3201,17 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>a3</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>*Alfa: -0,14%</t>
+          <t>4,00</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>*Alfa: −1,00%</t>
+          <t>3,99</t>
         </is>
       </c>
     </row>
@@ -3228,17 +3228,17 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>pl</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>R$ 42.983.282,75</t>
+          <t>Taxa de administração: 0,75% a.a. Taxa de performance: não há. Resgate: D+31. Rentabilidade isenta de IR para pessoa física.</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>R$ 37.299.076,05</t>
+          <t>Taxa global: 0,75% a.a. Taxa de performance: não há. Resgate: D+31. Rentabilidade isenta de IR para pessoa física.</t>
         </is>
       </c>
     </row>
@@ -3250,22 +3250,22 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>infraplus</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>k1</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>R$ 52.049.593,91</t>
+          <t>12M</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>R$ 46.597.018,20</t>
+          <t>Desde o início</t>
         </is>
       </c>
     </row>
@@ -3277,22 +3277,22 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>infraplus</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>{'total': '95', 'top': [{'p': '55%', 'n': 'energia elétrica'}, {'p': '15%', 'n': 'transporte e logística'}, {'p': '7%', 'n': 'saneamento'}]}</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>{'total': '97', 'top': [{'p': '53%', 'n': 'energia elétrica'}, {'p': '14%', 'n': 'transporte e logística'}, {'p': '8%', 'n': 'saneamento'}]}</t>
+          <t>88%</t>
         </is>
       </c>
     </row>
@@ -3304,22 +3304,22 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>infraplus</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>8,63</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>8,11</t>
+          <t>82%</t>
         </is>
       </c>
     </row>
@@ -3331,22 +3331,22 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>infraplus</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>4,00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>3,99</t>
+          <t>−14%</t>
         </is>
       </c>
     </row>
@@ -3358,22 +3358,22 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>infraplus</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>pl</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Taxa de administração: 0,75% a.a. Taxa de performance: não há. Resgate: D+31. Rentabilidade isenta de IR para pessoa física.</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Taxa global: 0,75% a.a. Taxa de performance: não há. Resgate: D+31. Rentabilidade isenta de IR para pessoa física.</t>
+          <t>R$ 44.023.801,59</t>
         </is>
       </c>
     </row>
@@ -3385,22 +3385,22 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>31/07/2026</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>R$ 37.965.174,74</t>
         </is>
       </c>
     </row>
@@ -3412,22 +3412,22 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Julho de 2026</t>
+          <t>{'total': '0', 'top': []}</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Setembro de 2026</t>
+          <t>{'total': '93', 'top': [{'p': '38%', 'n': 'energia elétrica'}, {'p': '22%', 'n': 'FIDC'}, {'p': '11%', 'n': 'transporte e logística'}]}</t>
         </is>
       </c>
     </row>
@@ -3439,22 +3439,22 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>julho de 2026</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>setembro de 2026</t>
+          <t>1,08</t>
         </is>
       </c>
     </row>
@@ -3466,22 +3466,22 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>JULHO DE 2026</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>SETEMBRO DE 2026</t>
+          <t>3,70</t>
         </is>
       </c>
     </row>
@@ -3493,22 +3493,22 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Julho 2026</t>
+          <t>Taxa de administração: 0,75% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+30. Rentabilidade isenta de IR para pessoa física.</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Setembro 2026</t>
+          <t>Taxa global: 0,75% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+30. Rentabilidade isenta de IR para pessoa física.</t>
         </is>
       </c>
     </row>
@@ -3530,12 +3530,12 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>-jul26</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>-set26</t>
+          <t>30/09/2026</t>
         </is>
       </c>
     </row>
@@ -3557,12 +3557,12 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>const ATUAL=6;</t>
+          <t>Julho de 2026</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>const ATUAL=8;</t>
+          <t>Setembro de 2026</t>
         </is>
       </c>
     </row>
@@ -3579,152 +3579,152 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>libs de exportação</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>CDN</t>
+          <t>julho de 2026</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>4 referências → vendor/ local (CDN como reserva)</t>
+          <t>setembro de 2026</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>tivio-post-credito-privado.html</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>103%</t>
+          <t>JULHO DE 2026</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>48%</t>
+          <t>SETEMBRO DE 2026</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>tivio-post-credito-privado.html</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>101%</t>
+          <t>Julho 2026</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>Setembro 2026</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>tivio-post-credito-privado.html</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>101%</t>
+          <t>-jul26</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>-set26</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>tivio-post-credito-privado.html</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>R$ 352,4 mi</t>
+          <t>const ATUAL=6;</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>R$ 339,3 mi</t>
+          <t>const ATUAL=8;</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>tivio-post-credito-privado.html</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>libs de exportação</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>104%</t>
+          <t>CDN</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>4 referências → vendor/ local (CDN como reserva)</t>
         </is>
       </c>
     </row>
@@ -3736,22 +3736,22 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>106%</t>
+          <t>103%</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>104%</t>
+          <t>48%</t>
         </is>
       </c>
     </row>
@@ -3763,22 +3763,22 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>109%</t>
+          <t>101%</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>106%</t>
+          <t>93%</t>
         </is>
       </c>
     </row>
@@ -3790,22 +3790,22 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>R$ 33,2 mi</t>
+          <t>101%</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>R$ 38,8 mi</t>
+          <t>95%</t>
         </is>
       </c>
     </row>
@@ -3817,22 +3817,22 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>adm</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>0,00% a.a. (vértice tx zero)</t>
+          <t>R$ 352,4 mi</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>0,15% a.a.</t>
+          <t>R$ 339,3 mi</t>
         </is>
       </c>
     </row>
@@ -3844,7 +3844,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -3854,12 +3854,12 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>104%</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>95%</t>
         </is>
       </c>
     </row>
@@ -3871,7 +3871,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -3881,12 +3881,12 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>86%</t>
+          <t>106%</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>87%</t>
+          <t>104%</t>
         </is>
       </c>
     </row>
@@ -3898,22 +3898,22 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>R$ 374,3 mi</t>
+          <t>109%</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>R$ 329,9 mi</t>
+          <t>106%</t>
         </is>
       </c>
     </row>
@@ -3925,22 +3925,22 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>2,13%</t>
+          <t>R$ 33,2 mi</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>0,14%</t>
+          <t>R$ 38,8 mi</t>
         </is>
       </c>
     </row>
@@ -3952,22 +3952,22 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>a1</t>
+          <t>adm</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>*Alfa: −3,03%</t>
+          <t>0,00% a.a. (vértice tx zero)</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>*Alfa: 1,41%</t>
+          <t>0,15% a.a.</t>
         </is>
       </c>
     </row>
@@ -3979,22 +3979,22 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>−5,35%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>6,43%</t>
+          <t>91%</t>
         </is>
       </c>
     </row>
@@ -4006,22 +4006,22 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>a2</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>*Alfa: −1,59%</t>
+          <t>86%</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>*Alfa: 1,13%</t>
+          <t>87%</t>
         </is>
       </c>
     </row>
@@ -4033,22 +4033,22 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>7,66%</t>
+          <t>R$ 374,3 mi</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>12,75%</t>
+          <t>R$ 329,9 mi</t>
         </is>
       </c>
     </row>
@@ -4065,17 +4065,17 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>a3</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>*Alfa: −6,22%</t>
+          <t>2,13%</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>*Alfa: 0,50%</t>
+          <t>0%</t>
         </is>
       </c>
     </row>
@@ -4092,17 +4092,17 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>a1</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>R$ 100,8 mi</t>
+          <t>*Alfa: −3,03%</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>R$ 70,7 mi</t>
+          <t>*Alfa: 1,41%</t>
         </is>
       </c>
     </row>
@@ -4114,22 +4114,22 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>perf</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>20% do que exceder o CDI</t>
+          <t>−5,35%</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>20% do que exceder 100% do CDI</t>
+          <t>6%</t>
         </is>
       </c>
     </row>
@@ -4141,22 +4141,22 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>a2</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>73%</t>
+          <t>*Alfa: −1,59%</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>144%</t>
+          <t>*Alfa: 1,13%</t>
         </is>
       </c>
     </row>
@@ -4168,22 +4168,22 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>74%</t>
+          <t>7,66%</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>83%</t>
+          <t>13%</t>
         </is>
       </c>
     </row>
@@ -4195,22 +4195,22 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>a3</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>81%</t>
+          <t>*Alfa: −6,22%</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>87%</t>
+          <t>*Alfa: 0,50%</t>
         </is>
       </c>
     </row>
@@ -4222,7 +4222,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -4232,12 +4232,12 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>R$ 102,7 mi</t>
+          <t>R$ 100,8 mi</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>R$ 95,5 mi</t>
+          <t>R$ 70,7 mi</t>
         </is>
       </c>
     </row>
@@ -4249,22 +4249,22 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>perf</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>20% do que exceder o CDI</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>141%</t>
+          <t>20% do que exceder 100% do CDI</t>
         </is>
       </c>
     </row>
@@ -4276,22 +4276,22 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>73%</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>144%</t>
         </is>
       </c>
     </row>
@@ -4303,22 +4303,22 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>74%</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>83%</t>
         </is>
       </c>
     </row>
@@ -4330,22 +4330,22 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>R$ 662,8 mi</t>
+          <t>81%</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>R$ 637,1 mi</t>
+          <t>87%</t>
         </is>
       </c>
     </row>
@@ -4357,22 +4357,22 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>31/07/2026</t>
+          <t>R$ 102,7 mi</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>R$ 95,5 mi</t>
         </is>
       </c>
     </row>
@@ -4384,22 +4384,22 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Julho de 2026</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Setembro de 2026</t>
+          <t>141%</t>
         </is>
       </c>
     </row>
@@ -4411,22 +4411,22 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>julho de 2026</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>setembro de 2026</t>
+          <t>98%</t>
         </is>
       </c>
     </row>
@@ -4438,22 +4438,22 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>JULHO DE 2026</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>SETEMBRO DE 2026</t>
+          <t>97%</t>
         </is>
       </c>
     </row>
@@ -4465,22 +4465,22 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Julho 2026</t>
+          <t>R$ 662,8 mi</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Setembro 2026</t>
+          <t>R$ 637,1 mi</t>
         </is>
       </c>
     </row>
@@ -4502,12 +4502,12 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>-jul26</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>-set26</t>
+          <t>30/09/2026</t>
         </is>
       </c>
     </row>
@@ -4529,12 +4529,12 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>const ATUAL=6;</t>
+          <t>Julho de 2026</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>const ATUAL=8;</t>
+          <t>Setembro de 2026</t>
         </is>
       </c>
     </row>
@@ -4551,61 +4551,61 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>libs de exportação</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>CDN</t>
+          <t>julho de 2026</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>4 referências → vendor/ local (CDN como reserva)</t>
+          <t>setembro de 2026</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>tivio-central.html</t>
+          <t>tivio-post-investment-solutions.html</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>s1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Julho 2026</t>
+          <t>JULHO DE 2026</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Setembro 2026</t>
+          <t>SETEMBRO DE 2026</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>tivio-central.html</t>
+          <t>tivio-post-investment-solutions.html</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>s2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -4622,81 +4622,81 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>tivio-central.html</t>
+          <t>tivio-post-investment-solutions.html</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>s8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Julho 2026</t>
+          <t>-jul26</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Setembro 2026</t>
+          <t>-set26</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>tivio-central.html</t>
+          <t>tivio-post-investment-solutions.html</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>e1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Julho 2026</t>
+          <t>const ATUAL=6;</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Setembro 2026</t>
+          <t>const ATUAL=8;</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>tivio-central.html</t>
+          <t>tivio-post-investment-solutions.html</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>libs de exportação</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Relatório de Gestão · Incentivado CDI 30</t>
+          <t>CDN</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Gerador de Relatório de Gestão · Incentivado CDI 30</t>
+          <t>4 referências → vendor/ local (CDN como reserva)</t>
         </is>
       </c>
     </row>
@@ -4708,22 +4708,22 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>s1</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>desc</t>
+          <t>date</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Relatório de gestão mensal do Tivio Institucional Inc CDI 30 FIF (debêntures incentivadas · CDI).</t>
+          <t>Julho 2026</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Construtor interativo, folha a folha. Os relatórios prontos do mês estão no card acima. Relatório de gestão mensal do Tivio Institucional Inc CDI 30 FIF (debêntures incentivadas · CDI).</t>
+          <t>Setembro 2026</t>
         </is>
       </c>
     </row>
@@ -4735,22 +4735,22 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>s2</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>date</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>cards de relatório</t>
+          <t>Julho 2026</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>2 registrados para Setembro 2026</t>
+          <t>Setembro 2026</t>
         </is>
       </c>
     </row>
@@ -4762,16 +4762,151 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
+          <t>s8</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Julho 2026</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Setembro 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>tivio-central.html</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>e1</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Julho 2026</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Setembro 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>tivio-central.html</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>r2</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Relatório de Gestão · Incentivado CDI 30</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Gerador de Relatório de Gestão · Incentivado CDI 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>tivio-central.html</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>r2</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>desc</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Relatório de gestão mensal do Tivio Institucional Inc CDI 30 FIF (debêntures incentivadas · CDI).</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Construtor interativo, folha a folha. Os relatórios prontos do mês estão no card acima. Relatório de gestão mensal do Tivio Institucional Inc CDI 30 FIF (debêntures incentivadas · CDI).</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>tivio-central.html</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C161" t="inlineStr">
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>cards de relatório</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>2 registrados para Setembro 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>tivio-central.html</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
         <is>
           <t>data automática</t>
         </is>
       </c>
-      <c r="D161" t="inlineStr"/>
-      <c r="E161" t="inlineStr">
+      <c r="D166" t="inlineStr"/>
+      <c r="E166" t="inlineStr">
         <is>
           <t>DATA_BASE=2026-09-30</t>
         </is>
@@ -11153,7 +11288,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>828947</v>
+        <v>828790</v>
       </c>
     </row>
     <row r="3">
@@ -11183,7 +11318,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>835427</v>
+        <v>835267</v>
       </c>
     </row>
     <row r="5">
@@ -11363,7 +11498,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>618771</v>
+        <v>618952</v>
       </c>
     </row>
     <row r="17">
@@ -11378,7 +11513,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>296290</v>
+        <v>296292</v>
       </c>
     </row>
     <row r="18">
@@ -11393,7 +11528,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>617212</v>
+        <v>617096</v>
       </c>
     </row>
     <row r="19">
@@ -11408,7 +11543,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>290880</v>
+        <v>290888</v>
       </c>
     </row>
     <row r="20">
@@ -11423,7 +11558,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>612974</v>
+        <v>612993</v>
       </c>
     </row>
     <row r="21">
@@ -11438,7 +11573,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>284126</v>
+        <v>284172</v>
       </c>
     </row>
     <row r="22">
@@ -11453,7 +11588,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>830146</v>
+        <v>830104</v>
       </c>
     </row>
     <row r="23">
@@ -11483,7 +11618,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>832464</v>
+        <v>832191</v>
       </c>
     </row>
     <row r="25">
@@ -11498,7 +11633,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1968015</v>
+        <v>1968199</v>
       </c>
     </row>
     <row r="26">
@@ -11513,7 +11648,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>830848</v>
+        <v>830709</v>
       </c>
     </row>
     <row r="27">
@@ -11528,7 +11663,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1959014</v>
+        <v>1958853</v>
       </c>
     </row>
     <row r="28">
@@ -11558,7 +11693,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1060482</v>
+        <v>1060491</v>
       </c>
     </row>
     <row r="30">
@@ -11618,7 +11753,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>114692</v>
+        <v>119683</v>
       </c>
     </row>
     <row r="34">
@@ -11633,7 +11768,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>127513</v>
+        <v>134052</v>
       </c>
     </row>
     <row r="35">
@@ -11648,7 +11783,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>105535</v>
+        <v>105526</v>
       </c>
     </row>
     <row r="36">

</xml_diff>

<commit_message>
AutomaTivio: linha das taxas maior nos posts de Destaques (14 -> 19 px)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -11288,7 +11288,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>828790</v>
+        <v>828947</v>
       </c>
     </row>
     <row r="3">
@@ -11318,7 +11318,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>835267</v>
+        <v>835427</v>
       </c>
     </row>
     <row r="5">
@@ -11573,7 +11573,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>284172</v>
+        <v>284127</v>
       </c>
     </row>
     <row r="22">
@@ -11588,7 +11588,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>830104</v>
+        <v>830146</v>
       </c>
     </row>
     <row r="23">
@@ -11603,7 +11603,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1960267</v>
+        <v>1960127</v>
       </c>
     </row>
     <row r="24">
@@ -11618,7 +11618,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>832191</v>
+        <v>832464</v>
       </c>
     </row>
     <row r="25">
@@ -11633,7 +11633,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1968199</v>
+        <v>1968015</v>
       </c>
     </row>
     <row r="26">
@@ -11648,7 +11648,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>830709</v>
+        <v>830848</v>
       </c>
     </row>
     <row r="27">
@@ -11663,7 +11663,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1958853</v>
+        <v>1959014</v>
       </c>
     </row>
     <row r="28">
@@ -11753,7 +11753,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>119683</v>
+        <v>119854</v>
       </c>
     </row>
     <row r="34">
@@ -11768,7 +11768,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>134052</v>
+        <v>134223</v>
       </c>
     </row>
     <row r="35">

</xml_diff>

<commit_message>
AutomaTivio: nos posts, rótulo e valor das taxas não se separam na quebra de linha
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -11288,7 +11288,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>828947</v>
+        <v>828790</v>
       </c>
     </row>
     <row r="3">
@@ -11513,7 +11513,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>296292</v>
+        <v>296099</v>
       </c>
     </row>
     <row r="18">
@@ -11528,7 +11528,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>617096</v>
+        <v>616955</v>
       </c>
     </row>
     <row r="19">
@@ -11543,7 +11543,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>290888</v>
+        <v>291169</v>
       </c>
     </row>
     <row r="20">
@@ -11558,7 +11558,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>612993</v>
+        <v>612857</v>
       </c>
     </row>
     <row r="21">
@@ -11573,7 +11573,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>284127</v>
+        <v>284172</v>
       </c>
     </row>
     <row r="22">
@@ -11588,7 +11588,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>830146</v>
+        <v>830104</v>
       </c>
     </row>
     <row r="23">
@@ -11603,7 +11603,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1960127</v>
+        <v>1960267</v>
       </c>
     </row>
     <row r="24">
@@ -11618,7 +11618,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>832464</v>
+        <v>832191</v>
       </c>
     </row>
     <row r="25">
@@ -11633,7 +11633,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1968015</v>
+        <v>1968199</v>
       </c>
     </row>
     <row r="26">
@@ -11648,7 +11648,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>830848</v>
+        <v>830709</v>
       </c>
     </row>
     <row r="27">
@@ -11663,7 +11663,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1959014</v>
+        <v>1958853</v>
       </c>
     </row>
     <row r="28">
@@ -11753,7 +11753,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>119854</v>
+        <v>120162</v>
       </c>
     </row>
     <row r="34">
@@ -11768,7 +11768,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>134223</v>
+        <v>134531</v>
       </c>
     </row>
     <row r="35">

</xml_diff>

<commit_message>
AutomaTivio: nos posts, cada item das taxas (ex.: a taxa de performance inteira) fica numa linha só
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -11288,7 +11288,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>828790</v>
+        <v>828947</v>
       </c>
     </row>
     <row r="3">
@@ -11513,7 +11513,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>296099</v>
+        <v>296292</v>
       </c>
     </row>
     <row r="18">
@@ -11543,7 +11543,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>291169</v>
+        <v>290888</v>
       </c>
     </row>
     <row r="20">
@@ -11558,7 +11558,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>612857</v>
+        <v>612993</v>
       </c>
     </row>
     <row r="21">
@@ -11573,7 +11573,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>284172</v>
+        <v>284127</v>
       </c>
     </row>
     <row r="22">
@@ -11588,7 +11588,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>830104</v>
+        <v>830146</v>
       </c>
     </row>
     <row r="23">
@@ -11603,7 +11603,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1960267</v>
+        <v>1960127</v>
       </c>
     </row>
     <row r="24">
@@ -11618,7 +11618,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>832191</v>
+        <v>832464</v>
       </c>
     </row>
     <row r="25">
@@ -11633,7 +11633,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1968199</v>
+        <v>1968015</v>
       </c>
     </row>
     <row r="26">
@@ -11648,7 +11648,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>830709</v>
+        <v>830848</v>
       </c>
     </row>
     <row r="27">
@@ -11753,7 +11753,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>120162</v>
+        <v>120495</v>
       </c>
     </row>
     <row r="34">
@@ -11768,7 +11768,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>134531</v>
+        <v>134864</v>
       </c>
     </row>
     <row r="35">

</xml_diff>

<commit_message>
AutomaTivio: todos os HTML da edição numa pasta só (central/)
- As páginas de relatório por vertical passam a ser geradas em central/, ao
  lado da Central, dos posts e dos e-mails; os links ficam na mesma pasta.
- central/vendor/ ganha as bibliotecas que as páginas de relatório usam; a
  pasta antiga relatorios/ é removida na rodada.
- Guia e contexto atualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -11528,7 +11528,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>616955</v>
+        <v>617096</v>
       </c>
     </row>
     <row r="19">
@@ -11663,7 +11663,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1958853</v>
+        <v>1959014</v>
       </c>
     </row>
     <row r="28">
@@ -11678,7 +11678,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3222930</v>
+        <v>3222919</v>
       </c>
     </row>
     <row r="29">
@@ -11693,7 +11693,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1060491</v>
+        <v>1060480</v>
       </c>
     </row>
     <row r="30">
@@ -11798,7 +11798,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>65886</v>
+        <v>65858</v>
       </c>
     </row>
     <row r="37">

</xml_diff>

<commit_message>
AutomaTivio: Ágora vira o cartão quadrado; botão centralizado na exportação
- E-mail: a versão Ágora passa a ser o cartão quadrado (rentabilidade em
  destaque); a aba "Quadrado" separada sai.
- Exportação PNG: o botão "Ver relatório completo" do cartão quadrado sai
  com o texto no centro (antes subia para o topo do botão).
- run.py --saidas aceita também destaques e emails.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -11288,7 +11288,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>828947</v>
+        <v>828790</v>
       </c>
     </row>
     <row r="3">
@@ -11333,7 +11333,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1966288</v>
+        <v>1966259</v>
       </c>
     </row>
     <row r="6">
@@ -11588,7 +11588,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>830146</v>
+        <v>830104</v>
       </c>
     </row>
     <row r="23">
@@ -11723,7 +11723,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>176977</v>
+        <v>177281</v>
       </c>
     </row>
     <row r="32">

</xml_diff>

<commit_message>
AutomaTivio: páginas Saiba mais do HGD30 e do HYD60 (previdência), com números da carteira FIFE
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -5009,7 +5009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -5043,12 +5043,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BV Top Gestor Crédito Privado</t>
+          <t>Tivio HGD30</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -5065,12 +5065,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>hyd60</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tivio Top Gestor HY</t>
+          <t>Tivio HYD60</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -5087,12 +5087,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BV Top Gestor RF Ativo</t>
+          <t>BV Top Gestor Crédito Privado</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -5109,100 +5109,100 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>topgestormacro</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BV Top Gestor Macro</t>
+          <t>Tivio Top Gestor HY</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>rentabilidade</t>
+          <t>comentário do gestor</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>sem cotas na dados_mensais</t>
+          <t>não preenchido no arquivo de comentários</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>topgestorlongonly</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Top Gestor Ações Long Only</t>
+          <t>BV Top Gestor RF Ativo</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>rentabilidade</t>
+          <t>comentário do gestor</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>sem cotas na dados_mensais</t>
+          <t>não preenchido no arquivo de comentários</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestormacro</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Tivio Top Manager Global</t>
+          <t>BV Top Gestor Macro</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>comentário do gestor</t>
+          <t>rentabilidade</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>não preenchido no arquivo de comentários</t>
+          <t>sem cotas na dados_mensais</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topgestorlongonly</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tivio RF Ativo Longo Prazo</t>
+          <t>Top Gestor Ações Long Only</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>comentário do gestor</t>
+          <t>rentabilidade</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>não preenchido no arquivo de comentários</t>
+          <t>sem cotas na dados_mensais</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tivio Prev Low Vol Itaú</t>
+          <t>Tivio Top Manager Global</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -5219,20 +5219,64 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>ativorf</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Tivio RF Ativo Longo Prazo</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>comentário do gestor</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>não preenchido no arquivo de comentários</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>prevlowvol</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Tivio Prev Low Vol Itaú</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>comentário do gestor</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>não preenchido no arquivo de comentários</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>atuarial</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Tivio Atuarial</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>rentabilidade</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>sem cotas na dados_mensais</t>
         </is>
@@ -5332,7 +5376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K115"/>
+  <dimension ref="A1:K127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8008,17 +8052,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>BV Top Gestor Crédito Privado</t>
+          <t>Tivio HGD30</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
+          <t>TIVIO HGD30 RF CP FIFE RL</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -8035,35 +8079,35 @@
         <v>46265</v>
       </c>
       <c r="G62" t="n">
-        <v>0.005219350133194078</v>
+        <v>0.0108528654278528</v>
       </c>
       <c r="H62" t="n">
         <v>0.01082559188004661</v>
       </c>
       <c r="I62" t="n">
-        <v>-0.005606241746852536</v>
+        <v>2.727354780618363e-05</v>
       </c>
       <c r="J62" t="n">
-        <v>0.4821306946564481</v>
+        <v>1.002519358581812</v>
       </c>
       <c r="K62" t="n">
-        <v>-0.06456129582370584</v>
+        <v>0.0003238255429589554</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>BV Top Gestor Crédito Privado</t>
+          <t>Tivio HGD30</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
+          <t>TIVIO HGD30 RF CP FIFE RL</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -8080,35 +8124,35 @@
         <v>46022</v>
       </c>
       <c r="G63" t="n">
-        <v>0.09822271466718724</v>
+        <v>0.1071791004655822</v>
       </c>
       <c r="H63" t="n">
         <v>0.1051127846901438</v>
       </c>
       <c r="I63" t="n">
-        <v>-0.006890070022956607</v>
+        <v>0.002066315775438365</v>
       </c>
       <c r="J63" t="n">
-        <v>0.9344506946203789</v>
+        <v>1.019658082330609</v>
       </c>
       <c r="K63" t="n">
-        <v>-0.008392753749412729</v>
+        <v>0.002520519554925826</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>BV Top Gestor Crédito Privado</t>
+          <t>Tivio HGD30</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
+          <t>TIVIO HGD30 RF CP FIFE RL</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -8125,35 +8169,35 @@
         <v>45930</v>
       </c>
       <c r="G64" t="n">
-        <v>0.1373601954243717</v>
+        <v>0.146604148478189</v>
       </c>
       <c r="H64" t="n">
         <v>0.1447903912030524</v>
       </c>
       <c r="I64" t="n">
-        <v>-0.007430195778680648</v>
+        <v>0.001813757275136663</v>
       </c>
       <c r="J64" t="n">
-        <v>0.9486830878973134</v>
+        <v>1.012526779298448</v>
       </c>
       <c r="K64" t="n">
-        <v>-0.006516216027085298</v>
+        <v>0.001590674727792951</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>BV Top Gestor Crédito Privado</t>
+          <t>Tivio HGD30</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
+          <t>TIVIO HGD30 RF CP FIFE RL</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -8167,38 +8211,28 @@
         </is>
       </c>
       <c r="F65" s="1" t="n">
-        <v>45561</v>
-      </c>
-      <c r="G65" t="n">
-        <v>0.2920431856569192</v>
-      </c>
-      <c r="H65" t="n">
-        <v>0.2980670513506256</v>
-      </c>
-      <c r="I65" t="n">
-        <v>-0.006023865693706387</v>
-      </c>
-      <c r="J65" t="n">
-        <v>0.9797902328807878</v>
-      </c>
-      <c r="K65" t="n">
-        <v>-0.002327632629077092</v>
-      </c>
+        <v>45786</v>
+      </c>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>BV Top Gestor Crédito Privado</t>
+          <t>Tivio HGD30</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
+          <t>TIVIO HGD30 RF CP FIFE RL</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -8212,38 +8246,28 @@
         </is>
       </c>
       <c r="F66" s="1" t="n">
-        <v>45195</v>
-      </c>
-      <c r="G66" t="n">
-        <v>0.4695527796319496</v>
-      </c>
-      <c r="H66" t="n">
-        <v>0.4424561999402108</v>
-      </c>
-      <c r="I66" t="n">
-        <v>0.02709657969173884</v>
-      </c>
-      <c r="J66" t="n">
-        <v>1.06124127019895</v>
-      </c>
-      <c r="K66" t="n">
-        <v>0.006231139290297394</v>
-      </c>
+        <v>45786</v>
+      </c>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>BV Top Gestor Crédito Privado</t>
+          <t>Tivio HGD30</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
+          <t>TIVIO HGD30 RF CP FIFE RL</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -8257,38 +8281,38 @@
         </is>
       </c>
       <c r="F67" s="1" t="n">
-        <v>44706</v>
+        <v>45786</v>
       </c>
       <c r="G67" t="n">
-        <v>0.7203075669000001</v>
+        <v>0.2187760000000001</v>
       </c>
       <c r="H67" t="n">
-        <v>0.7084789393875421</v>
+        <v>0.2100212531349583</v>
       </c>
       <c r="I67" t="n">
-        <v>0.01182862751245795</v>
+        <v>0.00875474686504174</v>
       </c>
       <c r="J67" t="n">
-        <v>1.016695806826218</v>
+        <v>1.041685052033358</v>
       </c>
       <c r="K67" t="n">
-        <v>0.001593489935187264</v>
+        <v>0.005174439153091015</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>hyd60</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Tivio Top Gestor HY</t>
+          <t>Tivio HYD60</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>TIVIO TOP GESTOR HY FIF RL</t>
+          <t>TIVIO HYD60 FIFE CI MULT CP RL - Expandida</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -8305,35 +8329,35 @@
         <v>46265</v>
       </c>
       <c r="G68" t="n">
-        <v>0.01023196421218886</v>
+        <v>0.01062530137458406</v>
       </c>
       <c r="H68" t="n">
         <v>0.01082559188004661</v>
       </c>
       <c r="I68" t="n">
-        <v>-0.0005936276678577546</v>
+        <v>-0.0002002905054625526</v>
       </c>
       <c r="J68" t="n">
-        <v>0.9451644146171897</v>
+        <v>0.9814984245035394</v>
       </c>
       <c r="K68" t="n">
-        <v>-0.007024523465815835</v>
+        <v>-0.002375156005994805</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>hyd60</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Tivio Top Gestor HY</t>
+          <t>Tivio HYD60</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>TIVIO TOP GESTOR HY FIF RL</t>
+          <t>TIVIO HYD60 FIFE CI MULT CP RL - Expandida</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -8347,38 +8371,28 @@
         </is>
       </c>
       <c r="F69" s="1" t="n">
-        <v>46022</v>
-      </c>
-      <c r="G69" t="n">
-        <v>0.1091887763786945</v>
-      </c>
-      <c r="H69" t="n">
-        <v>0.1051127846901438</v>
-      </c>
-      <c r="I69" t="n">
-        <v>0.004075991688550662</v>
-      </c>
-      <c r="J69" t="n">
-        <v>1.038777316199605</v>
-      </c>
-      <c r="K69" t="n">
-        <v>0.004973518048338343</v>
-      </c>
+        <v>46085</v>
+      </c>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>hyd60</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Tivio Top Gestor HY</t>
+          <t>Tivio HYD60</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>TIVIO TOP GESTOR HY FIF RL</t>
+          <t>TIVIO HYD60 FIFE CI MULT CP RL - Expandida</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -8392,38 +8406,28 @@
         </is>
       </c>
       <c r="F70" s="1" t="n">
-        <v>45930</v>
-      </c>
-      <c r="G70" t="n">
-        <v>0.1532058020745011</v>
-      </c>
-      <c r="H70" t="n">
-        <v>0.1447903912030524</v>
-      </c>
-      <c r="I70" t="n">
-        <v>0.008415410871448703</v>
-      </c>
-      <c r="J70" t="n">
-        <v>1.058121335273188</v>
-      </c>
-      <c r="K70" t="n">
-        <v>0.007380444394986974</v>
-      </c>
+        <v>46085</v>
+      </c>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>hyd60</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Tivio Top Gestor HY</t>
+          <t>Tivio HYD60</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>TIVIO TOP GESTOR HY FIF RL</t>
+          <t>TIVIO HYD60 FIFE CI MULT CP RL - Expandida</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -8437,7 +8441,7 @@
         </is>
       </c>
       <c r="F71" s="1" t="n">
-        <v>45813</v>
+        <v>46085</v>
       </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr"/>
@@ -8448,17 +8452,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>hyd60</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Tivio Top Gestor HY</t>
+          <t>Tivio HYD60</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>TIVIO TOP GESTOR HY FIF RL</t>
+          <t>TIVIO HYD60 FIFE CI MULT CP RL - Expandida</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -8472,7 +8476,7 @@
         </is>
       </c>
       <c r="F72" s="1" t="n">
-        <v>45813</v>
+        <v>46085</v>
       </c>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr"/>
@@ -8483,17 +8487,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>hyd60</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Tivio Top Gestor HY</t>
+          <t>Tivio HYD60</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>TIVIO TOP GESTOR HY FIF RL</t>
+          <t>TIVIO HYD60 FIFE CI MULT CP RL - Expandida</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -8507,38 +8511,38 @@
         </is>
       </c>
       <c r="F73" s="1" t="n">
-        <v>45813</v>
+        <v>46085</v>
       </c>
       <c r="G73" t="n">
-        <v>0.2152430848</v>
+        <v>0.08733539999999995</v>
       </c>
       <c r="H73" t="n">
-        <v>0.1976126726386125</v>
+        <v>0.07982471914470612</v>
       </c>
       <c r="I73" t="n">
-        <v>0.0176304121613875</v>
+        <v>0.007510680855293828</v>
       </c>
       <c r="J73" t="n">
-        <v>1.089217011874686</v>
+        <v>1.094089662146865</v>
       </c>
       <c r="K73" t="n">
-        <v>0.01112061570541045</v>
+        <v>0.01211911820212941</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>BV Top Gestor RF Ativo</t>
+          <t>BV Top Gestor Crédito Privado</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
+          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -8555,35 +8559,35 @@
         <v>46265</v>
       </c>
       <c r="G74" t="n">
-        <v>0.009832721928012766</v>
+        <v>0.005219350133194078</v>
       </c>
       <c r="H74" t="n">
         <v>0.01082559188004661</v>
       </c>
       <c r="I74" t="n">
-        <v>-0.000992869952033848</v>
+        <v>-0.005606241746852536</v>
       </c>
       <c r="J74" t="n">
-        <v>0.9082849267702513</v>
+        <v>0.4821306946564481</v>
       </c>
       <c r="K74" t="n">
-        <v>-0.01172337186485095</v>
+        <v>-0.06456129582370584</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>BV Top Gestor RF Ativo</t>
+          <t>BV Top Gestor Crédito Privado</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
+          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8600,35 +8604,35 @@
         <v>46022</v>
       </c>
       <c r="G75" t="n">
-        <v>0.09190461218917045</v>
+        <v>0.09822271466718724</v>
       </c>
       <c r="H75" t="n">
         <v>0.1051127846901438</v>
       </c>
       <c r="I75" t="n">
-        <v>-0.01320817250097339</v>
+        <v>-0.006890070022956607</v>
       </c>
       <c r="J75" t="n">
-        <v>0.8743428542977999</v>
+        <v>0.9344506946203789</v>
       </c>
       <c r="K75" t="n">
-        <v>-0.01607272996257303</v>
+        <v>-0.008392753749412729</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>BV Top Gestor RF Ativo</t>
+          <t>BV Top Gestor Crédito Privado</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
+          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8645,35 +8649,35 @@
         <v>45930</v>
       </c>
       <c r="G76" t="n">
-        <v>0.129702412726495</v>
+        <v>0.1373601954243717</v>
       </c>
       <c r="H76" t="n">
         <v>0.1447903912030524</v>
       </c>
       <c r="I76" t="n">
-        <v>-0.01508797847655741</v>
+        <v>-0.007430195778680648</v>
       </c>
       <c r="J76" t="n">
-        <v>0.8957943386215581</v>
+        <v>0.9486830878973134</v>
       </c>
       <c r="K76" t="n">
-        <v>-0.01323184628895746</v>
+        <v>-0.006516216027085298</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>BV Top Gestor RF Ativo</t>
+          <t>BV Top Gestor Crédito Privado</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
+          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -8690,35 +8694,35 @@
         <v>45561</v>
       </c>
       <c r="G77" t="n">
-        <v>0.270242572217682</v>
+        <v>0.2920431856569192</v>
       </c>
       <c r="H77" t="n">
         <v>0.2980670513506256</v>
       </c>
       <c r="I77" t="n">
-        <v>-0.02782447913294361</v>
+        <v>-0.006023865693706387</v>
       </c>
       <c r="J77" t="n">
-        <v>0.906650268767168</v>
+        <v>0.9797902328807878</v>
       </c>
       <c r="K77" t="n">
-        <v>-0.01079702351532119</v>
+        <v>-0.002327632629077092</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>BV Top Gestor RF Ativo</t>
+          <t>BV Top Gestor Crédito Privado</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
+          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -8732,28 +8736,38 @@
         </is>
       </c>
       <c r="F78" s="1" t="n">
-        <v>45198</v>
-      </c>
-      <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr"/>
-      <c r="I78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
+        <v>45195</v>
+      </c>
+      <c r="G78" t="n">
+        <v>0.4695527796319496</v>
+      </c>
+      <c r="H78" t="n">
+        <v>0.4424561999402108</v>
+      </c>
+      <c r="I78" t="n">
+        <v>0.02709657969173884</v>
+      </c>
+      <c r="J78" t="n">
+        <v>1.06124127019895</v>
+      </c>
+      <c r="K78" t="n">
+        <v>0.006231139290297394</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>BV Top Gestor RF Ativo</t>
+          <t>BV Top Gestor Crédito Privado</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
+          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -8767,43 +8781,43 @@
         </is>
       </c>
       <c r="F79" s="1" t="n">
-        <v>45198</v>
+        <v>44706</v>
       </c>
       <c r="G79" t="n">
-        <v>0.399945644</v>
+        <v>0.7203075669000001</v>
       </c>
       <c r="H79" t="n">
-        <v>0.4404121868646469</v>
+        <v>0.7084789393875421</v>
       </c>
       <c r="I79" t="n">
-        <v>-0.0404665428646469</v>
+        <v>0.01182862751245795</v>
       </c>
       <c r="J79" t="n">
-        <v>0.9081166596393855</v>
+        <v>1.016695806826218</v>
       </c>
       <c r="K79" t="n">
-        <v>-0.009503710662674081</v>
+        <v>0.001593489935187264</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Tivio Top Manager Global</t>
+          <t>Tivio Top Gestor HY</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
+          <t>TIVIO TOP GESTOR HY FIF RL</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>MSCI ACWI</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -8815,40 +8829,40 @@
         <v>46265</v>
       </c>
       <c r="G80" t="n">
-        <v>0.001361630876498987</v>
+        <v>0.01023196421218886</v>
       </c>
       <c r="H80" t="n">
-        <v>-0.01270714044827159</v>
+        <v>0.01082559188004661</v>
       </c>
       <c r="I80" t="n">
-        <v>0.01406877132477058</v>
+        <v>-0.0005936276678577546</v>
       </c>
       <c r="J80" t="n">
-        <v>-0.1071547829381389</v>
+        <v>0.9451644146171897</v>
       </c>
       <c r="K80" t="n">
-        <v>0.1850574526325846</v>
+        <v>-0.007024523465815835</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Tivio Top Manager Global</t>
+          <t>Tivio Top Gestor HY</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
+          <t>TIVIO TOP GESTOR HY FIF RL</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>MSCI ACWI</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -8860,40 +8874,40 @@
         <v>46022</v>
       </c>
       <c r="G81" t="n">
-        <v>0.06432757633456698</v>
+        <v>0.1091887763786945</v>
       </c>
       <c r="H81" t="n">
-        <v>0.05306746240220672</v>
+        <v>0.1051127846901438</v>
       </c>
       <c r="I81" t="n">
-        <v>0.01126011393236026</v>
+        <v>0.004075991688550662</v>
       </c>
       <c r="J81" t="n">
-        <v>1.212184894898838</v>
+        <v>1.038777316199605</v>
       </c>
       <c r="K81" t="n">
-        <v>0.01443610338441359</v>
+        <v>0.004973518048338343</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Tivio Top Manager Global</t>
+          <t>Tivio Top Gestor HY</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
+          <t>TIVIO TOP GESTOR HY FIF RL</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>MSCI ACWI</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -8905,40 +8919,40 @@
         <v>45930</v>
       </c>
       <c r="G82" t="n">
-        <v>0.1275037236060828</v>
+        <v>0.1532058020745011</v>
       </c>
       <c r="H82" t="n">
-        <v>0.1224734191492385</v>
+        <v>0.1447903912030524</v>
       </c>
       <c r="I82" t="n">
-        <v>0.00503030445684427</v>
+        <v>0.008415410871448703</v>
       </c>
       <c r="J82" t="n">
-        <v>1.041072622057809</v>
+        <v>1.058121335273188</v>
       </c>
       <c r="K82" t="n">
-        <v>0.004499340868773238</v>
+        <v>0.007380444394986974</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Tivio Top Manager Global</t>
+          <t>Tivio Top Gestor HY</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
+          <t>TIVIO TOP GESTOR HY FIF RL</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>MSCI ACWI</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -8947,43 +8961,33 @@
         </is>
       </c>
       <c r="F83" s="1" t="n">
-        <v>45561</v>
-      </c>
-      <c r="G83" t="n">
-        <v>0.2322960043521065</v>
-      </c>
-      <c r="H83" t="n">
-        <v>0.2701236930973472</v>
-      </c>
-      <c r="I83" t="n">
-        <v>-0.03782768874524067</v>
-      </c>
-      <c r="J83" t="n">
-        <v>0.859961603843435</v>
-      </c>
-      <c r="K83" t="n">
-        <v>-0.01503350245593893</v>
-      </c>
+        <v>45813</v>
+      </c>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Tivio Top Manager Global</t>
+          <t>Tivio Top Gestor HY</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
+          <t>TIVIO TOP GESTOR HY FIF RL</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>MSCI ACWI</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -8992,43 +8996,33 @@
         </is>
       </c>
       <c r="F84" s="1" t="n">
-        <v>45195</v>
-      </c>
-      <c r="G84" t="n">
-        <v>0.6834526851150575</v>
-      </c>
-      <c r="H84" t="n">
-        <v>0.8062550197741138</v>
-      </c>
-      <c r="I84" t="n">
-        <v>-0.1228023346590563</v>
-      </c>
-      <c r="J84" t="n">
-        <v>0.8476879750857719</v>
-      </c>
-      <c r="K84" t="n">
-        <v>-0.02322669426482782</v>
-      </c>
+        <v>45813</v>
+      </c>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Tivio Top Manager Global</t>
+          <t>Tivio Top Gestor HY</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
+          <t>TIVIO TOP GESTOR HY FIF RL</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>MSCI ACWI</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -9037,38 +9031,38 @@
         </is>
       </c>
       <c r="F85" s="1" t="n">
-        <v>41978</v>
+        <v>45813</v>
       </c>
       <c r="G85" t="n">
-        <v>4.0049474242</v>
+        <v>0.2152430848</v>
       </c>
       <c r="H85" t="n">
-        <v>4.3466175936699</v>
+        <v>0.1976126726386125</v>
       </c>
       <c r="I85" t="n">
-        <v>-0.3416701694699</v>
+        <v>0.0176304121613875</v>
       </c>
       <c r="J85" t="n">
-        <v>0.9213940122159622</v>
+        <v>1.089217011874686</v>
       </c>
       <c r="K85" t="n">
-        <v>-0.005600653521803611</v>
+        <v>0.01112061570541045</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Tivio RF Ativo Longo Prazo</t>
+          <t>BV Top Gestor RF Ativo</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
+          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -9085,35 +9079,35 @@
         <v>46265</v>
       </c>
       <c r="G86" t="n">
-        <v>0.0155703610771285</v>
+        <v>0.009832721928012766</v>
       </c>
       <c r="H86" t="n">
         <v>0.01082559188004661</v>
       </c>
       <c r="I86" t="n">
-        <v>0.004744769197081888</v>
+        <v>-0.000992869952033848</v>
       </c>
       <c r="J86" t="n">
-        <v>1.43829189661466</v>
+        <v>0.9082849267702513</v>
       </c>
       <c r="K86" t="n">
-        <v>0.05780463920320189</v>
+        <v>-0.01172337186485095</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Tivio RF Ativo Longo Prazo</t>
+          <t>BV Top Gestor RF Ativo</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
+          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -9130,35 +9124,35 @@
         <v>46022</v>
       </c>
       <c r="G87" t="n">
-        <v>0.08726921494637052</v>
+        <v>0.09190461218917045</v>
       </c>
       <c r="H87" t="n">
         <v>0.1051127846901438</v>
       </c>
       <c r="I87" t="n">
-        <v>-0.01784356974377332</v>
+        <v>-0.01320817250097339</v>
       </c>
       <c r="J87" t="n">
-        <v>0.8302435826776601</v>
+        <v>0.8743428542977999</v>
       </c>
       <c r="K87" t="n">
-        <v>-0.02169748156471796</v>
+        <v>-0.01607272996257303</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Tivio RF Ativo Longo Prazo</t>
+          <t>BV Top Gestor RF Ativo</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
+          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -9175,35 +9169,35 @@
         <v>45930</v>
       </c>
       <c r="G88" t="n">
-        <v>0.1254024677775691</v>
+        <v>0.129702412726495</v>
       </c>
       <c r="H88" t="n">
         <v>0.1447903912030524</v>
       </c>
       <c r="I88" t="n">
-        <v>-0.01938792342548323</v>
+        <v>-0.01508797847655741</v>
       </c>
       <c r="J88" t="n">
-        <v>0.866096615497821</v>
+        <v>0.8957943386215581</v>
       </c>
       <c r="K88" t="n">
-        <v>-0.01700268091430945</v>
+        <v>-0.01323184628895746</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Tivio RF Ativo Longo Prazo</t>
+          <t>BV Top Gestor RF Ativo</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
+          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -9220,35 +9214,35 @@
         <v>45561</v>
       </c>
       <c r="G89" t="n">
-        <v>0.2544840968352924</v>
+        <v>0.270242572217682</v>
       </c>
       <c r="H89" t="n">
         <v>0.2980670513506256</v>
       </c>
       <c r="I89" t="n">
-        <v>-0.04358295451533323</v>
+        <v>-0.02782447913294361</v>
       </c>
       <c r="J89" t="n">
-        <v>0.853781374634175</v>
+        <v>0.906650268767168</v>
       </c>
       <c r="K89" t="n">
-        <v>-0.01696433769312999</v>
+        <v>-0.01079702351532119</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Tivio RF Ativo Longo Prazo</t>
+          <t>BV Top Gestor RF Ativo</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
+          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -9262,38 +9256,28 @@
         </is>
       </c>
       <c r="F90" s="1" t="n">
-        <v>45195</v>
-      </c>
-      <c r="G90" t="n">
-        <v>0.3777127110637792</v>
-      </c>
-      <c r="H90" t="n">
-        <v>0.4424561999402108</v>
-      </c>
-      <c r="I90" t="n">
-        <v>-0.06474348887643155</v>
-      </c>
-      <c r="J90" t="n">
-        <v>0.8536725468302165</v>
-      </c>
-      <c r="K90" t="n">
-        <v>-0.01521096373123265</v>
-      </c>
+        <v>45198</v>
+      </c>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Tivio RF Ativo Longo Prazo</t>
+          <t>BV Top Gestor RF Ativo</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
+          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -9307,43 +9291,43 @@
         </is>
       </c>
       <c r="F91" s="1" t="n">
-        <v>36392</v>
+        <v>45198</v>
       </c>
       <c r="G91" t="n">
-        <v>22.17376941860116</v>
+        <v>0.399945644</v>
       </c>
       <c r="H91" t="n">
-        <v>21.93717469453623</v>
+        <v>0.4404121868646469</v>
       </c>
       <c r="I91" t="n">
-        <v>0.2365947240649326</v>
+        <v>-0.0404665428646469</v>
       </c>
       <c r="J91" t="n">
-        <v>1.010785104616223</v>
+        <v>0.9081166596393855</v>
       </c>
       <c r="K91" t="n">
-        <v>0.0003791455748300976</v>
+        <v>-0.009503710662674081</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Tivio Prev Low Vol Itaú</t>
+          <t>Tivio Top Manager Global</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
+          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>MSCI ACWI</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -9355,40 +9339,40 @@
         <v>46265</v>
       </c>
       <c r="G92" t="n">
-        <v>0.01528942439290315</v>
+        <v>0.001361630876498987</v>
       </c>
       <c r="H92" t="n">
-        <v>0.01082559188004661</v>
+        <v>-0.01270714044827159</v>
       </c>
       <c r="I92" t="n">
-        <v>0.004463832512856536</v>
+        <v>0.01406877132477058</v>
       </c>
       <c r="J92" t="n">
-        <v>1.412340735021069</v>
+        <v>-0.1071547829381389</v>
       </c>
       <c r="K92" t="n">
-        <v>0.05429853764221493</v>
+        <v>0.1850574526325846</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Tivio Prev Low Vol Itaú</t>
+          <t>Tivio Top Manager Global</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
+          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>MSCI ACWI</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -9400,40 +9384,40 @@
         <v>46022</v>
       </c>
       <c r="G93" t="n">
-        <v>0.1025226903097796</v>
+        <v>0.06432757633456698</v>
       </c>
       <c r="H93" t="n">
-        <v>0.1051127846901438</v>
+        <v>0.05306746240220672</v>
       </c>
       <c r="I93" t="n">
-        <v>-0.002590094380364283</v>
+        <v>0.01126011393236026</v>
       </c>
       <c r="J93" t="n">
-        <v>0.9753589024589209</v>
+        <v>1.212184894898838</v>
       </c>
       <c r="K93" t="n">
-        <v>-0.003157118560559224</v>
+        <v>0.01443610338441359</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Tivio Prev Low Vol Itaú</t>
+          <t>Tivio Top Manager Global</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
+          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>MSCI ACWI</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -9445,40 +9429,40 @@
         <v>45930</v>
       </c>
       <c r="G94" t="n">
-        <v>0.1410909765555666</v>
+        <v>0.1275037236060828</v>
       </c>
       <c r="H94" t="n">
-        <v>0.1447903912030524</v>
+        <v>0.1224734191492385</v>
       </c>
       <c r="I94" t="n">
-        <v>-0.003699414647485799</v>
+        <v>0.00503030445684427</v>
       </c>
       <c r="J94" t="n">
-        <v>0.9744498608177818</v>
+        <v>1.041072622057809</v>
       </c>
       <c r="K94" t="n">
-        <v>-0.00324437507950126</v>
+        <v>0.004499340868773238</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Tivio Prev Low Vol Itaú</t>
+          <t>Tivio Top Manager Global</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
+          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>MSCI ACWI</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -9490,40 +9474,40 @@
         <v>45561</v>
       </c>
       <c r="G95" t="n">
-        <v>0.2822773175556004</v>
+        <v>0.2322960043521065</v>
       </c>
       <c r="H95" t="n">
-        <v>0.2980670513506256</v>
+        <v>0.2701236930973472</v>
       </c>
       <c r="I95" t="n">
-        <v>-0.01578973379502524</v>
+        <v>-0.03782768874524067</v>
       </c>
       <c r="J95" t="n">
-        <v>0.9470262354611907</v>
+        <v>0.859961603843435</v>
       </c>
       <c r="K95" t="n">
-        <v>-0.00611271794908208</v>
+        <v>-0.01503350245593893</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Tivio Prev Low Vol Itaú</t>
+          <t>Tivio Top Manager Global</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
+          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>MSCI ACWI</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -9535,40 +9519,40 @@
         <v>45195</v>
       </c>
       <c r="G96" t="n">
-        <v>0.4184670843779219</v>
+        <v>0.6834526851150575</v>
       </c>
       <c r="H96" t="n">
-        <v>0.4424561999402108</v>
+        <v>0.8062550197741138</v>
       </c>
       <c r="I96" t="n">
-        <v>-0.02398911556228889</v>
+        <v>-0.1228023346590563</v>
       </c>
       <c r="J96" t="n">
-        <v>0.9457819427877142</v>
+        <v>0.8476879750857719</v>
       </c>
       <c r="K96" t="n">
-        <v>-0.005581961690141801</v>
+        <v>-0.02322669426482782</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Tivio Prev Low Vol Itaú</t>
+          <t>Tivio Top Manager Global</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
+          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>MSCI ACWI</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -9577,38 +9561,38 @@
         </is>
       </c>
       <c r="F97" s="1" t="n">
-        <v>44917</v>
+        <v>41978</v>
       </c>
       <c r="G97" t="n">
-        <v>0.56223</v>
+        <v>4.0049474242</v>
       </c>
       <c r="H97" t="n">
-        <v>0.5882420554079393</v>
+        <v>4.3466175936699</v>
       </c>
       <c r="I97" t="n">
-        <v>-0.02601205540793927</v>
+        <v>-0.3416701694699</v>
       </c>
       <c r="J97" t="n">
-        <v>0.9557800140795778</v>
+        <v>0.9213940122159622</v>
       </c>
       <c r="K97" t="n">
-        <v>-0.004389281550695734</v>
+        <v>-0.005600653521803611</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus CDI</t>
+          <t>Tivio RF Ativo Longo Prazo</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
+          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -9625,35 +9609,35 @@
         <v>46265</v>
       </c>
       <c r="G98" t="n">
-        <v>-0.001462081025388806</v>
+        <v>0.0155703610771285</v>
       </c>
       <c r="H98" t="n">
         <v>0.01082559188004661</v>
       </c>
       <c r="I98" t="n">
-        <v>-0.01228767290543542</v>
+        <v>0.004744769197081888</v>
       </c>
       <c r="J98" t="n">
-        <v>-0.1350578371685771</v>
+        <v>1.43829189661466</v>
       </c>
       <c r="K98" t="n">
-        <v>-0.1365046674965383</v>
+        <v>0.05780463920320189</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus CDI</t>
+          <t>Tivio RF Ativo Longo Prazo</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
+          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -9670,35 +9654,35 @@
         <v>46022</v>
       </c>
       <c r="G99" t="n">
-        <v>0.08638432471204283</v>
+        <v>0.08726921494637052</v>
       </c>
       <c r="H99" t="n">
         <v>0.1051127846901438</v>
       </c>
       <c r="I99" t="n">
-        <v>-0.01872845997810102</v>
+        <v>-0.01784356974377332</v>
       </c>
       <c r="J99" t="n">
-        <v>0.8218250992654261</v>
+        <v>0.8302435826776601</v>
       </c>
       <c r="K99" t="n">
-        <v>-0.0227702919562276</v>
+        <v>-0.02169748156471796</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus CDI</t>
+          <t>Tivio RF Ativo Longo Prazo</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
+          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -9712,28 +9696,38 @@
         </is>
       </c>
       <c r="F100" s="1" t="n">
-        <v>45950</v>
-      </c>
-      <c r="G100" t="inlineStr"/>
-      <c r="H100" t="inlineStr"/>
-      <c r="I100" t="inlineStr"/>
-      <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr"/>
+        <v>45930</v>
+      </c>
+      <c r="G100" t="n">
+        <v>0.1254024677775691</v>
+      </c>
+      <c r="H100" t="n">
+        <v>0.1447903912030524</v>
+      </c>
+      <c r="I100" t="n">
+        <v>-0.01938792342548323</v>
+      </c>
+      <c r="J100" t="n">
+        <v>0.866096615497821</v>
+      </c>
+      <c r="K100" t="n">
+        <v>-0.01700268091430945</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus CDI</t>
+          <t>Tivio RF Ativo Longo Prazo</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
+          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -9747,28 +9741,38 @@
         </is>
       </c>
       <c r="F101" s="1" t="n">
-        <v>45950</v>
-      </c>
-      <c r="G101" t="inlineStr"/>
-      <c r="H101" t="inlineStr"/>
-      <c r="I101" t="inlineStr"/>
-      <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
+        <v>45561</v>
+      </c>
+      <c r="G101" t="n">
+        <v>0.2544840968352924</v>
+      </c>
+      <c r="H101" t="n">
+        <v>0.2980670513506256</v>
+      </c>
+      <c r="I101" t="n">
+        <v>-0.04358295451533323</v>
+      </c>
+      <c r="J101" t="n">
+        <v>0.853781374634175</v>
+      </c>
+      <c r="K101" t="n">
+        <v>-0.01696433769312999</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus CDI</t>
+          <t>Tivio RF Ativo Longo Prazo</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
+          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -9782,28 +9786,38 @@
         </is>
       </c>
       <c r="F102" s="1" t="n">
-        <v>45950</v>
-      </c>
-      <c r="G102" t="inlineStr"/>
-      <c r="H102" t="inlineStr"/>
-      <c r="I102" t="inlineStr"/>
-      <c r="J102" t="inlineStr"/>
-      <c r="K102" t="inlineStr"/>
+        <v>45195</v>
+      </c>
+      <c r="G102" t="n">
+        <v>0.3777127110637792</v>
+      </c>
+      <c r="H102" t="n">
+        <v>0.4424561999402108</v>
+      </c>
+      <c r="I102" t="n">
+        <v>-0.06474348887643155</v>
+      </c>
+      <c r="J102" t="n">
+        <v>0.8536725468302165</v>
+      </c>
+      <c r="K102" t="n">
+        <v>-0.01521096373123265</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus CDI</t>
+          <t>Tivio RF Ativo Longo Prazo</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
+          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -9817,43 +9831,43 @@
         </is>
       </c>
       <c r="F103" s="1" t="n">
-        <v>45950</v>
+        <v>36392</v>
       </c>
       <c r="G103" t="n">
-        <v>0.1194341999999999</v>
+        <v>22.17376941860116</v>
       </c>
       <c r="H103" t="n">
-        <v>0.1359909271883835</v>
+        <v>21.93717469453623</v>
       </c>
       <c r="I103" t="n">
-        <v>-0.01655672718838352</v>
+        <v>0.2365947240649326</v>
       </c>
       <c r="J103" t="n">
-        <v>0.8782512368237032</v>
+        <v>1.010785104616223</v>
       </c>
       <c r="K103" t="n">
-        <v>-0.0154899691480026</v>
+        <v>0.0003791455748300976</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>esplanada</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Tivio Esplanada</t>
+          <t>Tivio Prev Low Vol Itaú</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>IMA-B 5</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -9865,40 +9879,40 @@
         <v>46265</v>
       </c>
       <c r="G104" t="n">
-        <v>0.01003070736812051</v>
+        <v>0.01528942439290315</v>
       </c>
       <c r="H104" t="n">
-        <v>0.0200519906458918</v>
+        <v>0.01082559188004661</v>
       </c>
       <c r="I104" t="n">
-        <v>-0.0100212832777713</v>
+        <v>0.004463832512856536</v>
       </c>
       <c r="J104" t="n">
-        <v>0.5002349913910203</v>
+        <v>1.412340735021069</v>
       </c>
       <c r="K104" t="n">
-        <v>-0.1117254109753738</v>
+        <v>0.05429853764221493</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>esplanada</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Tivio Esplanada</t>
+          <t>Tivio Prev Low Vol Itaú</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>IMA-B 5</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -9910,40 +9924,40 @@
         <v>46022</v>
       </c>
       <c r="G105" t="n">
-        <v>0.07172731728642034</v>
+        <v>0.1025226903097796</v>
       </c>
       <c r="H105" t="n">
-        <v>0.1136619152554992</v>
+        <v>0.1051127846901438</v>
       </c>
       <c r="I105" t="n">
-        <v>-0.04193459796907884</v>
+        <v>-0.002590094380364283</v>
       </c>
       <c r="J105" t="n">
-        <v>0.6310584959367033</v>
+        <v>0.9753589024589209</v>
       </c>
       <c r="K105" t="n">
-        <v>-0.05040838364525002</v>
+        <v>-0.003157118560559224</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>esplanada</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Tivio Esplanada</t>
+          <t>Tivio Prev Low Vol Itaú</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>IMA-B 5</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -9955,40 +9969,40 @@
         <v>45930</v>
       </c>
       <c r="G106" t="n">
-        <v>0.09357535556093843</v>
+        <v>0.1410909765555666</v>
       </c>
       <c r="H106" t="n">
-        <v>0.1479693332684646</v>
+        <v>0.1447903912030524</v>
       </c>
       <c r="I106" t="n">
-        <v>-0.05439397770752619</v>
+        <v>-0.003699414647485799</v>
       </c>
       <c r="J106" t="n">
-        <v>0.6323969534360354</v>
+        <v>0.9744498608177818</v>
       </c>
       <c r="K106" t="n">
-        <v>-0.0475669929009177</v>
+        <v>-0.00324437507950126</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>esplanada</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Tivio Esplanada</t>
+          <t>Tivio Prev Low Vol Itaú</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>IMA-B 5</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -9997,33 +10011,43 @@
         </is>
       </c>
       <c r="F107" s="1" t="n">
-        <v>45586</v>
-      </c>
-      <c r="G107" t="inlineStr"/>
-      <c r="H107" t="inlineStr"/>
-      <c r="I107" t="inlineStr"/>
-      <c r="J107" t="inlineStr"/>
-      <c r="K107" t="inlineStr"/>
+        <v>45561</v>
+      </c>
+      <c r="G107" t="n">
+        <v>0.2822773175556004</v>
+      </c>
+      <c r="H107" t="n">
+        <v>0.2980670513506256</v>
+      </c>
+      <c r="I107" t="n">
+        <v>-0.01578973379502524</v>
+      </c>
+      <c r="J107" t="n">
+        <v>0.9470262354611907</v>
+      </c>
+      <c r="K107" t="n">
+        <v>-0.00611271794908208</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>esplanada</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Tivio Esplanada</t>
+          <t>Tivio Prev Low Vol Itaú</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>IMA-B 5</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -10032,33 +10056,43 @@
         </is>
       </c>
       <c r="F108" s="1" t="n">
-        <v>45586</v>
-      </c>
-      <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
-      <c r="I108" t="inlineStr"/>
-      <c r="J108" t="inlineStr"/>
-      <c r="K108" t="inlineStr"/>
+        <v>45195</v>
+      </c>
+      <c r="G108" t="n">
+        <v>0.4184670843779219</v>
+      </c>
+      <c r="H108" t="n">
+        <v>0.4424561999402108</v>
+      </c>
+      <c r="I108" t="n">
+        <v>-0.02398911556228889</v>
+      </c>
+      <c r="J108" t="n">
+        <v>0.9457819427877142</v>
+      </c>
+      <c r="K108" t="n">
+        <v>-0.005581961690141801</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>esplanada</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Tivio Esplanada</t>
+          <t>Tivio Prev Low Vol Itaú</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>IMA-B 5</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -10067,38 +10101,38 @@
         </is>
       </c>
       <c r="F109" s="1" t="n">
-        <v>45586</v>
+        <v>44917</v>
       </c>
       <c r="G109" t="n">
-        <v>0.2135222000000001</v>
+        <v>0.56223</v>
       </c>
       <c r="H109" t="n">
-        <v>0.2465452463189715</v>
+        <v>0.5882420554079393</v>
       </c>
       <c r="I109" t="n">
-        <v>-0.03302304631897135</v>
+        <v>-0.02601205540793927</v>
       </c>
       <c r="J109" t="n">
-        <v>0.8660568523951693</v>
+        <v>0.9557800140795778</v>
       </c>
       <c r="K109" t="n">
-        <v>-0.01382518449086667</v>
+        <v>-0.004389281550695734</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>legacy</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Tivio Legacy Prev</t>
+          <t>Tivio Infra Plus CDI</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -10115,35 +10149,35 @@
         <v>46265</v>
       </c>
       <c r="G110" t="n">
-        <v>0.01025992096101835</v>
+        <v>-0.001462081025388806</v>
       </c>
       <c r="H110" t="n">
         <v>0.01082559188004661</v>
       </c>
       <c r="I110" t="n">
-        <v>-0.0005656709190282605</v>
+        <v>-0.01228767290543542</v>
       </c>
       <c r="J110" t="n">
-        <v>0.9477468830068416</v>
+        <v>-0.1350578371685771</v>
       </c>
       <c r="K110" t="n">
-        <v>-0.006694722873975767</v>
+        <v>-0.1365046674965383</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>legacy</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Tivio Legacy Prev</t>
+          <t>Tivio Infra Plus CDI</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -10160,35 +10194,35 @@
         <v>46022</v>
       </c>
       <c r="G111" t="n">
-        <v>0.1002856499041807</v>
+        <v>0.08638432471204283</v>
       </c>
       <c r="H111" t="n">
         <v>0.1051127846901438</v>
       </c>
       <c r="I111" t="n">
-        <v>-0.004827134785963194</v>
+        <v>-0.01872845997810102</v>
       </c>
       <c r="J111" t="n">
-        <v>0.9540766158922263</v>
+        <v>0.8218250992654261</v>
       </c>
       <c r="K111" t="n">
-        <v>-0.00588181858317427</v>
+        <v>-0.0227702919562276</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>legacy</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Tivio Legacy Prev</t>
+          <t>Tivio Infra Plus CDI</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -10202,38 +10236,28 @@
         </is>
       </c>
       <c r="F112" s="1" t="n">
-        <v>45930</v>
-      </c>
-      <c r="G112" t="n">
-        <v>0.1394310574216069</v>
-      </c>
-      <c r="H112" t="n">
-        <v>0.1447903912030524</v>
-      </c>
-      <c r="I112" t="n">
-        <v>-0.005359333781445486</v>
-      </c>
-      <c r="J112" t="n">
-        <v>0.9629855701271667</v>
-      </c>
-      <c r="K112" t="n">
-        <v>-0.004700105358509954</v>
-      </c>
+        <v>45950</v>
+      </c>
+      <c r="G112" t="inlineStr"/>
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>legacy</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Tivio Legacy Prev</t>
+          <t>Tivio Infra Plus CDI</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -10247,38 +10271,28 @@
         </is>
       </c>
       <c r="F113" s="1" t="n">
-        <v>45561</v>
-      </c>
-      <c r="G113" t="n">
-        <v>0.288834593654415</v>
-      </c>
-      <c r="H113" t="n">
-        <v>0.2980670513506256</v>
-      </c>
-      <c r="I113" t="n">
-        <v>-0.009232457696210616</v>
-      </c>
-      <c r="J113" t="n">
-        <v>0.9690255677225116</v>
-      </c>
-      <c r="K113" t="n">
-        <v>-0.00356964896216394</v>
-      </c>
+        <v>45950</v>
+      </c>
+      <c r="G113" t="inlineStr"/>
+      <c r="H113" t="inlineStr"/>
+      <c r="I113" t="inlineStr"/>
+      <c r="J113" t="inlineStr"/>
+      <c r="K113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>legacy</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Tivio Legacy Prev</t>
+          <t>Tivio Infra Plus CDI</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -10292,66 +10306,576 @@
         </is>
       </c>
       <c r="F114" s="1" t="n">
-        <v>45195</v>
-      </c>
-      <c r="G114" t="n">
-        <v>0.4630786945344103</v>
-      </c>
-      <c r="H114" t="n">
-        <v>0.4424561999402108</v>
-      </c>
-      <c r="I114" t="n">
-        <v>0.02062249459419951</v>
-      </c>
-      <c r="J114" t="n">
-        <v>1.046609121076812</v>
-      </c>
-      <c r="K114" t="n">
-        <v>0.004749361817451225</v>
-      </c>
+        <v>45950</v>
+      </c>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr"/>
+      <c r="J114" t="inlineStr"/>
+      <c r="K114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
+          <t>infrapluscdi</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Tivio Infra Plus CDI</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>inicio</t>
+        </is>
+      </c>
+      <c r="F115" s="1" t="n">
+        <v>45950</v>
+      </c>
+      <c r="G115" t="n">
+        <v>0.1194341999999999</v>
+      </c>
+      <c r="H115" t="n">
+        <v>0.1359909271883835</v>
+      </c>
+      <c r="I115" t="n">
+        <v>-0.01655672718838352</v>
+      </c>
+      <c r="J115" t="n">
+        <v>0.8782512368237032</v>
+      </c>
+      <c r="K115" t="n">
+        <v>-0.0154899691480026</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>esplanada</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Tivio Esplanada</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>IMA-B 5</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="F116" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="G116" t="n">
+        <v>0.01003070736812051</v>
+      </c>
+      <c r="H116" t="n">
+        <v>0.0200519906458918</v>
+      </c>
+      <c r="I116" t="n">
+        <v>-0.0100212832777713</v>
+      </c>
+      <c r="J116" t="n">
+        <v>0.5002349913910203</v>
+      </c>
+      <c r="K116" t="n">
+        <v>-0.1117254109753738</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>esplanada</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Tivio Esplanada</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>IMA-B 5</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="F117" s="1" t="n">
+        <v>46022</v>
+      </c>
+      <c r="G117" t="n">
+        <v>0.07172731728642034</v>
+      </c>
+      <c r="H117" t="n">
+        <v>0.1136619152554992</v>
+      </c>
+      <c r="I117" t="n">
+        <v>-0.04193459796907884</v>
+      </c>
+      <c r="J117" t="n">
+        <v>0.6310584959367033</v>
+      </c>
+      <c r="K117" t="n">
+        <v>-0.05040838364525002</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>esplanada</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Tivio Esplanada</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>IMA-B 5</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>12m</t>
+        </is>
+      </c>
+      <c r="F118" s="1" t="n">
+        <v>45930</v>
+      </c>
+      <c r="G118" t="n">
+        <v>0.09357535556093843</v>
+      </c>
+      <c r="H118" t="n">
+        <v>0.1479693332684646</v>
+      </c>
+      <c r="I118" t="n">
+        <v>-0.05439397770752619</v>
+      </c>
+      <c r="J118" t="n">
+        <v>0.6323969534360354</v>
+      </c>
+      <c r="K118" t="n">
+        <v>-0.0475669929009177</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>esplanada</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Tivio Esplanada</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>IMA-B 5</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>24m</t>
+        </is>
+      </c>
+      <c r="F119" s="1" t="n">
+        <v>45586</v>
+      </c>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr"/>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>esplanada</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Tivio Esplanada</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>IMA-B 5</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>36m</t>
+        </is>
+      </c>
+      <c r="F120" s="1" t="n">
+        <v>45586</v>
+      </c>
+      <c r="G120" t="inlineStr"/>
+      <c r="H120" t="inlineStr"/>
+      <c r="I120" t="inlineStr"/>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>esplanada</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Tivio Esplanada</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>IMA-B 5</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>inicio</t>
+        </is>
+      </c>
+      <c r="F121" s="1" t="n">
+        <v>45586</v>
+      </c>
+      <c r="G121" t="n">
+        <v>0.2135222000000001</v>
+      </c>
+      <c r="H121" t="n">
+        <v>0.2465452463189715</v>
+      </c>
+      <c r="I121" t="n">
+        <v>-0.03302304631897135</v>
+      </c>
+      <c r="J121" t="n">
+        <v>0.8660568523951693</v>
+      </c>
+      <c r="K121" t="n">
+        <v>-0.01382518449086667</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
           <t>legacy</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr">
+      <c r="B122" t="inlineStr">
         <is>
           <t>Tivio Legacy Prev</t>
         </is>
       </c>
-      <c r="C115" t="inlineStr">
+      <c r="C122" t="inlineStr">
         <is>
           <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
         </is>
       </c>
-      <c r="D115" t="inlineStr">
+      <c r="D122" t="inlineStr">
         <is>
           <t>CDI</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr">
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="F122" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="G122" t="n">
+        <v>0.01025992096101835</v>
+      </c>
+      <c r="H122" t="n">
+        <v>0.01082559188004661</v>
+      </c>
+      <c r="I122" t="n">
+        <v>-0.0005656709190282605</v>
+      </c>
+      <c r="J122" t="n">
+        <v>0.9477468830068416</v>
+      </c>
+      <c r="K122" t="n">
+        <v>-0.006694722873975767</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>legacy</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="F123" s="1" t="n">
+        <v>46022</v>
+      </c>
+      <c r="G123" t="n">
+        <v>0.1002856499041807</v>
+      </c>
+      <c r="H123" t="n">
+        <v>0.1051127846901438</v>
+      </c>
+      <c r="I123" t="n">
+        <v>-0.004827134785963194</v>
+      </c>
+      <c r="J123" t="n">
+        <v>0.9540766158922263</v>
+      </c>
+      <c r="K123" t="n">
+        <v>-0.00588181858317427</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>legacy</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>12m</t>
+        </is>
+      </c>
+      <c r="F124" s="1" t="n">
+        <v>45930</v>
+      </c>
+      <c r="G124" t="n">
+        <v>0.1394310574216069</v>
+      </c>
+      <c r="H124" t="n">
+        <v>0.1447903912030524</v>
+      </c>
+      <c r="I124" t="n">
+        <v>-0.005359333781445486</v>
+      </c>
+      <c r="J124" t="n">
+        <v>0.9629855701271667</v>
+      </c>
+      <c r="K124" t="n">
+        <v>-0.004700105358509954</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>legacy</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>24m</t>
+        </is>
+      </c>
+      <c r="F125" s="1" t="n">
+        <v>45561</v>
+      </c>
+      <c r="G125" t="n">
+        <v>0.288834593654415</v>
+      </c>
+      <c r="H125" t="n">
+        <v>0.2980670513506256</v>
+      </c>
+      <c r="I125" t="n">
+        <v>-0.009232457696210616</v>
+      </c>
+      <c r="J125" t="n">
+        <v>0.9690255677225116</v>
+      </c>
+      <c r="K125" t="n">
+        <v>-0.00356964896216394</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>legacy</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>36m</t>
+        </is>
+      </c>
+      <c r="F126" s="1" t="n">
+        <v>45195</v>
+      </c>
+      <c r="G126" t="n">
+        <v>0.4630786945344103</v>
+      </c>
+      <c r="H126" t="n">
+        <v>0.4424561999402108</v>
+      </c>
+      <c r="I126" t="n">
+        <v>0.02062249459419951</v>
+      </c>
+      <c r="J126" t="n">
+        <v>1.046609121076812</v>
+      </c>
+      <c r="K126" t="n">
+        <v>0.004749361817451225</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>legacy</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
         <is>
           <t>inicio</t>
         </is>
       </c>
-      <c r="F115" s="1" t="n">
+      <c r="F127" s="1" t="n">
         <v>39674</v>
       </c>
-      <c r="G115" t="n">
+      <c r="G127" t="n">
         <v>4.4092549</v>
       </c>
-      <c r="H115" t="n">
+      <c r="H127" t="n">
         <v>4.604775473331634</v>
       </c>
-      <c r="I115" t="n">
+      <c r="I127" t="n">
         <v>-0.1955205733316348</v>
       </c>
-      <c r="J115" t="n">
+      <c r="J127" t="n">
         <v>0.957539607639073</v>
       </c>
-      <c r="K115" t="n">
+      <c r="K127" t="n">
         <v>-0.001963351321792373</v>
       </c>
     </row>
@@ -10366,7 +10890,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -10732,27 +11256,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BV Top Gestor Crédito Privado</t>
+          <t>Tivio HGD30</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>36.157.723/0001-46</t>
+          <t>59.889.169/0001-97</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0,25% a.a.</t>
+          <t>0,30% a.a.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Não há</t>
+          <t>16% do que exceder 100% do CDI</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -10764,27 +11288,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>hyd60</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Tivio Top Gestor HY</t>
+          <t>Tivio HYD60</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>61.026.657/0001-12</t>
+          <t>64.111.034/0001-36</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0,35% a.a.</t>
+          <t>0,50% a.a.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Não há</t>
+          <t>20% do que exceder 100% do CDI</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -10796,22 +11320,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BV Top Gestor RF Ativo</t>
+          <t>BV Top Gestor Crédito Privado</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>26.190.911/0001-12</t>
+          <t>36.157.723/0001-46</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0,15% a.a.</t>
+          <t>0,25% a.a.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -10828,22 +11352,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Tivio Top Manager Global</t>
+          <t>Tivio Top Gestor HY</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>13.614.712/0001-42</t>
+          <t>61.026.657/0001-12</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0,70% a.a.</t>
+          <t>0,35% a.a.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -10860,27 +11384,27 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Tivio RF Ativo Longo Prazo</t>
+          <t>BV Top Gestor RF Ativo</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>00.836.263/0001-35</t>
+          <t>26.190.911/0001-12</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0,50% a.a.</t>
+          <t>0,15% a.a.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>20% do que exceder 100% do CDI</t>
+          <t>Não há</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -10892,22 +11416,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Tivio Prev Low Vol Itaú</t>
+          <t>Tivio Top Manager Global</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>45.512.215/0001-20</t>
+          <t>13.614.712/0001-42</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0,80% a.a.</t>
+          <t>0,70% a.a.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -10924,27 +11448,27 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus CDI</t>
+          <t>Tivio RF Ativo Longo Prazo</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>62.791.756/0001-53</t>
+          <t>00.836.263/0001-35</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0,75% a.a.</t>
+          <t>0,50% a.a.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Não há</t>
+          <t>20% do que exceder 100% do CDI</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -10956,22 +11480,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>esplanada</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Tivio Esplanada</t>
+          <t>Tivio Prev Low Vol Itaú</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>54.853.793/0001-10</t>
+          <t>45.512.215/0001-20</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0,475% a.a.</t>
+          <t>0,80% a.a.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -10988,30 +11512,94 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>infrapluscdi</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Tivio Infra Plus CDI</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>62.791.756/0001-53</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>0,75% a.a.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Não há</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>esplanada</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Tivio Esplanada</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>54.853.793/0001-10</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>0,475% a.a.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Não há</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>legacy</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>Tivio Legacy Prev</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>09.083.848/0001-04</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>0,50% a.a.</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>Não há</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>não</t>
         </is>
@@ -11028,7 +11616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -11141,24 +11729,24 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>tivio-email-fundos-credito.html</t>
+          <t>relatorio/credito_estruturado</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>alt180</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>o texto se refere a "julho" como o mês corrente — a data base é setembro</t>
+          <t>selos sem arquivo local em assets/selos (qr) — saem pela URL do site, e podem não aparecer nas exportações. Ver assets/selos/LEIA-ME.md</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>tivio-email-fundos-credito.html</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -11168,7 +11756,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Mz', 'Fiagro Sr']</t>
+          <t>o texto se refere a "julho" como o mês corrente — a data base é setembro</t>
         </is>
       </c>
     </row>
@@ -11180,29 +11768,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>alt90</t>
+          <t>alt180</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Sr']</t>
+          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Mz', 'Fiagro Sr']</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>tivio-post-credito-estruturado.html</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>topgestormacro</t>
+          <t>alt90</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>sem dados — rentabilidade e PL mantidos</t>
+          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Sr']</t>
         </is>
       </c>
     </row>
@@ -11214,7 +11802,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>topgestorlongonly</t>
+          <t>topgestormacro</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -11226,15 +11814,32 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>tivio-post-investment-solutions.html</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>topgestorlongonly</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>sem dados — rentabilidade e PL mantidos</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>tivio-central.html</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>tivio-central.html</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>card "Gerador de Relatório de Gestão · Incentivado CDI 30" removido: aponta para "Tivio Incentivado CDI 30 - Relatório de Gestão Mensal.html", que não existe nesta edição</t>
         </is>
@@ -11251,7 +11856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -11279,570 +11884,180 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tivio Banks - Relatório de Gestão - Setembro 2026.pdf</t>
+          <t>Relatório de Gestão - Crédito Privado - Setembro 2026.html</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>828790</v>
+        <v>3222919</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tivio Banks - Relatório de Gestão - Setembro 2026.pptx</t>
+          <t>Relatório de Gestão - Crédito Estruturado - Setembro 2026.html</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>pptx</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1959157</v>
+        <v>1060480</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tivio Institucional - Relatório de Gestão - Setembro 2026.pdf</t>
+          <t>tivio-hgd30-saiba-mais.html</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>835427</v>
+        <v>55563</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tivio Institucional - Relatório de Gestão - Setembro 2026.pptx</t>
+          <t>tivio-hyd60-saiba-mais.html</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>pptx</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1966259</v>
+        <v>58928</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tivio Institucional 15 - Relatório de Gestão - Setembro 2026.pdf</t>
+          <t>tivio-construtor-one-pager.html</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>838981</v>
+        <v>88025</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Tivio Institucional 15 - Relatório de Gestão - Setembro 2026.pptx</t>
+          <t>tivio-email-fundos-credito.html</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>pptx</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1985711</v>
+        <v>177281</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Tivio Institucional 30 - Relatório de Gestão - Setembro 2026.pdf</t>
+          <t>tivio-email-nordea-studio.html</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>834703</v>
+        <v>50469</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Tivio Institucional 30 - Relatório de Gestão - Setembro 2026.pptx</t>
+          <t>tivio-post-credito-estruturado.html</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>pptx</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1960500</v>
+        <v>120495</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus - Relatório de Gestão - Setembro 2026.pdf</t>
+          <t>tivio-post-credito-privado.html</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>809398</v>
+        <v>134864</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus - Relatório de Gestão - Setembro 2026.pptx</t>
+          <t>tivio-post-investment-solutions.html</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>pptx</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1945318</v>
+        <v>105526</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Tivio BVP - Relatório de Gestão - Setembro 2026.pdf</t>
+          <t>tivio-central.html</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>817905</v>
+        <v>65858</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Tivio BVP - Relatório de Gestão - Setembro 2026.pptx</t>
+          <t>index.html</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>pptx</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1942870</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Tivio RF CP - Relatório de Gestão - Setembro 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>827596</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Tivio RF CP - Relatório de Gestão - Setembro 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>1956665</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Tivio ALT 180 - Relatório de Gestão - Setembro 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>618952</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Tivio ALT 180 - Relatório de Gestão - Setembro 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>296292</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Tivio ALT 90 - Relatório de Gestão - Setembro 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>617096</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Tivio ALT 90 - Relatório de Gestão - Setembro 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>290888</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Tivio ALT Light - Relatório de Gestão - Setembro 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>612993</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Tivio ALT Light - Relatório de Gestão - Setembro 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>284127</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Tivio Infra Plus CDI - Relatório de Gestão - Setembro 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>830104</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Tivio Infra Plus CDI - Relatório de Gestão - Setembro 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>1960127</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Tivio Esplanada - Relatório de Gestão - Setembro 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>832464</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Tivio Esplanada - Relatório de Gestão - Setembro 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>1968015</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Tivio Legacy Prev - Relatório de Gestão - Setembro 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>830848</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Tivio Legacy Prev - Relatório de Gestão - Setembro 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>1959014</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Relatório de Gestão - Crédito Privado - Setembro 2026.html</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>3222919</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Relatório de Gestão - Crédito Estruturado - Setembro 2026.html</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>1060480</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>tivio-construtor-one-pager.html</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>88025</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>tivio-email-fundos-credito.html</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>177281</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>tivio-email-nordea-studio.html</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>50469</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>tivio-post-credito-estruturado.html</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>120495</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>tivio-post-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>134864</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>tivio-post-investment-solutions.html</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>105526</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>65858</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>destaques</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>jpg</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>4096</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>emails</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>png</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>index.html</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
         <v>394</v>
       </c>
     </row>

</xml_diff>

<commit_message>
AutomaTivio: previdência (HGD30/HYD60) com Informativo PPTX+PDF e gerador de e-mail; disclaimer novo nos Destaques; data de início do Infra Plus
- Informativo: preenche o PPTX dos clientes (mês, texto, PL, duration, alocação, rating, composição, setores) e gera PDF pelo PowerPoint; HYD60 ganha página de rentabilidade
- E-mail: gerador em central/ (PNG por bloco, ZIP, HTML) e, na rodada, PNG + HTML + .eml com imagens embutidas
- HYD60 com rentabilidade e histórico em todos os materiais; alocação do mês na previsão
- Composição por setor (Bancário inclui debênture de banco), sobre o total da carteira
- Texto do gestor em entrada/previdencia.md; config em configs/previdencia.yml
- Cards na Central: páginas Saiba mais, e-mail e Informativos
- Disclaimer "Material de divulgação" nos três carrosséis de Destaques
- Infra Plus: data de início exibida 15/07/2019 (gráfico segue a DePara)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -11616,7 +11616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -11746,24 +11746,24 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>tivio-email-fundos-credito.html</t>
+          <t>landing/hyd60</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>alt180</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>o texto se refere a "julho" como o mês corrente — a data base é setembro</t>
+          <t>selos sem arquivo local em assets/selos (qr) — saem pela URL do site, e podem não aparecer nas exportações. Ver assets/selos/LEIA-ME.md</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>tivio-email-fundos-credito.html</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -11773,7 +11773,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Mz', 'Fiagro Sr']</t>
+          <t>o texto se refere a "julho" como o mês corrente — a data base é setembro</t>
         </is>
       </c>
     </row>
@@ -11785,29 +11785,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>alt90</t>
+          <t>alt180</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Sr']</t>
+          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Mz', 'Fiagro Sr']</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>tivio-post-credito-estruturado.html</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>topgestormacro</t>
+          <t>alt90</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>sem dados — rentabilidade e PL mantidos</t>
+          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Sr']</t>
         </is>
       </c>
     </row>
@@ -11819,7 +11819,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>topgestorlongonly</t>
+          <t>topgestormacro</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -11831,15 +11831,32 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>tivio-post-investment-solutions.html</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>topgestorlongonly</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>sem dados — rentabilidade e PL mantidos</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>tivio-central.html</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>tivio-central.html</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>card "Gerador de Relatório de Gestão · Incentivado CDI 30" removido: aponta para "Tivio Incentivado CDI 30 - Relatório de Gestão Mensal.html", que não existe nesta edição</t>
         </is>
@@ -11856,7 +11873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -11884,180 +11901,705 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Relatório de Gestão - Crédito Privado - Setembro 2026.html</t>
+          <t>Tivio Banks - Relatório de Gestão - Setembro 2026.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3222919</v>
+        <v>828790</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Relatório de Gestão - Crédito Estruturado - Setembro 2026.html</t>
+          <t>Tivio Banks - Relatório de Gestão - Setembro 2026.pptx</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pptx</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1060480</v>
+        <v>1959157</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>tivio-hgd30-saiba-mais.html</t>
+          <t>Tivio Institucional - Relatório de Gestão - Setembro 2026.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>55563</v>
+        <v>835427</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>tivio-hyd60-saiba-mais.html</t>
+          <t>Tivio Institucional - Relatório de Gestão - Setembro 2026.pptx</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pptx</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>58928</v>
+        <v>1966288</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>tivio-construtor-one-pager.html</t>
+          <t>Tivio Institucional 15 - Relatório de Gestão - Setembro 2026.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>88025</v>
+        <v>838981</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>tivio-email-fundos-credito.html</t>
+          <t>Tivio Institucional 15 - Relatório de Gestão - Setembro 2026.pptx</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pptx</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>177281</v>
+        <v>1985711</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>tivio-email-nordea-studio.html</t>
+          <t>Tivio Institucional 30 - Relatório de Gestão - Setembro 2026.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>50469</v>
+        <v>834703</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>Tivio Institucional 30 - Relatório de Gestão - Setembro 2026.pptx</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pptx</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>120495</v>
+        <v>1960500</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>tivio-post-credito-privado.html</t>
+          <t>Tivio Infra Plus - Relatório de Gestão - Setembro 2026.pdf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>134864</v>
+        <v>809394</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>Tivio Infra Plus - Relatório de Gestão - Setembro 2026.pptx</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pptx</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>105526</v>
+        <v>1945317</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>tivio-central.html</t>
+          <t>Tivio BVP - Relatório de Gestão - Setembro 2026.pdf</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>65858</v>
+        <v>817905</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Tivio BVP - Relatório de Gestão - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1942870</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Tivio RF CP - Relatório de Gestão - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>827596</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Tivio RF CP - Relatório de Gestão - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1956665</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Tivio ALT 180 - Relatório de Gestão - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>618952</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Tivio ALT 180 - Relatório de Gestão - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>296292</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Tivio ALT 90 - Relatório de Gestão - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>617096</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Tivio ALT 90 - Relatório de Gestão - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>290888</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Tivio ALT Light - Relatório de Gestão - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>612993</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Tivio ALT Light - Relatório de Gestão - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>284127</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Tivio Infra Plus CDI - Relatório de Gestão - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>830146</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Tivio Infra Plus CDI - Relatório de Gestão - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1960267</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Tivio Esplanada - Relatório de Gestão - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>832191</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Tivio Esplanada - Relatório de Gestão - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1968199</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev - Relatório de Gestão - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>830709</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev - Relatório de Gestão - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1958853</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Relatório de Gestão - Crédito Privado - Setembro 2026.html</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>3222919</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Relatório de Gestão - Crédito Estruturado - Setembro 2026.html</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1060480</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>tivio-hgd30-saiba-mais.html</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>54182</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>tivio-hyd60-saiba-mais.html</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>60645</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>tivio-email-previdencia.html</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1503841</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>tivio-construtor-one-pager.html</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>88025</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>tivio-email-fundos-credito.html</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>177281</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>tivio-email-nordea-studio.html</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>50469</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>tivio-post-credito-estruturado.html</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>118195</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>tivio-post-credito-privado.html</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>132564</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>tivio-post-investment-solutions.html</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>103226</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>tivio-central.html</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>67785</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>destaques</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>jpg</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>4096</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>emails</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>png</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>hgd30</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>png</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>4096</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>hyd60</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>png</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>4096</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Informativo - HGD30 - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>4796542</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Informativo - HGD30 - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>510725</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Informativo - HYD60 - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>5421445</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Informativo - HYD60 - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>584211</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>index.html</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>html</t>
         </is>
       </c>
-      <c r="C13" t="n">
+      <c r="C48" t="n">
         <v>394</v>
       </c>
     </row>

</xml_diff>

<commit_message>
AutomaTivio: comentário de previdência automático, capa do HYD60 no e-mail e disclaimer maior nos Destaques
- Texto do HGD30/HYD60 montado sozinho: mercado do Institucional (comentarios.md) + frase com os números + complemento do mês (previdencia.md)
- Informativo: a letra da caixa de texto encolhe quando o texto do mês não cabe
- E-mail HYD60: capa publicada com o mês trocado por cima
- Destaques: disclaimer em 27 px, preenchendo a folha

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -12225,7 +12225,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1960267</v>
+        <v>1960127</v>
       </c>
     </row>
     <row r="24">
@@ -12240,7 +12240,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>832191</v>
+        <v>832464</v>
       </c>
     </row>
     <row r="25">
@@ -12255,7 +12255,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1968199</v>
+        <v>1968015</v>
       </c>
     </row>
     <row r="26">
@@ -12270,7 +12270,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>830709</v>
+        <v>830848</v>
       </c>
     </row>
     <row r="27">
@@ -12285,7 +12285,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1958853</v>
+        <v>1959014</v>
       </c>
     </row>
     <row r="28">
@@ -12345,7 +12345,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>60645</v>
+        <v>60953</v>
       </c>
     </row>
     <row r="32">
@@ -12360,7 +12360,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1503841</v>
+        <v>1614994</v>
       </c>
     </row>
     <row r="33">
@@ -12420,7 +12420,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>118195</v>
+        <v>118194</v>
       </c>
     </row>
     <row r="37">
@@ -12435,7 +12435,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>132564</v>
+        <v>132563</v>
       </c>
     </row>
     <row r="38">
@@ -12450,7 +12450,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>103226</v>
+        <v>103225</v>
       </c>
     </row>
     <row r="39">
@@ -12540,7 +12540,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4796542</v>
+        <v>4796546</v>
       </c>
     </row>
     <row r="45">
@@ -12555,7 +12555,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>510725</v>
+        <v>510468</v>
       </c>
     </row>
     <row r="46">
@@ -12570,7 +12570,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>5421445</v>
+        <v>5421585</v>
       </c>
     </row>
     <row r="47">
@@ -12585,7 +12585,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>584211</v>
+        <v>583788</v>
       </c>
     </row>
     <row r="48">

</xml_diff>

<commit_message>
AutomaTivio: comentário de previdência só no comentarios.md; páginas Saiba mais com ECharts, logo horizontal e características do HYD60
- Complemento do HGD30/HYD60 nas seções do próprio fundo em entrada/comentarios.md (previdencia.md removido); loader ignora notas <!-- -->
- Páginas: alocação em meia-rosca (HYD60 com retorno estimado), composição em rosca, setores e rating em ECharts, histórico com área
- Logo horizontal no topo, títulos menores
- HYD60: nome, CNPJ, data de início, PL, público alvo e taxas; benefícios no desenho do material publicado

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -5009,7 +5009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -5043,12 +5043,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>hgd30</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Tivio HGD30</t>
+          <t>BV Top Gestor Crédito Privado</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -5065,12 +5065,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>hyd60</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tivio HYD60</t>
+          <t>Tivio Top Gestor HY</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -5087,12 +5087,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BV Top Gestor Crédito Privado</t>
+          <t>BV Top Gestor RF Ativo</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -5109,100 +5109,100 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>topgestormacro</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tivio Top Gestor HY</t>
+          <t>BV Top Gestor Macro</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>comentário do gestor</t>
+          <t>rentabilidade</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>não preenchido no arquivo de comentários</t>
+          <t>sem cotas na dados_mensais</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestorlongonly</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BV Top Gestor RF Ativo</t>
+          <t>Top Gestor Ações Long Only</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>comentário do gestor</t>
+          <t>rentabilidade</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>não preenchido no arquivo de comentários</t>
+          <t>sem cotas na dados_mensais</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>topgestormacro</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BV Top Gestor Macro</t>
+          <t>Tivio Top Manager Global</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>rentabilidade</t>
+          <t>comentário do gestor</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>sem cotas na dados_mensais</t>
+          <t>não preenchido no arquivo de comentários</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>topgestorlongonly</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Top Gestor Ações Long Only</t>
+          <t>Tivio RF Ativo Longo Prazo</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>rentabilidade</t>
+          <t>comentário do gestor</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>sem cotas na dados_mensais</t>
+          <t>não preenchido no arquivo de comentários</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tivio Top Manager Global</t>
+          <t>Tivio Prev Low Vol Itaú</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -5219,64 +5219,20 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>atuarial</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Tivio RF Ativo Longo Prazo</t>
+          <t>Tivio Atuarial</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>comentário do gestor</t>
+          <t>rentabilidade</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
-        <is>
-          <t>não preenchido no arquivo de comentários</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>prevlowvol</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Tivio Prev Low Vol Itaú</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>comentário do gestor</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>não preenchido no arquivo de comentários</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>atuarial</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Tivio Atuarial</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>rentabilidade</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
         <is>
           <t>sem cotas na dados_mensais</t>
         </is>
@@ -12045,7 +12001,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1945317</v>
+        <v>1945467</v>
       </c>
     </row>
     <row r="12">
@@ -12135,7 +12091,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>296292</v>
+        <v>296099</v>
       </c>
     </row>
     <row r="18">
@@ -12150,7 +12106,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>617096</v>
+        <v>616955</v>
       </c>
     </row>
     <row r="19">
@@ -12165,7 +12121,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>290888</v>
+        <v>291169</v>
       </c>
     </row>
     <row r="20">
@@ -12180,7 +12136,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>612993</v>
+        <v>612857</v>
       </c>
     </row>
     <row r="21">
@@ -12195,7 +12151,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>284127</v>
+        <v>284172</v>
       </c>
     </row>
     <row r="22">
@@ -12210,7 +12166,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>830146</v>
+        <v>830104</v>
       </c>
     </row>
     <row r="23">
@@ -12225,7 +12181,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1960127</v>
+        <v>1960267</v>
       </c>
     </row>
     <row r="24">
@@ -12240,7 +12196,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>832464</v>
+        <v>832191</v>
       </c>
     </row>
     <row r="25">
@@ -12255,7 +12211,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1968015</v>
+        <v>1968199</v>
       </c>
     </row>
     <row r="26">
@@ -12270,7 +12226,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>830848</v>
+        <v>830709</v>
       </c>
     </row>
     <row r="27">
@@ -12285,7 +12241,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1959014</v>
+        <v>1958853</v>
       </c>
     </row>
     <row r="28">
@@ -12330,7 +12286,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>54182</v>
+        <v>56678</v>
       </c>
     </row>
     <row r="31">
@@ -12345,7 +12301,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>60953</v>
+        <v>64369</v>
       </c>
     </row>
     <row r="32">
@@ -12540,7 +12496,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4796546</v>
+        <v>4796541</v>
       </c>
     </row>
     <row r="45">
@@ -12570,7 +12526,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>5421585</v>
+        <v>5421581</v>
       </c>
     </row>
     <row r="47">

</xml_diff>

<commit_message>
AutomaTivio: Saiba mais como site externo (menu no cabeçalho, sem link para a Central); PDF dos Destaques também em pdf/
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -12001,7 +12001,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1945467</v>
+        <v>1945317</v>
       </c>
     </row>
     <row r="12">
@@ -12091,7 +12091,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>296099</v>
+        <v>296292</v>
       </c>
     </row>
     <row r="18">
@@ -12106,7 +12106,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>616955</v>
+        <v>617096</v>
       </c>
     </row>
     <row r="19">
@@ -12121,7 +12121,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>291169</v>
+        <v>290888</v>
       </c>
     </row>
     <row r="20">
@@ -12136,7 +12136,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>612857</v>
+        <v>612993</v>
       </c>
     </row>
     <row r="21">
@@ -12151,7 +12151,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>284172</v>
+        <v>284127</v>
       </c>
     </row>
     <row r="22">
@@ -12286,7 +12286,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>56678</v>
+        <v>56779</v>
       </c>
     </row>
     <row r="31">
@@ -12301,7 +12301,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>64369</v>
+        <v>64470</v>
       </c>
     </row>
     <row r="32">
@@ -12496,7 +12496,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4796541</v>
+        <v>4796542</v>
       </c>
     </row>
     <row r="45">
@@ -12526,7 +12526,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>5421581</v>
+        <v>5421582</v>
       </c>
     </row>
     <row r="47">

</xml_diff>

<commit_message>
AutomaTivio: Informativo na fonte Versos (instalada para o usuário e embutida no PPTX)
- assets/fontes: Versos (woff2 do CDN da marca + ttf para o PowerPoint) e Versos Light
- exporters/previdencia: instala o que falta, carrega na sessão do Windows e grava o PPTX com a fonte embutida antes do PDF
- texto do gestor e gráfico novo do HYD60 em Versos (antes herdavam a Aptos do tema)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -12166,7 +12166,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>830104</v>
+        <v>830146</v>
       </c>
     </row>
     <row r="23">
@@ -12181,7 +12181,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1960267</v>
+        <v>1960127</v>
       </c>
     </row>
     <row r="24">
@@ -12196,7 +12196,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>832191</v>
+        <v>832464</v>
       </c>
     </row>
     <row r="25">
@@ -12211,7 +12211,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1968199</v>
+        <v>1968015</v>
       </c>
     </row>
     <row r="26">
@@ -12226,7 +12226,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>830709</v>
+        <v>830848</v>
       </c>
     </row>
     <row r="27">
@@ -12241,7 +12241,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1958853</v>
+        <v>1959014</v>
       </c>
     </row>
     <row r="28">
@@ -12256,7 +12256,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3222919</v>
+        <v>3700787</v>
       </c>
     </row>
     <row r="29">
@@ -12271,7 +12271,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1060480</v>
+        <v>1538348</v>
       </c>
     </row>
     <row r="30">
@@ -12286,7 +12286,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>56779</v>
+        <v>534647</v>
       </c>
     </row>
     <row r="31">
@@ -12301,7 +12301,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>64470</v>
+        <v>542338</v>
       </c>
     </row>
     <row r="32">
@@ -12316,7 +12316,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1614994</v>
+        <v>2092862</v>
       </c>
     </row>
     <row r="33">
@@ -12496,7 +12496,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4796542</v>
+        <v>4796546</v>
       </c>
     </row>
     <row r="45">
@@ -12511,7 +12511,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>510468</v>
+        <v>419349</v>
       </c>
     </row>
     <row r="46">
@@ -12526,7 +12526,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>5421582</v>
+        <v>5421628</v>
       </c>
     </row>
     <row r="47">
@@ -12541,7 +12541,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>583788</v>
+        <v>550546</v>
       </c>
     </row>
     <row r="48">

</xml_diff>

<commit_message>
AutomaTivio: Saiba mais na pasta landing page, setas no menu, setores em treemap e número da meia-rosca no lugar
- saida/AAAA-MM/landing page/ com vendor/echarts (site externo); cards da Central apontam para lá
- menu do cabeçalho numa linha no desktop, com setas quando não cabe
- meia-rosca e rosca medidas em pixel: o número fica sempre dentro do vão
- exposição setorial em treemap (só no site; e-mail e Informativo seguem em barras)
- rótulo "Carrego (Setembro 2026)" como no material publicado

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -12286,7 +12286,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>534647</v>
+        <v>540082</v>
       </c>
     </row>
     <row r="31">
@@ -12301,7 +12301,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>542338</v>
+        <v>547770</v>
       </c>
     </row>
     <row r="32">
@@ -12316,7 +12316,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2092862</v>
+        <v>2092859</v>
       </c>
     </row>
     <row r="33">
@@ -12421,7 +12421,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>67785</v>
+        <v>67857</v>
       </c>
     </row>
     <row r="40">
@@ -12496,7 +12496,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4796546</v>
+        <v>4796543</v>
       </c>
     </row>
     <row r="45">
@@ -12526,7 +12526,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>5421628</v>
+        <v>5421631</v>
       </c>
     </row>
     <row r="47">

</xml_diff>

<commit_message>
AutomaTivio: QR Code novo (redes da Tivio Capital) em todos os materiais
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -11572,7 +11572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -11617,202 +11617,151 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>relatorio/bvp</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>bvp</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>selos sem arquivo local em assets/selos (qr) — saem pela URL do site, e podem não aparecer nas exportações. Ver assets/selos/LEIA-ME.md</t>
+          <t>logo não encontrado em assets/logos (procurei "tivio_bvp")</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>relatorio/bvp</t>
+          <t>relatorio/atuarial</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>bvp</t>
+          <t>atuarial</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>logo não encontrado em assets/logos (procurei "tivio_bvp")</t>
+          <t>relatório não gerado: sem dados nesta edição</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>relatorio/atuarial</t>
+          <t>relatorio/credito_privado</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>atuarial</t>
+          <t>bvp</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>relatório não gerado: sem dados nesta edição</t>
+          <t>logo não encontrado em assets/logos (procurei "tivio_bvp")</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>relatorio/credito_privado</t>
+          <t>tivio-email-fundos-credito.html</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>bvp</t>
+          <t>alt180</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>logo não encontrado em assets/logos (procurei "tivio_bvp")</t>
+          <t>o texto se refere a "julho" como o mês corrente — a data base é setembro</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>relatorio/credito_estruturado</t>
+          <t>tivio-post-credito-estruturado.html</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>alt180</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>selos sem arquivo local em assets/selos (qr) — saem pela URL do site, e podem não aparecer nas exportações. Ver assets/selos/LEIA-ME.md</t>
+          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Mz', 'Fiagro Sr']</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>landing/hyd60</t>
+          <t>tivio-post-credito-estruturado.html</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>alt90</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>selos sem arquivo local em assets/selos (qr) — saem pela URL do site, e podem não aparecer nas exportações. Ver assets/selos/LEIA-ME.md</t>
+          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Sr']</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>tivio-email-fundos-credito.html</t>
+          <t>tivio-post-investment-solutions.html</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>alt180</t>
+          <t>topgestormacro</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>o texto se refere a "julho" como o mês corrente — a data base é setembro</t>
+          <t>sem dados — rentabilidade e PL mantidos</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>tivio-post-investment-solutions.html</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>alt180</t>
+          <t>topgestorlongonly</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Mz', 'Fiagro Sr']</t>
+          <t>sem dados — rentabilidade e PL mantidos</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>tivio-central.html</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>alt90</t>
+          <t>tivio-central.html</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
-        <is>
-          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Sr']</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>tivio-post-investment-solutions.html</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>topgestormacro</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>sem dados — rentabilidade e PL mantidos</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>tivio-post-investment-solutions.html</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>topgestorlongonly</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>sem dados — rentabilidade e PL mantidos</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
         <is>
           <t>card "Gerador de Relatório de Gestão · Incentivado CDI 30" removido: aponta para "Tivio Incentivado CDI 30 - Relatório de Gestão Mensal.html", que não existe nesta edição</t>
         </is>
@@ -11866,7 +11815,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>828790</v>
+        <v>808818</v>
       </c>
     </row>
     <row r="3">
@@ -11881,7 +11830,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1959157</v>
+        <v>1964410</v>
       </c>
     </row>
     <row r="4">
@@ -11896,7 +11845,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>835427</v>
+        <v>815298</v>
       </c>
     </row>
     <row r="5">
@@ -11911,7 +11860,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1966288</v>
+        <v>1971592</v>
       </c>
     </row>
     <row r="6">
@@ -11926,7 +11875,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>838981</v>
+        <v>818853</v>
       </c>
     </row>
     <row r="7">
@@ -11941,7 +11890,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1985711</v>
+        <v>1990766</v>
       </c>
     </row>
     <row r="8">
@@ -11956,7 +11905,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>834703</v>
+        <v>814574</v>
       </c>
     </row>
     <row r="9">
@@ -11971,7 +11920,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1960500</v>
+        <v>1965551</v>
       </c>
     </row>
     <row r="10">
@@ -11986,7 +11935,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>809394</v>
+        <v>789265</v>
       </c>
     </row>
     <row r="11">
@@ -12001,7 +11950,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1945317</v>
+        <v>1950734</v>
       </c>
     </row>
     <row r="12">
@@ -12016,7 +11965,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>817905</v>
+        <v>797776</v>
       </c>
     </row>
     <row r="13">
@@ -12031,7 +11980,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1942870</v>
+        <v>1947704</v>
       </c>
     </row>
     <row r="14">
@@ -12046,7 +11995,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>827596</v>
+        <v>807467</v>
       </c>
     </row>
     <row r="15">
@@ -12061,7 +12010,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1956665</v>
+        <v>1961950</v>
       </c>
     </row>
     <row r="16">
@@ -12076,7 +12025,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>618952</v>
+        <v>598823</v>
       </c>
     </row>
     <row r="17">
@@ -12091,7 +12040,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>296292</v>
+        <v>300534</v>
       </c>
     </row>
     <row r="18">
@@ -12106,7 +12055,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>617096</v>
+        <v>596967</v>
       </c>
     </row>
     <row r="19">
@@ -12121,7 +12070,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>290888</v>
+        <v>296395</v>
       </c>
     </row>
     <row r="20">
@@ -12136,7 +12085,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>612993</v>
+        <v>592864</v>
       </c>
     </row>
     <row r="21">
@@ -12151,7 +12100,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>284127</v>
+        <v>289334</v>
       </c>
     </row>
     <row r="22">
@@ -12166,7 +12115,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>830146</v>
+        <v>810017</v>
       </c>
     </row>
     <row r="23">
@@ -12181,7 +12130,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1960127</v>
+        <v>1965143</v>
       </c>
     </row>
     <row r="24">
@@ -12196,7 +12145,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>832464</v>
+        <v>812335</v>
       </c>
     </row>
     <row r="25">
@@ -12211,7 +12160,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1968015</v>
+        <v>1973341</v>
       </c>
     </row>
     <row r="26">
@@ -12226,7 +12175,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>830848</v>
+        <v>810719</v>
       </c>
     </row>
     <row r="27">
@@ -12241,7 +12190,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1959014</v>
+        <v>1964297</v>
       </c>
     </row>
     <row r="28">
@@ -12256,7 +12205,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3700787</v>
+        <v>4965627</v>
       </c>
     </row>
     <row r="29">
@@ -12271,7 +12220,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1538348</v>
+        <v>1917800</v>
       </c>
     </row>
     <row r="30">
@@ -12331,7 +12280,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>88025</v>
+        <v>88038</v>
       </c>
     </row>
     <row r="34">
@@ -12376,7 +12325,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>118194</v>
+        <v>118207</v>
       </c>
     </row>
     <row r="37">
@@ -12391,7 +12340,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>132563</v>
+        <v>132576</v>
       </c>
     </row>
     <row r="38">
@@ -12406,7 +12355,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>103225</v>
+        <v>103238</v>
       </c>
     </row>
     <row r="39">
@@ -12496,7 +12445,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4796543</v>
+        <v>4829263</v>
       </c>
     </row>
     <row r="45">
@@ -12511,7 +12460,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>419349</v>
+        <v>422658</v>
       </c>
     </row>
     <row r="46">
@@ -12526,7 +12475,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>5421631</v>
+        <v>5454350</v>
       </c>
     </row>
     <row r="47">
@@ -12541,7 +12490,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>550546</v>
+        <v>553845</v>
       </c>
     </row>
     <row r="48">

</xml_diff>

<commit_message>
AutomaTivio: texto do HYD60 de setembro; comentário colado com HTML é convertido e o mercado próprio do fundo vale
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -11815,7 +11815,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>808818</v>
+        <v>808661</v>
       </c>
     </row>
     <row r="3">
@@ -12250,7 +12250,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>547770</v>
+        <v>547647</v>
       </c>
     </row>
     <row r="32">
@@ -12265,7 +12265,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2092859</v>
+        <v>2092660</v>
       </c>
     </row>
     <row r="33">
@@ -12445,7 +12445,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4829263</v>
+        <v>4829264</v>
       </c>
     </row>
     <row r="45">
@@ -12460,7 +12460,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>422658</v>
+        <v>423404</v>
       </c>
     </row>
     <row r="46">
@@ -12475,7 +12475,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>5454350</v>
+        <v>5454369</v>
       </c>
     </row>
     <row r="47">
@@ -12490,7 +12490,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>553845</v>
+        <v>554208</v>
       </c>
     </row>
     <row r="48">

</xml_diff>

<commit_message>
AutomaTivio: comentários do seu comentarios.md (HTML colado convertido, bloco novo vale sobre o antigo); Institucional 30 e Infra Plus CDI no e-mail da Ágora
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E166"/>
+  <dimension ref="A1:E174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -712,7 +712,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>infra</t>
+          <t>inst30</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -722,12 +722,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>[['Fundo', '1,10%', '4,66%', '10,20%', '19,42%', '29,69%', '75,20%', True], ['IMA-B 5', '1,24%', '7,80%', '12,94%', '22,65%', '32,69%', '85,54%', False], ['Alfa', '−0,14%', '−3,14%', '−2,75%', '−3,24%', '−3,01%', '−10,35%', False], ['%', '89%', '60%', '79%', '86%', '91%', '88%', False]]</t>
+          <t>[['Fundo', '—', '—', '—', '—', '—', '—', True], ['CDI', '—', '—', '—', '—', '—', '—', False], ['Alfa', '—', '—', '—', '—', '—', '—', False], ['%', '—', '—', '—', '—', '—', '—', False]]</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>[['Fundo', '1,01%', '7,05%', '9,10%', '20,79%', '32,41%', '79,20%', True], ['IMA-B 5', '2,01%', '11,37%', '14,80%', '25,30%', '36,15%', '91,68%', False], ['Alfa', '−1,00%', '−4,32%', '−5,70%', '−4,50%', '−3,74%', '−12,48%', False], ['%', '50,31%', '62,03%', '61,51%', '82,20%', '89,65%', '86,39%', False]]</t>
+          <t>[['Fundo', '1,10%', '10,65%', '14,53%', '−', '−', '27,31%', True], ['CDI', '1,08%', '10,51%', '14,48%', '−', '−', '27,07%', False], ['Alfa', '0,02%', '0,14%', '0,05%', '−', '−', '0,24%', False], ['%', '102%', '101%', '100%', '−', '−', '101%', False]]</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>infra</t>
+          <t>inst30</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -749,12 +749,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>[['Público Alvo', 'Investidores em geral'], ['Resgate', 'D+31'], ['Benchmark', 'IMA-B 5'], ['Taxa de Performance', 'Não há'], ['Taxa de Administração', '0,75% a.a.'], ['PL Médio (12M)', 'R$ 52,0 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
+          <t>[['Público Alvo', 'Investidores em geral'], ['Resgate', 'D+30'], ['Benchmark', 'CDI'], ['Taxa de Performance', '20% do que exceder 100% do CDI'], ['Taxa Global', '0,625% a.a.'], ['PL Médio (12M)', '—'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>[['Público Alvo', 'Investidores em geral'], ['Resgate', 'D+31'], ['Benchmark', 'IMA-B 5'], ['Taxa de Performance', 'Não há'], ['Taxa global', '0,75% a.a.'], ['PL Médio (12M)', 'R$ 46,6 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
+          <t>[['Público Alvo', 'Investidores em geral'], ['Resgate', 'D+30'], ['Benchmark', 'CDI'], ['Taxa de Performance', '20% do que exceder 100% do CDI'], ['Taxa global', '0,625% a.a.'], ['PL Médio (12M)', 'R$ 162,9 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
         </is>
       </c>
     </row>
@@ -766,7 +766,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>infra</t>
+          <t>inst30</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -776,12 +776,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>O TIVIO INFRA PLUS apresentou rentabilidade, isenta de imposto de renda, de 1,10% no mês, acumulando 4,66% no ano. A gestão manteve postura cautelosa, priorizando o encurtamento da duration. Destacam-se as debêntures de RUMO e NTS, enquanto Alloha Fibra foi a maior detratora.</t>
+          <t>O TIVIO INSTITUCIONAL 30 apresentou rentabilidade no mês. Na parcela de corporativos, os maiores atribuidores de resultado foram para Tupy e Randon, enquanto Hapvida foi o maior detrator.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>O TIVIO INFRA PLUS apresentou rentabilidade, isenta de imposto de renda, de 1,01% no mês, acumulando 7,05% no ano. A gestão manteve postura cautelosa, priorizando o encurtamento da duration. Destacam-se as debêntures de RUMO e NTS, enquanto Alloha Fibra foi a maior detratora.</t>
+          <t>O TIVIO INSTITUCIONAL 30 apresentou rentabilidade de 1,10% no mês (102% do CDI), acumulando 10,65% no ano. Na parcela de corporativos, os maiores atribuidores de resultado foram para Tupy e Randon, enquanto Hapvida foi o maior detrator.</t>
         </is>
       </c>
     </row>
@@ -793,7 +793,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>altlight</t>
+          <t>infra</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -803,12 +803,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>[['Fundo', '1,23%', '8,73%', '−', '−', '−', '11,79%', True], ['CDI', '1,22%', '8,14%', '−', '−', '−', '10,19%', False], ['CDI+', '0,12%', '0,94%', '−', '−', '−', '2,05%', False], ['%', '101%', '107%', '−', '−', '−', '116%', False]]</t>
+          <t>[['Fundo', '1,10%', '4,66%', '10,20%', '19,42%', '29,69%', '75,20%', True], ['IMA-B 5', '1,24%', '7,80%', '12,94%', '22,65%', '32,69%', '85,54%', False], ['Alfa', '−0,14%', '−3,14%', '−2,75%', '−3,24%', '−3,01%', '−10,35%', False], ['%', '89%', '60%', '79%', '86%', '91%', '88%', False]]</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>[['Fundo', '1,03%', '10,64%', '−', '−', '−', '13,76%', True], ['CDI', '1,08%', '10,51%', '−', '−', '−', '12,60%', False], ['CDI+', '−0,58%', '0,16%', '−', '−', '−', '1,17%', False], ['%', '95,47%', '101,22%', '−', '−', '−', '109,18%', False]]</t>
+          <t>[['Fundo', '1,01%', '7,05%', '9,10%', '20,79%', '32,41%', '79,20%', True], ['IMA-B 5', '2,01%', '11,37%', '14,80%', '25,30%', '36,15%', '91,68%', False], ['Alfa', '−1,00%', '−4,32%', '−5,70%', '−4,50%', '−3,74%', '−12,48%', False], ['%', '50,31%', '62,03%', '61,51%', '82,20%', '89,65%', '86,39%', False]]</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>altlight</t>
+          <t>infra</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -830,12 +830,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>[['Público Alvo', 'Investidor qualificado'], ['Resgate', 'D+50'], ['Benchmark', 'CDI'], ['Taxa de Performance', '15% do que exceder CDI+0,65%'], ['Taxa de Administração', '1,15% a.a.'], ['PL (desde o início)', 'R$ 26,9 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
+          <t>[['Público Alvo', 'Investidores em geral'], ['Resgate', 'D+31'], ['Benchmark', 'IMA-B 5'], ['Taxa de Performance', 'Não há'], ['Taxa de Administração', '0,75% a.a.'], ['PL Médio (12M)', 'R$ 52,0 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>[['Público Alvo', 'Investidor qualificado'], ['Resgate', 'D+50'], ['Benchmark', 'CDI'], ['Taxa de Performance', '15% do retorno que exceder CDI+0,65%'], ['Taxa global', '1,15% a.a.'], ['PL (desde o início)', 'R$ 20,6 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
+          <t>[['Público Alvo', 'Investidores em geral'], ['Resgate', 'D+31'], ['Benchmark', 'IMA-B 5'], ['Taxa de Performance', 'Não há'], ['Taxa global', '0,75% a.a.'], ['PL Médio (12M)', 'R$ 46,6 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>altlight</t>
+          <t>infra</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -857,12 +857,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>O TIVIO ALT LIGHT apresentou rentabilidade de 1,23% no mês (101% do CDI), acumulando 8,73% no ano e 11,79% desde o início (116% do CDI). A parcela de debêntures foi a principal contribuidora, seguida pela parcela de crédito estruturado.</t>
+          <t>O TIVIO INFRA PLUS apresentou rentabilidade, isenta de imposto de renda, de 1,10% no mês, acumulando 4,66% no ano. A gestão manteve postura cautelosa, priorizando o encurtamento da duration. Destacam-se as debêntures de RUMO e NTS, enquanto Alloha Fibra foi a maior detratora.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>O TIVIO ALT LIGHT rendeu 1,03% no mês (95,47% do CDI), acumulando 10,64% no ano e 13,76% desde o início (CDI+1,17% ao ano). A parcela de debêntures foi a principal contribuidora, seguida pela parcela de crédito estruturado.</t>
+          <t>O TIVIO INFRA PLUS apresentou rentabilidade, isenta de imposto de renda, de 1,01% no mês, acumulando 7,05% no ano. A gestão manteve postura cautelosa, priorizando o encurtamento da duration. Destacam-se as debêntures de RUMO e NTS, enquanto Alloha Fibra foi a maior detratora.</t>
         </is>
       </c>
     </row>
@@ -874,7 +874,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>alt180</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -884,12 +884,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>[['Fundo', '1,45%', '9,76%', '18,56%', '−', '−', '31,44%', True], ['CDI', '1,22%', '8,14%', '14,65%', '−', '−', '24,08%', False], ['CDI+', '2,56%', '2,61%', '3,42%', '−', '−', '3,66%', False], ['%', '119%', '120%', '127%', '−', '−', '131%', False]]</t>
+          <t>[['Fundo', '—', '—', '—', '—', '—', '—', True], ['CDI', '—', '—', '—', '—', '—', '—', False], ['%', '—', '—', '—', '—', '—', '—', False]]</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>[['Fundo', '1,29%', '12,62%', '17,85%', '−', '−', '34,87%', True], ['CDI', '1,08%', '10,51%', '14,48%', '−', '−', '26,79%', False], ['CDI+', '2,53%', '2,58%', '2,95%', '−', '−', '3,55%', False], ['%', '119,45%', '120,09%', '123,25%', '−', '−', '130,15%', False]]</t>
+          <t>[['Fundo', '−0,15%', '8,64%', '−', '−', '−', '11,94%', True], ['CDI', '1,08%', '10,51%', '−', '−', '−', '13,60%', False], ['%', '−14%', '82%', '−', '−', '−', '88%', False]]</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>alt180</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -911,12 +911,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>[['Público Alvo', 'Investidores qualificados, Multi Family e Family Offices'], ['Resgate', 'D+180'], ['Benchmark', 'CDI'], ['Taxa de Performance', '20% do que exceder o CDI'], ['Taxa de Administração', '1,15% a.a.'], ['PL Médio (12M)', 'R$ 84,8 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
+          <t>[['Público Alvo', 'Investidores em geral'], ['Resgate', 'D+30'], ['Benchmark', 'CDI'], ['Taxa de Performance', 'Não há'], ['Taxa Global', '0,75% a.a.'], ['PL Médio (12M)', '—'], ['Aplicação Mínima', 'R$ 100,00']]</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>[['Público Alvo', 'Investidores qualificados, Multi Family e Family Offices'], ['Resgate', 'D+180'], ['Benchmark', 'CDI'], ['Taxa de Performance', '20% do que exceder do CDI'], ['Taxa global', '1,15% a.a.'], ['PL Médio (12M)', 'R$ 104,6 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
+          <t>[['Público Alvo', 'Investidores em geral'], ['Resgate', 'D+30'], ['Benchmark', 'CDI'], ['Taxa de Performance', 'Não há'], ['Taxa global', '0,75% a.a.'], ['PL Médio (12M)', 'R$ 38,0 mi'], ['Aplicação Mínima', 'R$ 100,00']]</t>
         </is>
       </c>
     </row>
@@ -928,7 +928,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>alt180</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -938,12 +938,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>O TIVIO ALT 180 rendeu 1,45% no mês (119% do CDI), acumulando 9,76% no ano e 31,44% desde o início (CDI+3,66% ao ano). Em julho aumentamos a exposição a FIDCs de Consignado Público, com elevada pulverização e baixa inadimplência.</t>
+          <t>O TIVIO INFRA PLUS CDI apresentou rentabilidade no mês. Na atribuição de performance, pode-se destacar as debêntures de Copel e CPFL, enquanto as de Energisa foram as maiores detratoras.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>O TIVIO ALT 180 rendeu 1,29% no mês (119,45% do CDI), acumulando 12,62% no ano e 34,87% desde o início (CDI+3,55% ao ano). Em julho aumentamos a exposição a FIDCs de Consignado Público, com elevada pulverização e baixa inadimplência.</t>
+          <t>O TIVIO INFRA PLUS CDI apresentou rentabilidade de −0,15% no mês (−14% do CDI), acumulando 8,64% no ano. Na atribuição de performance, pode-se destacar as debêntures de Copel e CPFL, enquanto as de Energisa foram as maiores detratoras.</t>
         </is>
       </c>
     </row>
@@ -955,7 +955,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>alt90</t>
+          <t>altlight</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -965,12 +965,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>[['Fundo', '1,36%', '9,06%', '16,72%', '−', '−', '19,79%', True], ['CDI', '1,22%', '8,14%', '14,65%', '−', '−', '17,13%', False], ['CDI+', '1,59%', '1,48%', '1,81%', '−', '−', '1,97%', False], ['%', '112%', '111%', '114%', '−', '−', '115%', False]]</t>
+          <t>[['Fundo', '1,23%', '8,73%', '−', '−', '−', '11,79%', True], ['CDI', '1,22%', '8,14%', '−', '−', '−', '10,19%', False], ['CDI+', '0,12%', '0,94%', '−', '−', '−', '2,05%', False], ['%', '101%', '107%', '−', '−', '−', '116%', False]]</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>[['Fundo', '1,17%', '11,69%', '16,25%', '−', '−', '22,67%', True], ['CDI', '1,08%', '10,51%', '14,48%', '−', '−', '19,70%', False], ['CDI+', '1,07%', '1,44%', '1,55%', '−', '−', '1,88%', False], ['%', '108,27%', '111,24%', '112,21%', '−', '−', '115,11%', False]]</t>
+          <t>[['Fundo', '1,03%', '10,64%', '−', '−', '−', '13,76%', True], ['CDI', '1,08%', '10,51%', '−', '−', '−', '12,60%', False], ['CDI+', '−0,58%', '0,16%', '−', '−', '−', '1,17%', False], ['%', '95,47%', '101,22%', '−', '−', '−', '109,18%', False]]</t>
         </is>
       </c>
     </row>
@@ -982,7 +982,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>alt90</t>
+          <t>altlight</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -992,12 +992,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>[['Público Alvo', 'Investidor qualificado'], ['Resgate', 'D+90'], ['Benchmark', 'CDI'], ['Taxa de Performance', '10% do que exceder o CDI'], ['Taxa de Administração', '1,25% a.a.'], ['PL Médio (12M)', 'R$ 14,3 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
+          <t>[['Público Alvo', 'Investidor qualificado'], ['Resgate', 'D+50'], ['Benchmark', 'CDI'], ['Taxa de Performance', '15% do que exceder CDI+0,65%'], ['Taxa de Administração', '1,15% a.a.'], ['PL (desde o início)', 'R$ 26,9 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>[['Público Alvo', 'Investidor qualificado'], ['Resgate', 'D+90'], ['Benchmark', 'CDI'], ['Taxa de Performance', '10% do que exceder do CDI'], ['Taxa global', '1,25% a.a.'], ['PL Médio (12M)', 'R$ 16,9 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
+          <t>[['Público Alvo', 'Investidor qualificado'], ['Resgate', 'D+50'], ['Benchmark', 'CDI'], ['Taxa de Performance', '15% do retorno que exceder CDI+0,65%'], ['Taxa global', '1,15% a.a.'], ['PL (desde o início)', 'R$ 20,6 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>alt90</t>
+          <t>altlight</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1019,12 +1019,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>O TIVIO ALT 90 rendeu 1,36% no mês (112% do CDI), acumulando 9,06% no ano e 19,79% desde o início (CDI+1,97% ao ano). A estratégia segue concentrada em FIDCs de cotas sênior, buscando retorno superior ao CDI com baixa volatilidade.</t>
+          <t>O TIVIO ALT LIGHT apresentou rentabilidade de 1,23% no mês (101% do CDI), acumulando 8,73% no ano e 11,79% desde o início (116% do CDI). A parcela de debêntures foi a principal contribuidora, seguida pela parcela de crédito estruturado.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>O TIVIO ALT 90 rendeu 1,17% no mês (108,27% do CDI), acumulando 11,69% no ano e 22,67% desde o início (CDI+1,88% ao ano). A estratégia segue concentrada em FIDCs de cotas sênior, buscando retorno superior ao CDI com baixa volatilidade.</t>
+          <t>O TIVIO ALT LIGHT rendeu 1,03% no mês (95,47% do CDI), acumulando 10,64% no ano e 13,76% desde o início (CDI+1,17% ao ano). A parcela de debêntures foi a principal contribuidora, seguida pela parcela de crédito estruturado.</t>
         </is>
       </c>
     </row>
@@ -1036,22 +1036,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>alt180</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>HIST</t>
+          <t>rows</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>até 2026-07</t>
+          <t>[['Fundo', '1,45%', '9,76%', '18,56%', '−', '−', '31,44%', True], ['CDI', '1,22%', '8,14%', '14,65%', '−', '−', '24,08%', False], ['CDI+', '2,56%', '2,61%', '3,42%', '−', '−', '3,66%', False], ['%', '119%', '120%', '127%', '−', '−', '131%', False]]</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>até 2026-09 (210 meses)</t>
+          <t>[['Fundo', '1,29%', '12,62%', '17,85%', '−', '−', '34,87%', True], ['CDI', '1,08%', '10,51%', '14,48%', '−', '−', '26,79%', False], ['CDI+', '2,53%', '2,58%', '2,95%', '−', '−', '3,55%', False], ['%', '119,45%', '120,09%', '123,25%', '−', '−', '130,15%', False]]</t>
         </is>
       </c>
     </row>
@@ -1063,22 +1063,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>alt180</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>HIST</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>até 2026-07</t>
+          <t>[['Público Alvo', 'Investidores qualificados, Multi Family e Family Offices'], ['Resgate', 'D+180'], ['Benchmark', 'CDI'], ['Taxa de Performance', '20% do que exceder o CDI'], ['Taxa de Administração', '1,15% a.a.'], ['PL Médio (12M)', 'R$ 84,8 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>até 2026-09 (257 meses)</t>
+          <t>[['Público Alvo', 'Investidores qualificados, Multi Family e Family Offices'], ['Resgate', 'D+180'], ['Benchmark', 'CDI'], ['Taxa de Performance', '20% do que exceder do CDI'], ['Taxa global', '1,15% a.a.'], ['PL Médio (12M)', 'R$ 104,6 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
         </is>
       </c>
     </row>
@@ -1090,22 +1090,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>inst15</t>
+          <t>alt180</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>HIST</t>
+          <t>comment</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>até 2026-07</t>
+          <t>O TIVIO ALT 180 rendeu 1,45% no mês (119% do CDI), acumulando 9,76% no ano e 31,44% desde o início (CDI+3,66% ao ano). Em julho aumentamos a exposição a FIDCs de Consignado Público, com elevada pulverização e baixa inadimplência.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>até 2026-09 (296 meses)</t>
+          <t>O TIVIO ALT 180 rendeu 1,29% no mês (119,45% do CDI), acumulando 12,62% no ano e 34,87% desde o início (CDI+3,55% ao ano). Em julho aumentamos a exposição a FIDCs de Consignado Público, com elevada pulverização e baixa inadimplência.</t>
         </is>
       </c>
     </row>
@@ -1117,22 +1117,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>infra</t>
+          <t>alt90</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>HIST</t>
+          <t>rows</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>até 2026-07</t>
+          <t>[['Fundo', '1,36%', '9,06%', '16,72%', '−', '−', '19,79%', True], ['CDI', '1,22%', '8,14%', '14,65%', '−', '−', '17,13%', False], ['CDI+', '1,59%', '1,48%', '1,81%', '−', '−', '1,97%', False], ['%', '112%', '111%', '114%', '−', '−', '115%', False]]</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>até 2026-09 (65 meses)</t>
+          <t>[['Fundo', '1,17%', '11,69%', '16,25%', '−', '−', '22,67%', True], ['CDI', '1,08%', '10,51%', '14,48%', '−', '−', '19,70%', False], ['CDI+', '1,07%', '1,44%', '1,55%', '−', '−', '1,88%', False], ['%', '108,27%', '111,24%', '112,21%', '−', '−', '115,11%', False]]</t>
         </is>
       </c>
     </row>
@@ -1144,22 +1144,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>altlight</t>
+          <t>alt90</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>HIST</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>até 2026-07</t>
+          <t>[['Público Alvo', 'Investidor qualificado'], ['Resgate', 'D+90'], ['Benchmark', 'CDI'], ['Taxa de Performance', '10% do que exceder o CDI'], ['Taxa de Administração', '1,25% a.a.'], ['PL Médio (12M)', 'R$ 14,3 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>até 2026-09 (11 meses)</t>
+          <t>[['Público Alvo', 'Investidor qualificado'], ['Resgate', 'D+90'], ['Benchmark', 'CDI'], ['Taxa de Performance', '10% do que exceder do CDI'], ['Taxa global', '1,25% a.a.'], ['PL Médio (12M)', 'R$ 16,9 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
         </is>
       </c>
     </row>
@@ -1171,22 +1171,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>alt180</t>
+          <t>alt90</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>HIST</t>
+          <t>comment</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>até 2026-07</t>
+          <t>O TIVIO ALT 90 rendeu 1,36% no mês (112% do CDI), acumulando 9,06% no ano e 19,79% desde o início (CDI+1,97% ao ano). A estratégia segue concentrada em FIDCs de cotas sênior, buscando retorno superior ao CDI com baixa volatilidade.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>até 2026-09 (22 meses)</t>
+          <t>O TIVIO ALT 90 rendeu 1,17% no mês (108,27% do CDI), acumulando 11,69% no ano e 22,67% desde o início (CDI+1,88% ao ano). A estratégia segue concentrada em FIDCs de cotas sênior, buscando retorno superior ao CDI com baixa volatilidade.</t>
         </is>
       </c>
     </row>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>alt90</t>
+          <t>banks</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>até 2026-09 (16 meses)</t>
+          <t>até 2026-09 (210 meses)</t>
         </is>
       </c>
     </row>
@@ -1225,22 +1225,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>HIST</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>31/07/2026</t>
+          <t>até 2026-07</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>até 2026-09 (257 meses)</t>
         </is>
       </c>
     </row>
@@ -1252,22 +1252,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>inst15</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>HIST</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Julho de 2026</t>
+          <t>até 2026-07</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Setembro de 2026</t>
+          <t>até 2026-09 (296 meses)</t>
         </is>
       </c>
     </row>
@@ -1279,22 +1279,22 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>infra</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>HIST</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>julho de 2026</t>
+          <t>até 2026-07</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>setembro de 2026</t>
+          <t>até 2026-09 (65 meses)</t>
         </is>
       </c>
     </row>
@@ -1306,29 +1306,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>altlight</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>libs de exportação</t>
+          <t>HIST</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>CDN</t>
+          <t>até 2026-07</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>4 referências → vendor/ local (CDN como reserva)</t>
+          <t>até 2026-09 (11 meses)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>tivio-email-fundos-credito.html</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1338,206 +1338,206 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>b1val</t>
+          <t>HIST</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>R$ 148.155.859,36</t>
+          <t>até 2026-07</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>R$ 153.589.286,51</t>
+          <t>até 2026-09 (22 meses)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>tivio-email-fundos-credito.html</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>alt180</t>
+          <t>alt90</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>b2val</t>
+          <t>HIST</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>R$ 84.791.205,56</t>
+          <t>até 2026-07</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>R$ 104.590.801,56</t>
+          <t>até 2026-09 (16 meses)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>tivio-email-fundos-credito.html</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>alt180</t>
+          <t>inst30</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>HIST</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>127%</t>
+          <t>até 2026-07</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>123%</t>
+          <t>até 2026-09 (22 meses)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>tivio-email-fundos-credito.html</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>alt180</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>HIST</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>[{'n': 'FIDCs Cotas Sênior', 'p': 49.6}, {'n': 'FIDCs Cotas Mezanino', 'p': 27.5}, {'n': 'Liquidez', 'p': 9.3}, {'n': 'Crédito Estruturado', 'p': 5.5}, {'n': 'Crédito Privado', 'p': 3.5}, {'n': 'Precatório', 'p': 2.8}, {'n': 'Fiagro', 'p': 2.0}]</t>
+          <t>até 2026-07</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>[{'n': 'FIDCs Cota Sênior', 'p': 49.3}, {'n': 'FIDCs Cota Mezanino', 'p': 27.0}, {'n': 'Liquidez', 'p': 9.1}, {'n': 'Crédito Estruturado', 'p': 5.5}, {'n': 'Crédito Privado', 'p': 3.4}, {'n': 'Fiagro', 'p': 3.2}, {'n': 'Precatório', 'p': 2.8}]</t>
+          <t>até 2026-09 (12 meses)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>tivio-email-fundos-credito.html</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>alt180</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Taxa de administração e gestão: 1,15% a.a. Taxa de performance: 20% do que exceder do CDI. Resgate: D+180.</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Taxa global: 1,15% a.a. Taxa de performance: 20% do que exceder do CDI. Resgate: D+180.</t>
+          <t>30/09/2026</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>tivio-email-fundos-credito.html</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>alt90</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>b1val</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>R$ 19.936.394,95</t>
+          <t>Julho de 2026</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>R$ 20.954.147,09</t>
+          <t>Setembro de 2026</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>tivio-email-fundos-credito.html</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>alt90</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>b2val</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>R$ 14.275.935,66</t>
+          <t>julho de 2026</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>R$ 16.917.619,85</t>
+          <t>setembro de 2026</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>tivio-email-fundos-credito.html</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>alt90</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>libs de exportação</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>114%</t>
+          <t>CDN</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>112%</t>
+          <t>4 referências → vendor/ local (CDN como reserva)</t>
         </is>
       </c>
     </row>
@@ -1549,22 +1549,22 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>alt90</t>
+          <t>alt180</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>b1val</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>112%</t>
+          <t>R$ 148.155.859,36</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>108%</t>
+          <t>R$ 153.589.286,51</t>
         </is>
       </c>
     </row>
@@ -1576,22 +1576,22 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>alt90</t>
+          <t>alt180</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>b2val</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>[{'n': 'FIDCs Cotas Sênior', 'p': 81.3}, {'n': 'Liquidez', 'p': 11.9}, {'n': 'Crédito Privado', 'p': 3.6}, {'n': 'Crédito Estruturado', 'p': 2.8}, {'n': 'FIDC Mezanino', 'p': 0.6}]</t>
+          <t>R$ 84.791.205,56</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>[{'n': 'FIDCs Cota Sênior', 'p': 76.7}, {'n': 'Liquidez', 'p': 15.7}, {'n': 'Crédito Privado', 'p': 3.5}, {'n': 'Crédito Estruturado', 'p': 2.8}, {'n': 'Fiagro', 'p': 1.5}, {'n': 'FIDCs Cota Mezanino', 'p': 0.5}]</t>
+          <t>R$ 104.590.801,56</t>
         </is>
       </c>
     </row>
@@ -1603,22 +1603,22 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>alt90</t>
+          <t>alt180</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Taxa de administração e gestão: 1,25% a.a. Taxa de performance: 10% do que exceder do CDI. Resgate: D+90.</t>
+          <t>127%</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Taxa global: 1,25% a.a. Taxa de performance: 10% do que exceder do CDI. Resgate: D+90.</t>
+          <t>123%</t>
         </is>
       </c>
     </row>
@@ -1630,22 +1630,22 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>altlight</t>
+          <t>alt180</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>b1val</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>R$ 26.861.672,93</t>
+          <t>[{'n': 'FIDCs Cotas Sênior', 'p': 49.6}, {'n': 'FIDCs Cotas Mezanino', 'p': 27.5}, {'n': 'Liquidez', 'p': 9.3}, {'n': 'Crédito Estruturado', 'p': 5.5}, {'n': 'Crédito Privado', 'p': 3.5}, {'n': 'Precatório', 'p': 2.8}, {'n': 'Fiagro', 'p': 2.0}]</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>R$ 20.571.241,16</t>
+          <t>[{'n': 'FIDCs Cota Sênior', 'p': 49.3}, {'n': 'FIDCs Cota Mezanino', 'p': 27.0}, {'n': 'Liquidez', 'p': 9.1}, {'n': 'Crédito Estruturado', 'p': 5.5}, {'n': 'Crédito Privado', 'p': 3.4}, {'n': 'Fiagro', 'p': 3.2}, {'n': 'Precatório', 'p': 2.8}]</t>
         </is>
       </c>
     </row>
@@ -1657,22 +1657,22 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>altlight</t>
+          <t>alt180</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>b2val</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>R$ 17.309.791,01</t>
+          <t>Taxa de administração e gestão: 1,15% a.a. Taxa de performance: 20% do que exceder do CDI. Resgate: D+180.</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>R$ 19.052.692,02</t>
+          <t>Taxa global: 1,15% a.a. Taxa de performance: 20% do que exceder do CDI. Resgate: D+180.</t>
         </is>
       </c>
     </row>
@@ -1684,22 +1684,22 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>altlight</t>
+          <t>alt90</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>b1val</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>116%</t>
+          <t>R$ 19.936.394,95</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>109%</t>
+          <t>R$ 20.954.147,09</t>
         </is>
       </c>
     </row>
@@ -1711,22 +1711,22 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>altlight</t>
+          <t>alt90</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>b2val</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>107%</t>
+          <t>R$ 14.275.935,66</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>101%</t>
+          <t>R$ 16.917.619,85</t>
         </is>
       </c>
     </row>
@@ -1738,22 +1738,22 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>altlight</t>
+          <t>alt90</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>101%</t>
+          <t>114%</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>112%</t>
         </is>
       </c>
     </row>
@@ -1765,22 +1765,22 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>altlight</t>
+          <t>alt90</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>[{'n': 'Bancário', 'p': 40.8}, {'n': 'Crédito Privado', 'p': 25.6}, {'n': 'FIDCs Cotas Sênior', 'p': 24.0}, {'n': 'Liquidez', 'p': 7.8}, {'n': 'FIP', 'p': 1.9}]</t>
+          <t>112%</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>[{'n': 'Bancário', 'p': 39.6}, {'n': 'FIDCs Cota Sênior', 'p': 25.9}, {'n': 'Crédito Privado', 'p': 23.8}, {'n': 'Liquidez', 'p': 8.2}, {'n': 'FIP', 'p': 2.4}]</t>
+          <t>108%</t>
         </is>
       </c>
     </row>
@@ -1792,22 +1792,22 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>altlight</t>
+          <t>alt90</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Taxa de administração e gestão: 1,15% a.a. Taxa de performance: 15% do retorno que exceder CDI+0,65%.</t>
+          <t>[{'n': 'FIDCs Cotas Sênior', 'p': 81.3}, {'n': 'Liquidez', 'p': 11.9}, {'n': 'Crédito Privado', 'p': 3.6}, {'n': 'Crédito Estruturado', 'p': 2.8}, {'n': 'FIDC Mezanino', 'p': 0.6}]</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Taxa global: 1,15% a.a. Taxa de performance: 15% do retorno que exceder CDI+0,65%.</t>
+          <t>[{'n': 'FIDCs Cota Sênior', 'p': 76.7}, {'n': 'Liquidez', 'p': 15.7}, {'n': 'Crédito Privado', 'p': 3.5}, {'n': 'Crédito Estruturado', 'p': 2.8}, {'n': 'Fiagro', 'p': 1.5}, {'n': 'FIDCs Cota Mezanino', 'p': 0.5}]</t>
         </is>
       </c>
     </row>
@@ -1819,22 +1819,22 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>alt90</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>31/07/2026</t>
+          <t>Taxa de administração e gestão: 1,25% a.a. Taxa de performance: 10% do que exceder do CDI. Resgate: D+90.</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>Taxa global: 1,25% a.a. Taxa de performance: 10% do que exceder do CDI. Resgate: D+90.</t>
         </is>
       </c>
     </row>
@@ -1846,22 +1846,22 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>altlight</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>b1val</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Julho de 2026</t>
+          <t>R$ 26.861.672,93</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Setembro de 2026</t>
+          <t>R$ 20.571.241,16</t>
         </is>
       </c>
     </row>
@@ -1873,22 +1873,22 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>altlight</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>b2val</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>julho de 2026</t>
+          <t>R$ 17.309.791,01</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>setembro de 2026</t>
+          <t>R$ 19.052.692,02</t>
         </is>
       </c>
     </row>
@@ -1900,22 +1900,22 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>altlight</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>JULHO DE 2026</t>
+          <t>116%</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>SETEMBRO DE 2026</t>
+          <t>109%</t>
         </is>
       </c>
     </row>
@@ -1927,22 +1927,22 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>altlight</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Julho 2026</t>
+          <t>107%</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Setembro 2026</t>
+          <t>101%</t>
         </is>
       </c>
     </row>
@@ -1954,22 +1954,22 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>altlight</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>-jul26</t>
+          <t>101%</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>-set26</t>
+          <t>95%</t>
         </is>
       </c>
     </row>
@@ -1981,22 +1981,22 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>altlight</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>const ATUAL=6;</t>
+          <t>[{'n': 'Bancário', 'p': 40.8}, {'n': 'Crédito Privado', 'p': 25.6}, {'n': 'FIDCs Cotas Sênior', 'p': 24.0}, {'n': 'Liquidez', 'p': 7.8}, {'n': 'FIP', 'p': 1.9}]</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>const ATUAL=8;</t>
+          <t>[{'n': 'Bancário', 'p': 39.6}, {'n': 'FIDCs Cota Sênior', 'p': 25.9}, {'n': 'Crédito Privado', 'p': 23.8}, {'n': 'Liquidez', 'p': 8.2}, {'n': 'FIP', 'p': 2.4}]</t>
         </is>
       </c>
     </row>
@@ -2008,238 +2008,238 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>altlight</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>libs de exportação</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>CDN</t>
+          <t>Taxa de administração e gestão: 1,15% a.a. Taxa de performance: 15% do retorno que exceder CDI+0,65%.</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>4 referências → vendor/ local (CDN como reserva)</t>
+          <t>Taxa global: 1,15% a.a. Taxa de performance: 15% do retorno que exceder CDI+0,65%.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>tivio-post-credito-privado.html</t>
+          <t>tivio-post-credito-estruturado.html</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>101%</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>30/09/2026</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>tivio-post-credito-privado.html</t>
+          <t>tivio-post-credito-estruturado.html</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>pl</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>R$ 1.698.520.740,05</t>
+          <t>Julho de 2026</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>R$ 1.826.931.618,96</t>
+          <t>Setembro de 2026</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>tivio-post-credito-privado.html</t>
+          <t>tivio-post-credito-estruturado.html</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>R$ 1.397.203.402,03</t>
+          <t>julho de 2026</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>R$ 1.510.000.753,13</t>
+          <t>setembro de 2026</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>tivio-post-credito-privado.html</t>
+          <t>tivio-post-credito-estruturado.html</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>{'total': '76', 'top': [{'p': '76,5%', 'n': 'financeiro'}, {'p': '23,7%', 'n': 'caixa'}]}</t>
+          <t>JULHO DE 2026</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>{'total': '75', 'top': [{'p': '75%', 'n': 'financeiro'}]}</t>
+          <t>SETEMBRO DE 2026</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>tivio-post-credito-privado.html</t>
+          <t>tivio-post-credito-estruturado.html</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>0,26</t>
+          <t>Julho 2026</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>0,25</t>
+          <t>Setembro 2026</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>tivio-post-credito-privado.html</t>
+          <t>tivio-post-credito-estruturado.html</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>1,12</t>
+          <t>-jul26</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>1,03</t>
+          <t>-set26</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>tivio-post-credito-privado.html</t>
+          <t>tivio-post-credito-estruturado.html</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Taxa de administração: 0,25% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
+          <t>const ATUAL=6;</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Taxa global: 0,25% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
+          <t>const ATUAL=8;</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>tivio-post-credito-privado.html</t>
+          <t>tivio-post-credito-estruturado.html</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>libs de exportação</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>CDN</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>99%</t>
+          <t>4 referências → vendor/ local (CDN como reserva)</t>
         </is>
       </c>
     </row>
@@ -2251,22 +2251,22 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>banks</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
+          <t>101%</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
           <t>100%</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>99%</t>
         </is>
       </c>
     </row>
@@ -2278,22 +2278,22 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>banks</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>pl</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>104%</t>
+          <t>R$ 1.698.520.740,05</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>R$ 1.826.931.618,96</t>
         </is>
       </c>
     </row>
@@ -2305,22 +2305,22 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>banks</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>pl</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>R$ 1.983.487.947,49</t>
+          <t>R$ 1.397.203.402,03</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>R$ 1.627.449.258,92</t>
+          <t>R$ 1.510.000.753,13</t>
         </is>
       </c>
     </row>
@@ -2332,22 +2332,22 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>banks</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>R$ 2.522.009.705,73</t>
+          <t>{'total': '76', 'top': [{'p': '76,5%', 'n': 'financeiro'}, {'p': '23,7%', 'n': 'caixa'}]}</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>R$ 2.427.900.811,01</t>
+          <t>{'total': '75', 'top': [{'p': '75%', 'n': 'financeiro'}]}</t>
         </is>
       </c>
     </row>
@@ -2359,22 +2359,22 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>banks</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>{'total': '69', 'top': [{'p': '52%', 'n': 'financeiro'}, {'p': '4%', 'n': 'energia elétrica'}, {'p': '2%', 'n': 'transporte e logística'}]}</t>
+          <t>0,26</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>{'total': '67', 'top': [{'p': '50%', 'n': 'financeiro'}, {'p': '5%', 'n': 'energia elétrica'}, {'p': '2%', 'n': 'FIDC'}]}</t>
+          <t>0,25</t>
         </is>
       </c>
     </row>
@@ -2386,7 +2386,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>banks</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -2396,12 +2396,12 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>0,44</t>
+          <t>1,12</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>0,43</t>
+          <t>1,03</t>
         </is>
       </c>
     </row>
@@ -2413,22 +2413,22 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>banks</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>1,20</t>
+          <t>Taxa de administração: 0,25% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>1,34</t>
+          <t>Taxa global: 0,25% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
         </is>
       </c>
     </row>
@@ -2445,17 +2445,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Taxa de administração: 0,20% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Taxa global: 0,20% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
+          <t>99%</t>
         </is>
       </c>
     </row>
@@ -2467,22 +2467,22 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>inst15</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>113%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>101%</t>
+          <t>99%</t>
         </is>
       </c>
     </row>
@@ -2494,22 +2494,22 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>inst15</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>pl</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>R$ 161.593.743,98</t>
+          <t>104%</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>R$ 156.246.478,91</t>
+          <t>95%</t>
         </is>
       </c>
     </row>
@@ -2521,22 +2521,22 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>inst15</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>pl</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>R$ 140.997.685,81</t>
+          <t>R$ 1.983.487.947,49</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>R$ 151.871.553,37</t>
+          <t>R$ 1.627.449.258,92</t>
         </is>
       </c>
     </row>
@@ -2548,22 +2548,22 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>inst15</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>{'total': '74', 'top': [{'p': '29%', 'n': 'financeiro'}, {'p': '13%', 'n': 'FIDC'}, {'p': '7%', 'n': 'energia elétrica'}]}</t>
+          <t>R$ 2.522.009.705,73</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>{'total': '70', 'top': [{'p': '28%', 'n': 'financeiro'}, {'p': '13%', 'n': 'FIDC'}, {'p': '7%', 'n': 'energia elétrica'}]}</t>
+          <t>R$ 2.427.900.811,01</t>
         </is>
       </c>
     </row>
@@ -2575,22 +2575,22 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>inst15</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>{'total': '69', 'top': [{'p': '52%', 'n': 'financeiro'}, {'p': '4%', 'n': 'energia elétrica'}, {'p': '2%', 'n': 'transporte e logística'}]}</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>0,91</t>
+          <t>{'total': '67', 'top': [{'p': '50%', 'n': 'financeiro'}, {'p': '5%', 'n': 'energia elétrica'}, {'p': '2%', 'n': 'FIDC'}]}</t>
         </is>
       </c>
     </row>
@@ -2602,7 +2602,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>inst15</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2612,12 +2612,12 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>1,97</t>
+          <t>0,44</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>1,74</t>
+          <t>0,43</t>
         </is>
       </c>
     </row>
@@ -2629,22 +2629,22 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>inst15</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>anos</t>
+          <t>1,20</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>ano</t>
+          <t>1,34</t>
         </is>
       </c>
     </row>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>inst15</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2666,12 +2666,12 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Taxa de administração: 0,45% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
+          <t>Taxa de administração: 0,20% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Taxa global: 0,50% a.a. Taxa de performance: 20% do que exceder 102,5% do CDI. Aplicação: D+0 · Resgate: D+0.</t>
+          <t>Taxa global: 0,20% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
         </is>
       </c>
     </row>
@@ -2683,22 +2683,22 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>inst30</t>
+          <t>inst15</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
+          <t>113%</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
           <t>101%</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>100%</t>
         </is>
       </c>
     </row>
@@ -2710,22 +2710,22 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>inst30</t>
+          <t>inst15</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>pl</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>113%</t>
+          <t>R$ 161.593.743,98</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>102%</t>
+          <t>R$ 156.246.478,91</t>
         </is>
       </c>
     </row>
@@ -2737,22 +2737,22 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>inst30</t>
+          <t>inst15</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>pl</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>R$ 143.232.764,20</t>
+          <t>R$ 140.997.685,81</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>R$ 138.199.759,13</t>
+          <t>R$ 151.871.553,37</t>
         </is>
       </c>
     </row>
@@ -2764,22 +2764,22 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>inst30</t>
+          <t>inst15</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>R$ 155.004.649,74</t>
+          <t>{'total': '74', 'top': [{'p': '29%', 'n': 'financeiro'}, {'p': '13%', 'n': 'FIDC'}, {'p': '7%', 'n': 'energia elétrica'}]}</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>R$ 162.868.029,59</t>
+          <t>{'total': '70', 'top': [{'p': '28%', 'n': 'financeiro'}, {'p': '13%', 'n': 'FIDC'}, {'p': '7%', 'n': 'energia elétrica'}]}</t>
         </is>
       </c>
     </row>
@@ -2791,22 +2791,22 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>inst30</t>
+          <t>inst15</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>{'total': '84', 'top': [{'p': '33%', 'n': 'financeiro'}, {'p': '15%', 'n': 'FIDC'}, {'p': '8%', 'n': 'energia elétrica'}]}</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>{'total': '79', 'top': [{'p': '31%', 'n': 'financeiro'}, {'p': '15%', 'n': 'FIDC'}, {'p': '8%', 'n': 'energia elétrica'}]}</t>
+          <t>0,91</t>
         </is>
       </c>
     </row>
@@ -2818,7 +2818,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>inst30</t>
+          <t>inst15</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2828,12 +2828,12 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1,97</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>1,02</t>
+          <t>1,74</t>
         </is>
       </c>
     </row>
@@ -2845,22 +2845,22 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>inst30</t>
+          <t>inst15</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>anos</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>1,79</t>
+          <t>ano</t>
         </is>
       </c>
     </row>
@@ -2872,22 +2872,22 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>inst30</t>
+          <t>inst15</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>anos</t>
+          <t>Taxa de administração: 0,45% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>ano</t>
+          <t>Taxa global: 0,50% a.a. Taxa de performance: 20% do que exceder 102,5% do CDI. Aplicação: D+0 · Resgate: D+0.</t>
         </is>
       </c>
     </row>
@@ -2904,17 +2904,17 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Taxa de administração: 0,63% a.a. Taxa de performance: 20% do que exceder o CDI. Resgate: D+30.</t>
+          <t>101%</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Taxa global: 0,625% a.a. Taxa de performance: 20% do que exceder 100% do CDI. Resgate: D+30.</t>
+          <t>100%</t>
         </is>
       </c>
     </row>
@@ -2926,22 +2926,22 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>infraplus</t>
+          <t>inst30</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>12,94%</t>
+          <t>113%</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>9,10%</t>
+          <t>102%</t>
         </is>
       </c>
     </row>
@@ -2953,22 +2953,22 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>infraplus</t>
+          <t>inst30</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>a1</t>
+          <t>pl</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>*Alfa: -2,75%</t>
+          <t>R$ 143.232.764,20</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>*Alfa: −5,70%</t>
+          <t>R$ 138.199.759,13</t>
         </is>
       </c>
     </row>
@@ -2980,22 +2980,22 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>infraplus</t>
+          <t>inst30</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>7,80%</t>
+          <t>R$ 155.004.649,74</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>7,05%</t>
+          <t>R$ 162.868.029,59</t>
         </is>
       </c>
     </row>
@@ -3007,22 +3007,22 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>infraplus</t>
+          <t>inst30</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>a2</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>*Alfa: -3,14%</t>
+          <t>{'total': '84', 'top': [{'p': '33%', 'n': 'financeiro'}, {'p': '15%', 'n': 'FIDC'}, {'p': '8%', 'n': 'energia elétrica'}]}</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>*Alfa: −4,32%</t>
+          <t>{'total': '79', 'top': [{'p': '31%', 'n': 'financeiro'}, {'p': '15%', 'n': 'FIDC'}, {'p': '8%', 'n': 'energia elétrica'}]}</t>
         </is>
       </c>
     </row>
@@ -3034,22 +3034,22 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>infraplus</t>
+          <t>inst30</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>1,24%</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>1,01%</t>
+          <t>1,02</t>
         </is>
       </c>
     </row>
@@ -3061,22 +3061,22 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>infraplus</t>
+          <t>inst30</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>a3</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>*Alfa: -0,14%</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>*Alfa: −1,00%</t>
+          <t>1,79</t>
         </is>
       </c>
     </row>
@@ -3088,22 +3088,22 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>infraplus</t>
+          <t>inst30</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>pl</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>R$ 42.983.282,75</t>
+          <t>anos</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>R$ 37.299.076,05</t>
+          <t>ano</t>
         </is>
       </c>
     </row>
@@ -3115,22 +3115,22 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>infraplus</t>
+          <t>inst30</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>R$ 52.049.593,91</t>
+          <t>Taxa de administração: 0,63% a.a. Taxa de performance: 20% do que exceder o CDI. Resgate: D+30.</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>R$ 46.597.018,20</t>
+          <t>Taxa global: 0,625% a.a. Taxa de performance: 20% do que exceder 100% do CDI. Resgate: D+30.</t>
         </is>
       </c>
     </row>
@@ -3147,17 +3147,17 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>{'total': '95', 'top': [{'p': '55%', 'n': 'energia elétrica'}, {'p': '15%', 'n': 'transporte e logística'}, {'p': '7%', 'n': 'saneamento'}]}</t>
+          <t>12,94%</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>{'total': '97', 'top': [{'p': '53%', 'n': 'energia elétrica'}, {'p': '14%', 'n': 'transporte e logística'}, {'p': '8%', 'n': 'saneamento'}]}</t>
+          <t>9,10%</t>
         </is>
       </c>
     </row>
@@ -3174,17 +3174,17 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>a1</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>8,63</t>
+          <t>*Alfa: -2,75%</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>8,11</t>
+          <t>*Alfa: −5,70%</t>
         </is>
       </c>
     </row>
@@ -3201,17 +3201,17 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>4,00</t>
+          <t>7,80%</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>3,99</t>
+          <t>7,05%</t>
         </is>
       </c>
     </row>
@@ -3228,17 +3228,17 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>a2</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Taxa de administração: 0,75% a.a. Taxa de performance: não há. Resgate: D+31. Rentabilidade isenta de IR para pessoa física.</t>
+          <t>*Alfa: -3,14%</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Taxa global: 0,75% a.a. Taxa de performance: não há. Resgate: D+31. Rentabilidade isenta de IR para pessoa física.</t>
+          <t>*Alfa: −4,32%</t>
         </is>
       </c>
     </row>
@@ -3250,22 +3250,22 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>infraplus</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>k1</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>12M</t>
+          <t>1,24%</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Desde o início</t>
+          <t>1,01%</t>
         </is>
       </c>
     </row>
@@ -3277,22 +3277,22 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>infraplus</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>a3</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>*Alfa: -0,14%</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>88%</t>
+          <t>*Alfa: −1,00%</t>
         </is>
       </c>
     </row>
@@ -3304,22 +3304,22 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>infraplus</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>pl</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>R$ 42.983.282,75</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>82%</t>
+          <t>R$ 37.299.076,05</t>
         </is>
       </c>
     </row>
@@ -3331,22 +3331,22 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>infraplus</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>R$ 52.049.593,91</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>−14%</t>
+          <t>R$ 46.597.018,20</t>
         </is>
       </c>
     </row>
@@ -3358,22 +3358,22 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>infraplus</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>pl</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>{'total': '95', 'top': [{'p': '55%', 'n': 'energia elétrica'}, {'p': '15%', 'n': 'transporte e logística'}, {'p': '7%', 'n': 'saneamento'}]}</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>R$ 44.023.801,59</t>
+          <t>{'total': '97', 'top': [{'p': '53%', 'n': 'energia elétrica'}, {'p': '14%', 'n': 'transporte e logística'}, {'p': '8%', 'n': 'saneamento'}]}</t>
         </is>
       </c>
     </row>
@@ -3385,22 +3385,22 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>infraplus</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>8,63</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>R$ 37.965.174,74</t>
+          <t>8,11</t>
         </is>
       </c>
     </row>
@@ -3412,22 +3412,22 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>infraplus</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>{'total': '0', 'top': []}</t>
+          <t>4,00</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>{'total': '93', 'top': [{'p': '38%', 'n': 'energia elétrica'}, {'p': '22%', 'n': 'FIDC'}, {'p': '11%', 'n': 'transporte e logística'}]}</t>
+          <t>3,99</t>
         </is>
       </c>
     </row>
@@ -3439,22 +3439,22 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>infraplus</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Taxa de administração: 0,75% a.a. Taxa de performance: não há. Resgate: D+31. Rentabilidade isenta de IR para pessoa física.</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>1,08</t>
+          <t>Taxa global: 0,75% a.a. Taxa de performance: não há. Resgate: D+31. Rentabilidade isenta de IR para pessoa física.</t>
         </is>
       </c>
     </row>
@@ -3471,17 +3471,17 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>k1</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12M</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>3,70</t>
+          <t>Desde o início</t>
         </is>
       </c>
     </row>
@@ -3498,17 +3498,17 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Taxa de administração: 0,75% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+30. Rentabilidade isenta de IR para pessoa física.</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Taxa global: 0,75% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+30. Rentabilidade isenta de IR para pessoa física.</t>
+          <t>88%</t>
         </is>
       </c>
     </row>
@@ -3520,22 +3520,22 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>31/07/2026</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>82%</t>
         </is>
       </c>
     </row>
@@ -3547,22 +3547,22 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Julho de 2026</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Setembro de 2026</t>
+          <t>−14%</t>
         </is>
       </c>
     </row>
@@ -3574,22 +3574,22 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>pl</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>julho de 2026</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>setembro de 2026</t>
+          <t>R$ 44.023.801,59</t>
         </is>
       </c>
     </row>
@@ -3601,22 +3601,22 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>JULHO DE 2026</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>SETEMBRO DE 2026</t>
+          <t>R$ 37.965.174,74</t>
         </is>
       </c>
     </row>
@@ -3628,22 +3628,22 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Julho 2026</t>
+          <t>{'total': '0', 'top': []}</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Setembro 2026</t>
+          <t>{'total': '93', 'top': [{'p': '38%', 'n': 'energia elétrica'}, {'p': '22%', 'n': 'FIDC'}, {'p': '11%', 'n': 'transporte e logística'}]}</t>
         </is>
       </c>
     </row>
@@ -3655,22 +3655,22 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>-jul26</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>-set26</t>
+          <t>1,08</t>
         </is>
       </c>
     </row>
@@ -3682,22 +3682,22 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>const ATUAL=6;</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>const ATUAL=8;</t>
+          <t>3,70</t>
         </is>
       </c>
     </row>
@@ -3709,238 +3709,238 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>libs de exportação</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>CDN</t>
+          <t>Taxa de administração: 0,75% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+30. Rentabilidade isenta de IR para pessoa física.</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>4 referências → vendor/ local (CDN como reserva)</t>
+          <t>Taxa global: 0,75% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+30. Rentabilidade isenta de IR para pessoa física.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>tivio-post-credito-privado.html</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>103%</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>48%</t>
+          <t>30/09/2026</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>tivio-post-credito-privado.html</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>101%</t>
+          <t>Julho de 2026</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>Setembro de 2026</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>tivio-post-credito-privado.html</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>101%</t>
+          <t>julho de 2026</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>setembro de 2026</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>tivio-post-credito-privado.html</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>R$ 352,4 mi</t>
+          <t>JULHO DE 2026</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>R$ 339,3 mi</t>
+          <t>SETEMBRO DE 2026</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>tivio-post-credito-privado.html</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>104%</t>
+          <t>Julho 2026</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>Setembro 2026</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>tivio-post-credito-privado.html</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>106%</t>
+          <t>-jul26</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>104%</t>
+          <t>-set26</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>tivio-post-credito-privado.html</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>109%</t>
+          <t>const ATUAL=6;</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>106%</t>
+          <t>const ATUAL=8;</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>tivio-post-credito-privado.html</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>libs de exportação</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>R$ 33,2 mi</t>
+          <t>CDN</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>R$ 38,8 mi</t>
+          <t>4 referências → vendor/ local (CDN como reserva)</t>
         </is>
       </c>
     </row>
@@ -3952,22 +3952,22 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>adm</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>0,00% a.a. (vértice tx zero)</t>
+          <t>103%</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>0,15% a.a.</t>
+          <t>48%</t>
         </is>
       </c>
     </row>
@@ -3979,22 +3979,22 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
+          <t>101%</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
           <t>93%</t>
-        </is>
-      </c>
-      <c r="E132" t="inlineStr">
-        <is>
-          <t>91%</t>
         </is>
       </c>
     </row>
@@ -4006,22 +4006,22 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>86%</t>
+          <t>101%</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>87%</t>
+          <t>95%</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -4043,12 +4043,12 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>R$ 374,3 mi</t>
+          <t>R$ 352,4 mi</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>R$ 329,9 mi</t>
+          <t>R$ 339,3 mi</t>
         </is>
       </c>
     </row>
@@ -4060,7 +4060,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -4070,12 +4070,12 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>2,13%</t>
+          <t>104%</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>95%</t>
         </is>
       </c>
     </row>
@@ -4087,22 +4087,22 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>a1</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>*Alfa: −3,03%</t>
+          <t>106%</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>*Alfa: 1,41%</t>
+          <t>104%</t>
         </is>
       </c>
     </row>
@@ -4114,22 +4114,22 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>−5,35%</t>
+          <t>109%</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>106%</t>
         </is>
       </c>
     </row>
@@ -4141,22 +4141,22 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>a2</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>*Alfa: −1,59%</t>
+          <t>R$ 33,2 mi</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>*Alfa: 1,13%</t>
+          <t>R$ 38,8 mi</t>
         </is>
       </c>
     </row>
@@ -4168,22 +4168,22 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>adm</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>7,66%</t>
+          <t>0,00% a.a. (vértice tx zero)</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>13%</t>
+          <t>0,15% a.a.</t>
         </is>
       </c>
     </row>
@@ -4195,22 +4195,22 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>a3</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>*Alfa: −6,22%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>*Alfa: 0,50%</t>
+          <t>91%</t>
         </is>
       </c>
     </row>
@@ -4222,22 +4222,22 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>R$ 100,8 mi</t>
+          <t>86%</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>R$ 70,7 mi</t>
+          <t>87%</t>
         </is>
       </c>
     </row>
@@ -4249,22 +4249,22 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>perf</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>20% do que exceder o CDI</t>
+          <t>R$ 374,3 mi</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>20% do que exceder 100% do CDI</t>
+          <t>R$ 329,9 mi</t>
         </is>
       </c>
     </row>
@@ -4276,7 +4276,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -4286,12 +4286,12 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>73%</t>
+          <t>2,13%</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>144%</t>
+          <t>0%</t>
         </is>
       </c>
     </row>
@@ -4303,22 +4303,22 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>a1</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>74%</t>
+          <t>*Alfa: −3,03%</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>83%</t>
+          <t>*Alfa: 1,41%</t>
         </is>
       </c>
     </row>
@@ -4330,22 +4330,22 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>81%</t>
+          <t>−5,35%</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>87%</t>
+          <t>6%</t>
         </is>
       </c>
     </row>
@@ -4357,22 +4357,22 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>a2</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>R$ 102,7 mi</t>
+          <t>*Alfa: −1,59%</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>R$ 95,5 mi</t>
+          <t>*Alfa: 1,13%</t>
         </is>
       </c>
     </row>
@@ -4384,22 +4384,22 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>7,66%</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>141%</t>
+          <t>13%</t>
         </is>
       </c>
     </row>
@@ -4411,22 +4411,22 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>a3</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>*Alfa: −6,22%</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>*Alfa: 0,50%</t>
         </is>
       </c>
     </row>
@@ -4438,22 +4438,22 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>R$ 100,8 mi</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>R$ 70,7 mi</t>
         </is>
       </c>
     </row>
@@ -4465,22 +4465,22 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>perf</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>R$ 662,8 mi</t>
+          <t>20% do que exceder o CDI</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>R$ 637,1 mi</t>
+          <t>20% do que exceder 100% do CDI</t>
         </is>
       </c>
     </row>
@@ -4492,22 +4492,22 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>31/07/2026</t>
+          <t>73%</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>144%</t>
         </is>
       </c>
     </row>
@@ -4519,22 +4519,22 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Julho de 2026</t>
+          <t>74%</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Setembro de 2026</t>
+          <t>83%</t>
         </is>
       </c>
     </row>
@@ -4546,22 +4546,22 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>julho de 2026</t>
+          <t>81%</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>setembro de 2026</t>
+          <t>87%</t>
         </is>
       </c>
     </row>
@@ -4573,22 +4573,22 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>JULHO DE 2026</t>
+          <t>R$ 102,7 mi</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>SETEMBRO DE 2026</t>
+          <t>R$ 95,5 mi</t>
         </is>
       </c>
     </row>
@@ -4600,22 +4600,22 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Julho 2026</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Setembro 2026</t>
+          <t>141%</t>
         </is>
       </c>
     </row>
@@ -4627,22 +4627,22 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>-jul26</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>-set26</t>
+          <t>98%</t>
         </is>
       </c>
     </row>
@@ -4654,22 +4654,22 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>const ATUAL=6;</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>const ATUAL=8;</t>
+          <t>97%</t>
         </is>
       </c>
     </row>
@@ -4681,191 +4681,191 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>libs de exportação</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>CDN</t>
+          <t>R$ 662,8 mi</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>4 referências → vendor/ local (CDN como reserva)</t>
+          <t>R$ 637,1 mi</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>tivio-central.html</t>
+          <t>tivio-post-investment-solutions.html</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>s1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Julho 2026</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Setembro 2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>tivio-central.html</t>
+          <t>tivio-post-investment-solutions.html</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>s2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Julho 2026</t>
+          <t>Julho de 2026</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Setembro 2026</t>
+          <t>Setembro de 2026</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>tivio-central.html</t>
+          <t>tivio-post-investment-solutions.html</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>s8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Julho 2026</t>
+          <t>julho de 2026</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Setembro 2026</t>
+          <t>setembro de 2026</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>tivio-central.html</t>
+          <t>tivio-post-investment-solutions.html</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>e1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Julho 2026</t>
+          <t>JULHO DE 2026</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Setembro 2026</t>
+          <t>SETEMBRO DE 2026</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>tivio-central.html</t>
+          <t>tivio-post-investment-solutions.html</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Relatório de Gestão · Incentivado CDI 30</t>
+          <t>Julho 2026</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Gerador de Relatório de Gestão · Incentivado CDI 30</t>
+          <t>Setembro 2026</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>tivio-central.html</t>
+          <t>tivio-post-investment-solutions.html</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>desc</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Relatório de gestão mensal do Tivio Institucional Inc CDI 30 FIF (debêntures incentivadas · CDI).</t>
+          <t>-jul26</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Construtor interativo, folha a folha. Os relatórios prontos do mês estão no card acima. Relatório de gestão mensal do Tivio Institucional Inc CDI 30 FIF (debêntures incentivadas · CDI).</t>
+          <t>-set26</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>tivio-central.html</t>
+          <t>tivio-post-investment-solutions.html</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -4875,38 +4875,254 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>cards de relatório</t>
+          <t>const ATUAL=6;</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>2 registrados para Setembro 2026</t>
+          <t>const ATUAL=8;</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
+          <t>tivio-post-investment-solutions.html</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>libs de exportação</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>CDN</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>4 referências → vendor/ local (CDN como reserva)</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
           <t>tivio-central.html</t>
         </is>
       </c>
-      <c r="B166" t="inlineStr">
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>s1</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Julho 2026</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Setembro 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>tivio-central.html</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>s2</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Julho 2026</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Setembro 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>tivio-central.html</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>s8</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Julho 2026</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Setembro 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>tivio-central.html</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>e1</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Julho 2026</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Setembro 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>tivio-central.html</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>r2</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Relatório de Gestão · Incentivado CDI 30</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Gerador de Relatório de Gestão · Incentivado CDI 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>tivio-central.html</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>r2</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>desc</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Relatório de gestão mensal do Tivio Institucional Inc CDI 30 FIF (debêntures incentivadas · CDI).</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Construtor interativo, folha a folha. Os relatórios prontos do mês estão no card acima. Relatório de gestão mensal do Tivio Institucional Inc CDI 30 FIF (debêntures incentivadas · CDI).</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>tivio-central.html</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C166" t="inlineStr">
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>cards de relatório</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>2 registrados para Setembro 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>tivio-central.html</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
         <is>
           <t>data automática</t>
         </is>
       </c>
-      <c r="D166" t="inlineStr"/>
-      <c r="E166" t="inlineStr">
+      <c r="D174" t="inlineStr"/>
+      <c r="E174" t="inlineStr">
         <is>
           <t>DATA_BASE=2026-09-30</t>
         </is>
@@ -11572,7 +11788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -11668,102 +11884,204 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>tivio-email-fundos-credito.html</t>
+          <t>landing/hgd30</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>alt180</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>o texto se refere a "julho" como o mês corrente — a data base é setembro</t>
+          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): Na atribuição de performance, a carteira de títulos bancários foi a principal re…</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>landing/hyd60</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>alt180</t>
+          <t>hyd60</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Mz', 'Fiagro Sr']</t>
+          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): - Na parcela de **crédito estruturado**, avanço na **diversificação da carteira*…</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>email/previdencia</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>alt90</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Sr']</t>
+          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): Na atribuição de performance, a carteira de títulos bancários foi a principal re…</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>email/previdencia</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>topgestormacro</t>
+          <t>hyd60</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>sem dados — rentabilidade e PL mantidos</t>
+          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): - Na parcela de **crédito estruturado**, avanço na **diversificação da carteira*…</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>tivio-email-fundos-credito.html</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>topgestorlongonly</t>
+          <t>alt180</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>sem dados — rentabilidade e PL mantidos</t>
+          <t>o texto se refere a "julho" como o mês corrente — a data base é setembro</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>tivio-post-credito-estruturado.html</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>alt180</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Mz', 'Fiagro Sr']</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>tivio-post-credito-estruturado.html</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>alt90</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Sr']</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>tivio-post-investment-solutions.html</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>topgestormacro</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>sem dados — rentabilidade e PL mantidos</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>tivio-post-investment-solutions.html</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>topgestorlongonly</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>sem dados — rentabilidade e PL mantidos</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>tivio-central.html</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>tivio-central.html</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>card "Gerador de Relatório de Gestão · Incentivado CDI 30" removido: aponta para "Tivio Incentivado CDI 30 - Relatório de Gestão Mensal.html", que não existe nesta edição</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>tivio-central.html</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>hgd30</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Informativo em PDF não gerado: precisa do PowerPoint instalado (o PPTX saiu; dá para salvar como PDF por ele)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>tivio-central.html</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>hyd60</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Informativo em PDF não gerado: precisa do PowerPoint instalado (o PPTX saiu; dá para salvar como PDF por ele)</t>
         </is>
       </c>
     </row>
@@ -11778,7 +12096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -12235,7 +12553,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>540082</v>
+        <v>540379</v>
       </c>
     </row>
     <row r="31">
@@ -12250,7 +12568,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>547647</v>
+        <v>547655</v>
       </c>
     </row>
     <row r="32">
@@ -12265,7 +12583,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2092660</v>
+        <v>2093582</v>
       </c>
     </row>
     <row r="33">
@@ -12295,7 +12613,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>177281</v>
+        <v>202964</v>
       </c>
     </row>
     <row r="35">
@@ -12445,66 +12763,36 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4829264</v>
+        <v>4829400</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Informativo - HGD30 - Setembro 2026.pdf</t>
+          <t>Informativo - HYD60 - Setembro 2026.pptx</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>pptx</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>423404</v>
+        <v>5454374</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Informativo - HYD60 - Setembro 2026.pptx</t>
+          <t>index.html</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>pptx</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>5454369</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Informativo - HYD60 - Setembro 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>554208</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>index.html</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C48" t="n">
         <v>394</v>
       </c>
     </row>

</xml_diff>

<commit_message>
AutomaTivio: Informativo apaga o PDF antigo antes de exportar e tenta de novo se o PowerPoint falhar
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -11788,7 +11788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -12048,40 +12048,6 @@
       <c r="C15" t="inlineStr">
         <is>
           <t>card "Gerador de Relatório de Gestão · Incentivado CDI 30" removido: aponta para "Tivio Incentivado CDI 30 - Relatório de Gestão Mensal.html", que não existe nesta edição</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>hgd30</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Informativo em PDF não gerado: precisa do PowerPoint instalado (o PPTX saiu; dá para salvar como PDF por ele)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>hyd60</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Informativo em PDF não gerado: precisa do PowerPoint instalado (o PPTX saiu; dá para salvar como PDF por ele)</t>
         </is>
       </c>
     </row>
@@ -12096,7 +12062,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -12763,36 +12729,66 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4829400</v>
+        <v>4829398</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Informativo - HYD60 - Setembro 2026.pptx</t>
+          <t>Informativo - HGD30 - Setembro 2026.pdf</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>pptx</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>5454374</v>
+        <v>422853</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>Informativo - HYD60 - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>5454374</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Informativo - HYD60 - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>554367</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>index.html</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>html</t>
         </is>
       </c>
-      <c r="C46" t="n">
+      <c r="C48" t="n">
         <v>394</v>
       </c>
     </row>

</xml_diff>

<commit_message>
AutomaTivio: cartão da Ágora na estrutura dos Destaques (% do CDI; Infra Plus com retorno, Alfa e nota do IMA-B 5)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -12579,7 +12579,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>202964</v>
+        <v>203856</v>
       </c>
     </row>
     <row r="35">
@@ -12759,7 +12759,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>5454374</v>
+        <v>5454371</v>
       </c>
     </row>
     <row r="47">

</xml_diff>

<commit_message>
AutomaTivio: datas de início oficiais (Infra Plus, ALT 90, Inst 15) em todos os materiais; áudio do HGD30; cartões do HYD60 da versão do Renan; ECharts pelo CDN no site
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E174"/>
+  <dimension ref="A1:E176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1846,22 +1846,22 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>altlight</t>
+          <t>alt90</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>b1val</t>
+          <t>inicio</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>R$ 26.861.672,93</t>
+          <t>27/05/2025</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>R$ 20.571.241,16</t>
+          <t>06/06/2025</t>
         </is>
       </c>
     </row>
@@ -1878,17 +1878,17 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>b2val</t>
+          <t>b1val</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>R$ 17.309.791,01</t>
+          <t>R$ 26.861.672,93</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>R$ 19.052.692,02</t>
+          <t>R$ 20.571.241,16</t>
         </is>
       </c>
     </row>
@@ -1905,17 +1905,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>b2val</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>116%</t>
+          <t>R$ 17.309.791,01</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>109%</t>
+          <t>R$ 19.052.692,02</t>
         </is>
       </c>
     </row>
@@ -1932,17 +1932,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>107%</t>
+          <t>116%</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>101%</t>
+          <t>109%</t>
         </is>
       </c>
     </row>
@@ -1959,17 +1959,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
+          <t>107%</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
           <t>101%</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>95%</t>
         </is>
       </c>
     </row>
@@ -1986,17 +1986,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>[{'n': 'Bancário', 'p': 40.8}, {'n': 'Crédito Privado', 'p': 25.6}, {'n': 'FIDCs Cotas Sênior', 'p': 24.0}, {'n': 'Liquidez', 'p': 7.8}, {'n': 'FIP', 'p': 1.9}]</t>
+          <t>101%</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>[{'n': 'Bancário', 'p': 39.6}, {'n': 'FIDCs Cota Sênior', 'p': 25.9}, {'n': 'Crédito Privado', 'p': 23.8}, {'n': 'Liquidez', 'p': 8.2}, {'n': 'FIP', 'p': 2.4}]</t>
+          <t>95%</t>
         </is>
       </c>
     </row>
@@ -2013,17 +2013,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Taxa de administração e gestão: 1,15% a.a. Taxa de performance: 15% do retorno que exceder CDI+0,65%.</t>
+          <t>[{'n': 'Bancário', 'p': 40.8}, {'n': 'Crédito Privado', 'p': 25.6}, {'n': 'FIDCs Cotas Sênior', 'p': 24.0}, {'n': 'Liquidez', 'p': 7.8}, {'n': 'FIP', 'p': 1.9}]</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Taxa global: 1,15% a.a. Taxa de performance: 15% do retorno que exceder CDI+0,65%.</t>
+          <t>[{'n': 'Bancário', 'p': 39.6}, {'n': 'FIDCs Cota Sênior', 'p': 25.9}, {'n': 'Crédito Privado', 'p': 23.8}, {'n': 'Liquidez', 'p': 8.2}, {'n': 'FIP', 'p': 2.4}]</t>
         </is>
       </c>
     </row>
@@ -2035,22 +2035,22 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>altlight</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>31/07/2026</t>
+          <t>Taxa de administração e gestão: 1,15% a.a. Taxa de performance: 15% do retorno que exceder CDI+0,65%.</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>Taxa global: 1,15% a.a. Taxa de performance: 15% do retorno que exceder CDI+0,65%.</t>
         </is>
       </c>
     </row>
@@ -2072,12 +2072,12 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Julho de 2026</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Setembro de 2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
     </row>
@@ -2099,12 +2099,12 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>julho de 2026</t>
+          <t>Julho de 2026</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>setembro de 2026</t>
+          <t>Setembro de 2026</t>
         </is>
       </c>
     </row>
@@ -2126,12 +2126,12 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>JULHO DE 2026</t>
+          <t>julho de 2026</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>SETEMBRO DE 2026</t>
+          <t>setembro de 2026</t>
         </is>
       </c>
     </row>
@@ -2153,12 +2153,12 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Julho 2026</t>
+          <t>JULHO DE 2026</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Setembro 2026</t>
+          <t>SETEMBRO DE 2026</t>
         </is>
       </c>
     </row>
@@ -2180,12 +2180,12 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>-jul26</t>
+          <t>Julho 2026</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>-set26</t>
+          <t>Setembro 2026</t>
         </is>
       </c>
     </row>
@@ -2207,12 +2207,12 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>const ATUAL=6;</t>
+          <t>-jul26</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>const ATUAL=8;</t>
+          <t>-set26</t>
         </is>
       </c>
     </row>
@@ -2229,44 +2229,44 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>libs de exportação</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>CDN</t>
+          <t>const ATUAL=6;</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>4 referências → vendor/ local (CDN como reserva)</t>
+          <t>const ATUAL=8;</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>tivio-post-credito-privado.html</t>
+          <t>tivio-post-credito-estruturado.html</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>libs de exportação</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>101%</t>
+          <t>CDN</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>4 referências → vendor/ local (CDN como reserva)</t>
         </is>
       </c>
     </row>
@@ -2283,17 +2283,17 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>pl</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>R$ 1.698.520.740,05</t>
+          <t>101%</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>R$ 1.826.931.618,96</t>
+          <t>100%</t>
         </is>
       </c>
     </row>
@@ -2310,17 +2310,17 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>pl</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>R$ 1.397.203.402,03</t>
+          <t>R$ 1.698.520.740,05</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>R$ 1.510.000.753,13</t>
+          <t>R$ 1.826.931.618,96</t>
         </is>
       </c>
     </row>
@@ -2337,17 +2337,17 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>{'total': '76', 'top': [{'p': '76,5%', 'n': 'financeiro'}, {'p': '23,7%', 'n': 'caixa'}]}</t>
+          <t>R$ 1.397.203.402,03</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>{'total': '75', 'top': [{'p': '75%', 'n': 'financeiro'}]}</t>
+          <t>R$ 1.510.000.753,13</t>
         </is>
       </c>
     </row>
@@ -2364,17 +2364,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>0,26</t>
+          <t>{'total': '76', 'top': [{'p': '76,5%', 'n': 'financeiro'}, {'p': '23,7%', 'n': 'caixa'}]}</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>0,25</t>
+          <t>{'total': '75', 'top': [{'p': '75%', 'n': 'financeiro'}]}</t>
         </is>
       </c>
     </row>
@@ -2396,12 +2396,12 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>1,12</t>
+          <t>0,26</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>1,03</t>
+          <t>0,25</t>
         </is>
       </c>
     </row>
@@ -2418,17 +2418,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Taxa de administração: 0,25% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
+          <t>1,12</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Taxa global: 0,25% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
+          <t>1,03</t>
         </is>
       </c>
     </row>
@@ -2440,22 +2440,22 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>banks</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>Taxa de administração: 0,25% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>99%</t>
+          <t>Taxa global: 0,25% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
         </is>
       </c>
     </row>
@@ -2472,7 +2472,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2499,17 +2499,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>104%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>99%</t>
         </is>
       </c>
     </row>
@@ -2526,17 +2526,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>pl</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>R$ 1.983.487.947,49</t>
+          <t>104%</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>R$ 1.627.449.258,92</t>
+          <t>95%</t>
         </is>
       </c>
     </row>
@@ -2553,17 +2553,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>pl</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>R$ 2.522.009.705,73</t>
+          <t>R$ 1.983.487.947,49</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>R$ 2.427.900.811,01</t>
+          <t>R$ 1.627.449.258,92</t>
         </is>
       </c>
     </row>
@@ -2580,17 +2580,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>{'total': '69', 'top': [{'p': '52%', 'n': 'financeiro'}, {'p': '4%', 'n': 'energia elétrica'}, {'p': '2%', 'n': 'transporte e logística'}]}</t>
+          <t>R$ 2.522.009.705,73</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>{'total': '67', 'top': [{'p': '50%', 'n': 'financeiro'}, {'p': '5%', 'n': 'energia elétrica'}, {'p': '2%', 'n': 'FIDC'}]}</t>
+          <t>R$ 2.427.900.811,01</t>
         </is>
       </c>
     </row>
@@ -2607,17 +2607,17 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0,44</t>
+          <t>{'total': '69', 'top': [{'p': '52%', 'n': 'financeiro'}, {'p': '4%', 'n': 'energia elétrica'}, {'p': '2%', 'n': 'transporte e logística'}]}</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>0,43</t>
+          <t>{'total': '67', 'top': [{'p': '50%', 'n': 'financeiro'}, {'p': '5%', 'n': 'energia elétrica'}, {'p': '2%', 'n': 'FIDC'}]}</t>
         </is>
       </c>
     </row>
@@ -2639,12 +2639,12 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>1,20</t>
+          <t>0,44</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>1,34</t>
+          <t>0,43</t>
         </is>
       </c>
     </row>
@@ -2661,17 +2661,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Taxa de administração: 0,20% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
+          <t>1,20</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Taxa global: 0,20% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
+          <t>1,34</t>
         </is>
       </c>
     </row>
@@ -2683,22 +2683,22 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>inst15</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>113%</t>
+          <t>Taxa de administração: 0,20% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>101%</t>
+          <t>Taxa global: 0,20% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
         </is>
       </c>
     </row>
@@ -2715,17 +2715,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>pl</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>R$ 161.593.743,98</t>
+          <t>113%</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>R$ 156.246.478,91</t>
+          <t>101%</t>
         </is>
       </c>
     </row>
@@ -2742,17 +2742,17 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>pl</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>R$ 140.997.685,81</t>
+          <t>R$ 161.593.743,98</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>R$ 151.871.553,37</t>
+          <t>R$ 156.246.478,91</t>
         </is>
       </c>
     </row>
@@ -2769,17 +2769,17 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>{'total': '74', 'top': [{'p': '29%', 'n': 'financeiro'}, {'p': '13%', 'n': 'FIDC'}, {'p': '7%', 'n': 'energia elétrica'}]}</t>
+          <t>R$ 140.997.685,81</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>{'total': '70', 'top': [{'p': '28%', 'n': 'financeiro'}, {'p': '13%', 'n': 'FIDC'}, {'p': '7%', 'n': 'energia elétrica'}]}</t>
+          <t>R$ 151.871.553,37</t>
         </is>
       </c>
     </row>
@@ -2796,17 +2796,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>{'total': '74', 'top': [{'p': '29%', 'n': 'financeiro'}, {'p': '13%', 'n': 'FIDC'}, {'p': '7%', 'n': 'energia elétrica'}]}</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>0,91</t>
+          <t>{'total': '70', 'top': [{'p': '28%', 'n': 'financeiro'}, {'p': '13%', 'n': 'FIDC'}, {'p': '7%', 'n': 'energia elétrica'}]}</t>
         </is>
       </c>
     </row>
@@ -2828,12 +2828,12 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>1,97</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>1,74</t>
+          <t>0,91</t>
         </is>
       </c>
     </row>
@@ -2850,17 +2850,17 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>anos</t>
+          <t>1,97</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>ano</t>
+          <t>1,74</t>
         </is>
       </c>
     </row>
@@ -2877,17 +2877,17 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Taxa de administração: 0,45% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
+          <t>anos</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Taxa global: 0,50% a.a. Taxa de performance: 20% do que exceder 102,5% do CDI. Aplicação: D+0 · Resgate: D+0.</t>
+          <t>ano</t>
         </is>
       </c>
     </row>
@@ -2899,22 +2899,22 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>inst30</t>
+          <t>inst15</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>101%</t>
+          <t>Taxa de administração: 0,45% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+0.</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>Taxa global: 0,50% a.a. Taxa de performance: 20% do que exceder 102,5% do CDI. Aplicação: D+0 · Resgate: D+0.</t>
         </is>
       </c>
     </row>
@@ -2931,17 +2931,17 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>113%</t>
+          <t>101%</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>102%</t>
+          <t>100%</t>
         </is>
       </c>
     </row>
@@ -2958,17 +2958,17 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>pl</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>R$ 143.232.764,20</t>
+          <t>113%</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>R$ 138.199.759,13</t>
+          <t>102%</t>
         </is>
       </c>
     </row>
@@ -2985,17 +2985,17 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>pl</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>R$ 155.004.649,74</t>
+          <t>R$ 143.232.764,20</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>R$ 162.868.029,59</t>
+          <t>R$ 138.199.759,13</t>
         </is>
       </c>
     </row>
@@ -3012,17 +3012,17 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>{'total': '84', 'top': [{'p': '33%', 'n': 'financeiro'}, {'p': '15%', 'n': 'FIDC'}, {'p': '8%', 'n': 'energia elétrica'}]}</t>
+          <t>R$ 155.004.649,74</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>{'total': '79', 'top': [{'p': '31%', 'n': 'financeiro'}, {'p': '15%', 'n': 'FIDC'}, {'p': '8%', 'n': 'energia elétrica'}]}</t>
+          <t>R$ 162.868.029,59</t>
         </is>
       </c>
     </row>
@@ -3039,17 +3039,17 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>{'total': '84', 'top': [{'p': '33%', 'n': 'financeiro'}, {'p': '15%', 'n': 'FIDC'}, {'p': '8%', 'n': 'energia elétrica'}]}</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>1,02</t>
+          <t>{'total': '79', 'top': [{'p': '31%', 'n': 'financeiro'}, {'p': '15%', 'n': 'FIDC'}, {'p': '8%', 'n': 'energia elétrica'}]}</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>1,79</t>
+          <t>1,02</t>
         </is>
       </c>
     </row>
@@ -3093,17 +3093,17 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>anos</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>ano</t>
+          <t>1,79</t>
         </is>
       </c>
     </row>
@@ -3120,17 +3120,17 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Taxa de administração: 0,63% a.a. Taxa de performance: 20% do que exceder o CDI. Resgate: D+30.</t>
+          <t>anos</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Taxa global: 0,625% a.a. Taxa de performance: 20% do que exceder 100% do CDI. Resgate: D+30.</t>
+          <t>ano</t>
         </is>
       </c>
     </row>
@@ -3142,22 +3142,22 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>infraplus</t>
+          <t>inst30</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>12,94%</t>
+          <t>Taxa de administração: 0,63% a.a. Taxa de performance: 20% do que exceder o CDI. Resgate: D+30.</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>9,10%</t>
+          <t>Taxa global: 0,625% a.a. Taxa de performance: 20% do que exceder 100% do CDI. Resgate: D+30.</t>
         </is>
       </c>
     </row>
@@ -3174,17 +3174,17 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>a1</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>*Alfa: -2,75%</t>
+          <t>12,94%</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>*Alfa: −5,70%</t>
+          <t>9,10%</t>
         </is>
       </c>
     </row>
@@ -3201,17 +3201,17 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>a1</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>7,80%</t>
+          <t>*Alfa: -2,75%</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>7,05%</t>
+          <t>*Alfa: −5,70%</t>
         </is>
       </c>
     </row>
@@ -3228,17 +3228,17 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>a2</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>*Alfa: -3,14%</t>
+          <t>7,80%</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>*Alfa: −4,32%</t>
+          <t>7,05%</t>
         </is>
       </c>
     </row>
@@ -3255,17 +3255,17 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>a2</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>1,24%</t>
+          <t>*Alfa: -3,14%</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>1,01%</t>
+          <t>*Alfa: −4,32%</t>
         </is>
       </c>
     </row>
@@ -3282,17 +3282,17 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>a3</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>*Alfa: -0,14%</t>
+          <t>1,24%</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>*Alfa: −1,00%</t>
+          <t>1,01%</t>
         </is>
       </c>
     </row>
@@ -3309,17 +3309,17 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>pl</t>
+          <t>a3</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>R$ 42.983.282,75</t>
+          <t>*Alfa: -0,14%</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>R$ 37.299.076,05</t>
+          <t>*Alfa: −1,00%</t>
         </is>
       </c>
     </row>
@@ -3336,17 +3336,17 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>pl</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>R$ 52.049.593,91</t>
+          <t>R$ 42.983.282,75</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>R$ 46.597.018,20</t>
+          <t>R$ 37.299.076,05</t>
         </is>
       </c>
     </row>
@@ -3363,17 +3363,17 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>{'total': '95', 'top': [{'p': '55%', 'n': 'energia elétrica'}, {'p': '15%', 'n': 'transporte e logística'}, {'p': '7%', 'n': 'saneamento'}]}</t>
+          <t>R$ 52.049.593,91</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>{'total': '97', 'top': [{'p': '53%', 'n': 'energia elétrica'}, {'p': '14%', 'n': 'transporte e logística'}, {'p': '8%', 'n': 'saneamento'}]}</t>
+          <t>R$ 46.597.018,20</t>
         </is>
       </c>
     </row>
@@ -3390,17 +3390,17 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>8,63</t>
+          <t>{'total': '95', 'top': [{'p': '55%', 'n': 'energia elétrica'}, {'p': '15%', 'n': 'transporte e logística'}, {'p': '7%', 'n': 'saneamento'}]}</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>8,11</t>
+          <t>{'total': '97', 'top': [{'p': '53%', 'n': 'energia elétrica'}, {'p': '14%', 'n': 'transporte e logística'}, {'p': '8%', 'n': 'saneamento'}]}</t>
         </is>
       </c>
     </row>
@@ -3422,12 +3422,12 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>4,00</t>
+          <t>8,63</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>3,99</t>
+          <t>8,11</t>
         </is>
       </c>
     </row>
@@ -3444,17 +3444,17 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Taxa de administração: 0,75% a.a. Taxa de performance: não há. Resgate: D+31. Rentabilidade isenta de IR para pessoa física.</t>
+          <t>4,00</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Taxa global: 0,75% a.a. Taxa de performance: não há. Resgate: D+31. Rentabilidade isenta de IR para pessoa física.</t>
+          <t>3,99</t>
         </is>
       </c>
     </row>
@@ -3466,22 +3466,22 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>infraplus</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>k1</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>12M</t>
+          <t>Taxa de administração: 0,75% a.a. Taxa de performance: não há. Resgate: D+31. Rentabilidade isenta de IR para pessoa física.</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Desde o início</t>
+          <t>Taxa global: 0,75% a.a. Taxa de performance: não há. Resgate: D+31. Rentabilidade isenta de IR para pessoa física.</t>
         </is>
       </c>
     </row>
@@ -3493,22 +3493,22 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>infraplus</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>inicio</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/12/2025</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>88%</t>
+          <t>15/07/2019</t>
         </is>
       </c>
     </row>
@@ -3525,17 +3525,17 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>k1</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12M</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>82%</t>
+          <t>Desde o início</t>
         </is>
       </c>
     </row>
@@ -3552,7 +3552,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -3562,7 +3562,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>−14%</t>
+          <t>88%</t>
         </is>
       </c>
     </row>
@@ -3579,7 +3579,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>pl</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -3589,7 +3589,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>R$ 44.023.801,59</t>
+          <t>82%</t>
         </is>
       </c>
     </row>
@@ -3606,7 +3606,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3616,7 +3616,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>R$ 37.965.174,74</t>
+          <t>−14%</t>
         </is>
       </c>
     </row>
@@ -3633,17 +3633,17 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>alloc</t>
+          <t>pl</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>{'total': '0', 'top': []}</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>{'total': '93', 'top': [{'p': '38%', 'n': 'energia elétrica'}, {'p': '22%', 'n': 'FIDC'}, {'p': '11%', 'n': 'transporte e logística'}]}</t>
+          <t>R$ 44.023.801,59</t>
         </is>
       </c>
     </row>
@@ -3660,7 +3660,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -3670,7 +3670,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>1,08</t>
+          <t>R$ 37.965.174,74</t>
         </is>
       </c>
     </row>
@@ -3687,17 +3687,17 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>val</t>
+          <t>alloc</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>{'total': '0', 'top': []}</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>3,70</t>
+          <t>{'total': '93', 'top': [{'p': '38%', 'n': 'energia elétrica'}, {'p': '22%', 'n': 'FIDC'}, {'p': '11%', 'n': 'transporte e logística'}]}</t>
         </is>
       </c>
     </row>
@@ -3714,17 +3714,17 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>taxas</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Taxa de administração: 0,75% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+30. Rentabilidade isenta de IR para pessoa física.</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Taxa global: 0,75% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+30. Rentabilidade isenta de IR para pessoa física.</t>
+          <t>1,08</t>
         </is>
       </c>
     </row>
@@ -3736,22 +3736,22 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>val</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>31/07/2026</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>3,70</t>
         </is>
       </c>
     </row>
@@ -3763,22 +3763,22 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>taxas</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Julho de 2026</t>
+          <t>Taxa de administração: 0,75% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+30. Rentabilidade isenta de IR para pessoa física.</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Setembro de 2026</t>
+          <t>Taxa global: 0,75% a.a. Taxa de performance: não há. Aplicação: D+0 · Resgate: D+30. Rentabilidade isenta de IR para pessoa física.</t>
         </is>
       </c>
     </row>
@@ -3800,12 +3800,12 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>julho de 2026</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>setembro de 2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
     </row>
@@ -3827,12 +3827,12 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>JULHO DE 2026</t>
+          <t>Julho de 2026</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>SETEMBRO DE 2026</t>
+          <t>Setembro de 2026</t>
         </is>
       </c>
     </row>
@@ -3854,12 +3854,12 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Julho 2026</t>
+          <t>julho de 2026</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Setembro 2026</t>
+          <t>setembro de 2026</t>
         </is>
       </c>
     </row>
@@ -3881,12 +3881,12 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>-jul26</t>
+          <t>JULHO DE 2026</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>-set26</t>
+          <t>SETEMBRO DE 2026</t>
         </is>
       </c>
     </row>
@@ -3908,12 +3908,12 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>const ATUAL=6;</t>
+          <t>Julho 2026</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>const ATUAL=8;</t>
+          <t>Setembro 2026</t>
         </is>
       </c>
     </row>
@@ -3930,71 +3930,71 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>libs de exportação</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>CDN</t>
+          <t>-jul26</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>4 referências → vendor/ local (CDN como reserva)</t>
+          <t>-set26</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>tivio-post-credito-privado.html</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>103%</t>
+          <t>const ATUAL=6;</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>48%</t>
+          <t>const ATUAL=8;</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>tivio-post-credito-privado.html</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>libs de exportação</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>101%</t>
+          <t>CDN</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>4 referências → vendor/ local (CDN como reserva)</t>
         </is>
       </c>
     </row>
@@ -4011,17 +4011,17 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>101%</t>
+          <t>103%</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>48%</t>
         </is>
       </c>
     </row>
@@ -4038,17 +4038,17 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>R$ 352,4 mi</t>
+          <t>101%</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>R$ 339,3 mi</t>
+          <t>93%</t>
         </is>
       </c>
     </row>
@@ -4060,17 +4060,17 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>104%</t>
+          <t>101%</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -4087,22 +4087,22 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>106%</t>
+          <t>R$ 352,4 mi</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>104%</t>
+          <t>R$ 339,3 mi</t>
         </is>
       </c>
     </row>
@@ -4119,17 +4119,17 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>109%</t>
+          <t>104%</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>106%</t>
+          <t>95%</t>
         </is>
       </c>
     </row>
@@ -4146,17 +4146,17 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>R$ 33,2 mi</t>
+          <t>106%</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>R$ 38,8 mi</t>
+          <t>104%</t>
         </is>
       </c>
     </row>
@@ -4168,22 +4168,22 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>adm</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>0,00% a.a. (vértice tx zero)</t>
+          <t>109%</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>0,15% a.a.</t>
+          <t>106%</t>
         </is>
       </c>
     </row>
@@ -4195,22 +4195,22 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>R$ 33,2 mi</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>R$ 38,8 mi</t>
         </is>
       </c>
     </row>
@@ -4227,17 +4227,17 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>adm</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>86%</t>
+          <t>0,00% a.a. (vértice tx zero)</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>87%</t>
+          <t>0,15% a.a.</t>
         </is>
       </c>
     </row>
@@ -4254,17 +4254,17 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>R$ 374,3 mi</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>R$ 329,9 mi</t>
+          <t>91%</t>
         </is>
       </c>
     </row>
@@ -4276,22 +4276,22 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>2,13%</t>
+          <t>86%</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>87%</t>
         </is>
       </c>
     </row>
@@ -4303,22 +4303,22 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>a1</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>*Alfa: −3,03%</t>
+          <t>R$ 374,3 mi</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>*Alfa: 1,41%</t>
+          <t>R$ 329,9 mi</t>
         </is>
       </c>
     </row>
@@ -4335,17 +4335,17 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>−5,35%</t>
+          <t>2,13%</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>0%</t>
         </is>
       </c>
     </row>
@@ -4362,17 +4362,17 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>a2</t>
+          <t>a1</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>*Alfa: −1,59%</t>
+          <t>*Alfa: −3,03%</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>*Alfa: 1,13%</t>
+          <t>*Alfa: 1,41%</t>
         </is>
       </c>
     </row>
@@ -4389,17 +4389,17 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>7,66%</t>
+          <t>−5,35%</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>13%</t>
+          <t>6%</t>
         </is>
       </c>
     </row>
@@ -4416,17 +4416,17 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>a3</t>
+          <t>a2</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>*Alfa: −6,22%</t>
+          <t>*Alfa: −1,59%</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>*Alfa: 0,50%</t>
+          <t>*Alfa: 1,13%</t>
         </is>
       </c>
     </row>
@@ -4443,17 +4443,17 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>R$ 100,8 mi</t>
+          <t>7,66%</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>R$ 70,7 mi</t>
+          <t>13%</t>
         </is>
       </c>
     </row>
@@ -4465,22 +4465,22 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>perf</t>
+          <t>a3</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>20% do que exceder o CDI</t>
+          <t>*Alfa: −6,22%</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>20% do que exceder 100% do CDI</t>
+          <t>*Alfa: 0,50%</t>
         </is>
       </c>
     </row>
@@ -4492,22 +4492,22 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>73%</t>
+          <t>R$ 100,8 mi</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>144%</t>
+          <t>R$ 70,7 mi</t>
         </is>
       </c>
     </row>
@@ -4524,17 +4524,17 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>perf</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>74%</t>
+          <t>20% do que exceder o CDI</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>83%</t>
+          <t>20% do que exceder 100% do CDI</t>
         </is>
       </c>
     </row>
@@ -4551,17 +4551,17 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>81%</t>
+          <t>73%</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>87%</t>
+          <t>144%</t>
         </is>
       </c>
     </row>
@@ -4578,17 +4578,17 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>R$ 102,7 mi</t>
+          <t>74%</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>R$ 95,5 mi</t>
+          <t>83%</t>
         </is>
       </c>
     </row>
@@ -4600,22 +4600,22 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>81%</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>141%</t>
+          <t>87%</t>
         </is>
       </c>
     </row>
@@ -4627,22 +4627,22 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>R$ 102,7 mi</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>R$ 95,5 mi</t>
         </is>
       </c>
     </row>
@@ -4659,17 +4659,17 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>141%</t>
         </is>
       </c>
     </row>
@@ -4686,17 +4686,17 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>R$ 662,8 mi</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>R$ 637,1 mi</t>
+          <t>98%</t>
         </is>
       </c>
     </row>
@@ -4708,22 +4708,22 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>31/07/2026</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>97%</t>
         </is>
       </c>
     </row>
@@ -4735,22 +4735,22 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>plm</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Julho de 2026</t>
+          <t>R$ 662,8 mi</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Setembro de 2026</t>
+          <t>R$ 637,1 mi</t>
         </is>
       </c>
     </row>
@@ -4772,12 +4772,12 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>julho de 2026</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>setembro de 2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
     </row>
@@ -4799,12 +4799,12 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>JULHO DE 2026</t>
+          <t>Julho de 2026</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>SETEMBRO DE 2026</t>
+          <t>Setembro de 2026</t>
         </is>
       </c>
     </row>
@@ -4826,12 +4826,12 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Julho 2026</t>
+          <t>julho de 2026</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Setembro 2026</t>
+          <t>setembro de 2026</t>
         </is>
       </c>
     </row>
@@ -4853,12 +4853,12 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>-jul26</t>
+          <t>JULHO DE 2026</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>-set26</t>
+          <t>SETEMBRO DE 2026</t>
         </is>
       </c>
     </row>
@@ -4880,12 +4880,12 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>const ATUAL=6;</t>
+          <t>Julho 2026</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>const ATUAL=8;</t>
+          <t>Setembro 2026</t>
         </is>
       </c>
     </row>
@@ -4902,71 +4902,71 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>libs de exportação</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>CDN</t>
+          <t>-jul26</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>4 referências → vendor/ local (CDN como reserva)</t>
+          <t>-set26</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>tivio-central.html</t>
+          <t>tivio-post-investment-solutions.html</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>s1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Julho 2026</t>
+          <t>const ATUAL=6;</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>Setembro 2026</t>
+          <t>const ATUAL=8;</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>tivio-central.html</t>
+          <t>tivio-post-investment-solutions.html</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>s2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>libs de exportação</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Julho 2026</t>
+          <t>CDN</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Setembro 2026</t>
+          <t>4 referências → vendor/ local (CDN como reserva)</t>
         </is>
       </c>
     </row>
@@ -4978,7 +4978,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>s8</t>
+          <t>s1</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -5005,7 +5005,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>e1</t>
+          <t>s2</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -5032,22 +5032,22 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>s8</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>date</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Relatório de Gestão · Incentivado CDI 30</t>
+          <t>Julho 2026</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Gerador de Relatório de Gestão · Incentivado CDI 30</t>
+          <t>Setembro 2026</t>
         </is>
       </c>
     </row>
@@ -5059,22 +5059,22 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>e1</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>desc</t>
+          <t>date</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Relatório de gestão mensal do Tivio Institucional Inc CDI 30 FIF (debêntures incentivadas · CDI).</t>
+          <t>Julho 2026</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Construtor interativo, folha a folha. Os relatórios prontos do mês estão no card acima. Relatório de gestão mensal do Tivio Institucional Inc CDI 30 FIF (debêntures incentivadas · CDI).</t>
+          <t>Setembro 2026</t>
         </is>
       </c>
     </row>
@@ -5086,22 +5086,22 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>title</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>cards de relatório</t>
+          <t>Relatório de Gestão · Incentivado CDI 30</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>2 registrados para Setembro 2026</t>
+          <t>Gerador de Relatório de Gestão · Incentivado CDI 30</t>
         </is>
       </c>
     </row>
@@ -5113,16 +5113,70 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
+          <t>r2</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>desc</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Relatório de gestão mensal do Tivio Institucional Inc CDI 30 FIF (debêntures incentivadas · CDI).</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Construtor interativo, folha a folha. Os relatórios prontos do mês estão no card acima. Relatório de gestão mensal do Tivio Institucional Inc CDI 30 FIF (debêntures incentivadas · CDI).</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>tivio-central.html</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C174" t="inlineStr">
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>cards de relatório</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>2 registrados para Setembro 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>tivio-central.html</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
         <is>
           <t>data automática</t>
         </is>
       </c>
-      <c r="D174" t="inlineStr"/>
-      <c r="E174" t="inlineStr">
+      <c r="D176" t="inlineStr"/>
+      <c r="E176" t="inlineStr">
         <is>
           <t>DATA_BASE=2026-09-30</t>
         </is>
@@ -12159,7 +12213,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>818853</v>
+        <v>818849</v>
       </c>
     </row>
     <row r="7">
@@ -12174,7 +12228,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1990766</v>
+        <v>1990765</v>
       </c>
     </row>
     <row r="8">
@@ -12519,7 +12573,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>540379</v>
+        <v>548567</v>
       </c>
     </row>
     <row r="31">
@@ -12534,7 +12588,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>547655</v>
+        <v>555260</v>
       </c>
     </row>
     <row r="32">
@@ -12549,7 +12603,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2093582</v>
+        <v>2093588</v>
       </c>
     </row>
     <row r="33">
@@ -12729,7 +12783,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4829398</v>
+        <v>4829397</v>
       </c>
     </row>
     <row r="45">
@@ -12759,7 +12813,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>5454371</v>
+        <v>5454370</v>
       </c>
     </row>
     <row r="47">

</xml_diff>

<commit_message>
AutomaTivio: carrossel dos ALT com uma cor por categoria (nomes novos FIDCs Cota Sênior/Mezanino e garantia de cor única)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -12116,7 +12116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -12144,705 +12144,210 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tivio Banks - Relatório de Gestão - Setembro 2026.pdf</t>
+          <t>Relatório de Gestão - Crédito Privado - Setembro 2026.html</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>808661</v>
+        <v>4965627</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tivio Banks - Relatório de Gestão - Setembro 2026.pptx</t>
+          <t>Relatório de Gestão - Crédito Estruturado - Setembro 2026.html</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>pptx</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1964410</v>
+        <v>1917800</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tivio Institucional - Relatório de Gestão - Setembro 2026.pdf</t>
+          <t>tivio-hgd30-saiba-mais.html</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>815298</v>
+        <v>548567</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tivio Institucional - Relatório de Gestão - Setembro 2026.pptx</t>
+          <t>tivio-hyd60-saiba-mais.html</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>pptx</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1971592</v>
+        <v>555260</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tivio Institucional 15 - Relatório de Gestão - Setembro 2026.pdf</t>
+          <t>tivio-email-previdencia.html</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>818849</v>
+        <v>2093588</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Tivio Institucional 15 - Relatório de Gestão - Setembro 2026.pptx</t>
+          <t>tivio-construtor-one-pager.html</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>pptx</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1990765</v>
+        <v>88038</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Tivio Institucional 30 - Relatório de Gestão - Setembro 2026.pdf</t>
+          <t>tivio-email-fundos-credito.html</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>814574</v>
+        <v>203856</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Tivio Institucional 30 - Relatório de Gestão - Setembro 2026.pptx</t>
+          <t>tivio-email-nordea-studio.html</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>pptx</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1965551</v>
+        <v>50469</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus - Relatório de Gestão - Setembro 2026.pdf</t>
+          <t>tivio-post-credito-estruturado.html</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>789265</v>
+        <v>118824</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus - Relatório de Gestão - Setembro 2026.pptx</t>
+          <t>tivio-post-credito-privado.html</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>pptx</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1950734</v>
+        <v>132576</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Tivio BVP - Relatório de Gestão - Setembro 2026.pdf</t>
+          <t>tivio-post-investment-solutions.html</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>797776</v>
+        <v>103238</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Tivio BVP - Relatório de Gestão - Setembro 2026.pptx</t>
+          <t>tivio-central.html</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>pptx</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1947704</v>
+        <v>67857</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Tivio RF CP - Relatório de Gestão - Setembro 2026.pdf</t>
+          <t>destaques</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>jpg</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>807467</v>
+        <v>4096</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Tivio RF CP - Relatório de Gestão - Setembro 2026.pptx</t>
+          <t>index.html</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>pptx</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1961950</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Tivio ALT 180 - Relatório de Gestão - Setembro 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>598823</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Tivio ALT 180 - Relatório de Gestão - Setembro 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>300534</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Tivio ALT 90 - Relatório de Gestão - Setembro 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>596967</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Tivio ALT 90 - Relatório de Gestão - Setembro 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>296395</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Tivio ALT Light - Relatório de Gestão - Setembro 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>592864</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Tivio ALT Light - Relatório de Gestão - Setembro 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>289334</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Tivio Infra Plus CDI - Relatório de Gestão - Setembro 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>810017</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Tivio Infra Plus CDI - Relatório de Gestão - Setembro 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>1965143</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Tivio Esplanada - Relatório de Gestão - Setembro 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>812335</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Tivio Esplanada - Relatório de Gestão - Setembro 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>1973341</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Tivio Legacy Prev - Relatório de Gestão - Setembro 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>810719</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Tivio Legacy Prev - Relatório de Gestão - Setembro 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>1964297</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Relatório de Gestão - Crédito Privado - Setembro 2026.html</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>4965627</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Relatório de Gestão - Crédito Estruturado - Setembro 2026.html</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>1917800</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>tivio-hgd30-saiba-mais.html</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>548567</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>tivio-hyd60-saiba-mais.html</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>555260</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>tivio-email-previdencia.html</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>2093588</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>tivio-construtor-one-pager.html</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>88038</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>tivio-email-fundos-credito.html</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>203856</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>tivio-email-nordea-studio.html</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>50469</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>tivio-post-credito-estruturado.html</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>118207</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>tivio-post-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>132576</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>tivio-post-investment-solutions.html</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>103238</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>67857</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>destaques</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>jpg</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>4096</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>emails</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>png</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>hgd30</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>png</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>4096</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>hyd60</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>png</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>4096</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Informativo - HGD30 - Setembro 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>4829397</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Informativo - HGD30 - Setembro 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C45" t="n">
-        <v>422853</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Informativo - HYD60 - Setembro 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>5454370</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Informativo - HYD60 - Setembro 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>554367</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>index.html</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C48" t="n">
         <v>394</v>
       </c>
     </row>

</xml_diff>

<commit_message>
AutomaTivio: rentabilidade do HGD30 e do HYD60 pela classe FIE (BRADESCO TIVIO … PGBL/VGBL), carteira e PL do FIFE; edição de setembro refeita
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -8555,19 +8555,19 @@
         <v>46265</v>
       </c>
       <c r="G68" t="n">
-        <v>0.01062530137458406</v>
+        <v>0.01015661305298132</v>
       </c>
       <c r="H68" t="n">
         <v>0.01082559188004661</v>
       </c>
       <c r="I68" t="n">
-        <v>-0.0002002905054625526</v>
+        <v>-0.0006689788270652919</v>
       </c>
       <c r="J68" t="n">
-        <v>0.9814984245035394</v>
+        <v>0.9382039490793725</v>
       </c>
       <c r="K68" t="n">
-        <v>-0.002375156005994805</v>
+        <v>-0.007912927345822274</v>
       </c>
     </row>
     <row r="69">
@@ -8740,19 +8740,19 @@
         <v>46085</v>
       </c>
       <c r="G73" t="n">
-        <v>0.08733539999999995</v>
+        <v>0.08469909999999992</v>
       </c>
       <c r="H73" t="n">
         <v>0.07982471914470612</v>
       </c>
       <c r="I73" t="n">
-        <v>0.007510680855293828</v>
+        <v>0.004874380855293792</v>
       </c>
       <c r="J73" t="n">
-        <v>1.094089662146865</v>
+        <v>1.061063551585537</v>
       </c>
       <c r="K73" t="n">
-        <v>0.01211911820212941</v>
+        <v>0.00785816559619934</v>
       </c>
     </row>
     <row r="74">
@@ -11842,7 +11842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -11887,102 +11887,102 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>relatorio/bvp</t>
+          <t>—</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>bvp</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>logo não encontrado em assets/logos (procurei "tivio_bvp")</t>
+          <t>sem cotas de "BRADESCO TIVIO HGD30 PGBL/VGBL" na dados_mensais: a rentabilidade saiu do TIVIO HGD30 FIFE RESP LIMITADA FIF RENDA FIXA CRÉDITO PRIVADO (inclua a classe na planilha para usar a dela)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>relatorio/atuarial</t>
+          <t>relatorio/bvp</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>atuarial</t>
+          <t>bvp</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>relatório não gerado: sem dados nesta edição</t>
+          <t>logo não encontrado em assets/logos (procurei "tivio_bvp")</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>relatorio/credito_privado</t>
+          <t>relatorio/atuarial</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>bvp</t>
+          <t>atuarial</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>logo não encontrado em assets/logos (procurei "tivio_bvp")</t>
+          <t>relatório não gerado: sem dados nesta edição</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>landing/hgd30</t>
+          <t>relatorio/credito_privado</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>hgd30</t>
+          <t>bvp</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): Na atribuição de performance, a carteira de títulos bancários foi a principal re…</t>
+          <t>logo não encontrado em assets/logos (procurei "tivio_bvp")</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>landing/hyd60</t>
+          <t>landing/hgd30</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>hyd60</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): - Na parcela de **crédito estruturado**, avanço na **diversificação da carteira*…</t>
+          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): Na atribuição de performance, a carteira de títulos bancários foi a principal re…</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>email/previdencia</t>
+          <t>landing/hyd60</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>hgd30</t>
+          <t>hyd60</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): Na atribuição de performance, a carteira de títulos bancários foi a principal re…</t>
+          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): - Na parcela de **crédito estruturado**, avanço na **diversificação da carteira*…</t>
         </is>
       </c>
     </row>
@@ -11994,36 +11994,36 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>hyd60</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): - Na parcela de **crédito estruturado**, avanço na **diversificação da carteira*…</t>
+          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): Na atribuição de performance, a carteira de títulos bancários foi a principal re…</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>tivio-email-fundos-credito.html</t>
+          <t>email/previdencia</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>alt180</t>
+          <t>hyd60</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>o texto se refere a "julho" como o mês corrente — a data base é setembro</t>
+          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): - Na parcela de **crédito estruturado**, avanço na **diversificação da carteira*…</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>tivio-email-fundos-credito.html</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -12033,7 +12033,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Mz', 'Fiagro Sr']</t>
+          <t>o texto se refere a "julho" como o mês corrente — a data base é setembro</t>
         </is>
       </c>
     </row>
@@ -12045,29 +12045,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>alt90</t>
+          <t>alt180</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Sr']</t>
+          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Mz', 'Fiagro Sr']</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>tivio-post-credito-estruturado.html</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>topgestormacro</t>
+          <t>alt90</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>sem dados — rentabilidade e PL mantidos</t>
+          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Sr']</t>
         </is>
       </c>
     </row>
@@ -12079,7 +12079,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>topgestorlongonly</t>
+          <t>topgestormacro</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -12091,15 +12091,32 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>tivio-post-investment-solutions.html</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>topgestorlongonly</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>sem dados — rentabilidade e PL mantidos</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>tivio-central.html</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>tivio-central.html</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>card "Gerador de Relatório de Gestão · Incentivado CDI 30" removido: aponta para "Tivio Incentivado CDI 30 - Relatório de Gestão Mensal.html", que não existe nesta edição</t>
         </is>
@@ -12116,7 +12133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -12144,210 +12161,975 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Relatório de Gestão - Crédito Privado - Setembro 2026.html</t>
+          <t>Tivio Banks - Relatório de Gestão - Setembro 2026.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4965627</v>
+        <v>808661</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Relatório de Gestão - Crédito Estruturado - Setembro 2026.html</t>
+          <t>Tivio Banks - Relatório de Gestão - Setembro 2026.pptx</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pptx</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1917800</v>
+        <v>1964410</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>tivio-hgd30-saiba-mais.html</t>
+          <t>Tivio Institucional - Relatório de Gestão - Setembro 2026.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>548567</v>
+        <v>815298</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>tivio-hyd60-saiba-mais.html</t>
+          <t>Tivio Institucional - Relatório de Gestão - Setembro 2026.pptx</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pptx</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>555260</v>
+        <v>1971592</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>tivio-email-previdencia.html</t>
+          <t>Tivio Institucional 15 - Relatório de Gestão - Setembro 2026.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2093588</v>
+        <v>818849</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>tivio-construtor-one-pager.html</t>
+          <t>Tivio Institucional 15 - Relatório de Gestão - Setembro 2026.pptx</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pptx</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>88038</v>
+        <v>1990765</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>tivio-email-fundos-credito.html</t>
+          <t>Tivio Institucional 30 - Relatório de Gestão - Setembro 2026.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>203856</v>
+        <v>814574</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>tivio-email-nordea-studio.html</t>
+          <t>Tivio Institucional 30 - Relatório de Gestão - Setembro 2026.pptx</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pptx</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>50469</v>
+        <v>1965551</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>Tivio Infra Plus - Relatório de Gestão - Setembro 2026.pdf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>118824</v>
+        <v>789265</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>tivio-post-credito-privado.html</t>
+          <t>Tivio Infra Plus - Relatório de Gestão - Setembro 2026.pptx</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pptx</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>132576</v>
+        <v>1950734</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>Tivio BVP - Relatório de Gestão - Setembro 2026.pdf</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>103238</v>
+        <v>797776</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>tivio-central.html</t>
+          <t>Tivio BVP - Relatório de Gestão - Setembro 2026.pptx</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pptx</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>67857</v>
+        <v>1947704</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>destaques</t>
+          <t>Tivio RF CP - Relatório de Gestão - Setembro 2026.pdf</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>jpg</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>4096</v>
+        <v>807467</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Tivio RF CP - Relatório de Gestão - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1961950</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Tivio ALT 180 - Relatório de Gestão - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>598823</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Tivio ALT 180 - Relatório de Gestão - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>300534</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Tivio ALT 90 - Relatório de Gestão - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>596967</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Tivio ALT 90 - Relatório de Gestão - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>296395</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Tivio ALT Light - Relatório de Gestão - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>592864</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Tivio ALT Light - Relatório de Gestão - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>289334</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Tivio Infra Plus CDI - Relatório de Gestão - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>810017</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Tivio Infra Plus CDI - Relatório de Gestão - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1965143</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Tivio Esplanada - Relatório de Gestão - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>812335</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Tivio Esplanada - Relatório de Gestão - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1973341</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev - Relatório de Gestão - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>810719</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev - Relatório de Gestão - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1964297</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Relatório de Gestão - Crédito Privado - Setembro 2026.html</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>4965627</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Relatório de Gestão - Crédito Estruturado - Setembro 2026.html</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1917800</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>tivio-hgd30-saiba-mais.html</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>548567</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>tivio-hyd60-saiba-mais.html</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>555259</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>tivio-email-previdencia.html</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>2093587</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>tivio-construtor-one-pager.html</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>88038</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>tivio-email-fundos-credito.html</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>203856</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>tivio-email-nordea-studio.html</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>50469</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>tivio-post-credito-estruturado.html</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>118824</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>tivio-post-credito-privado.html</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>132576</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>tivio-post-investment-solutions.html</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>103238</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>tivio-central.html</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>67857</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>destaques</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>jpg</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>4096</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>emails</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>png</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>hgd30</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>png</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>4096</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>hyd60</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>png</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>4096</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Informativo - HGD30 - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>4829399</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Informativo - HGD30 - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>422853</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Informativo - HYD60 - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>5454372</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Informativo - HYD60 - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>554378</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Tivio ALT 180 - ALT 90 - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>16816513</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Tivio ALT 180 - ALT 90 - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>3009396</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>BTG - ALT 180 - ALT 90 - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>15593104</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>BTG - ALT 180 - ALT 90 - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>2616247</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>XP - Tivio ALT 180 - ALT 90 - ALT Light - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>15041374</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>XP - Tivio ALT 180 - ALT 90 - ALT Light - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>2467250</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Deck - Tivio ALT 90 - Sem ROA - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>25551962</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Deck - Tivio ALT 90 - Sem ROA - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>2649979</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Deck - Tivio ALT 90 - Com ROA - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>23546223</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Deck - Tivio ALT 90 - Com ROA - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>2643349</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Deck - Tivio ALT 180 - Sem ROA - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>26316559</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Deck - Tivio ALT 180 - Sem ROA - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>4115895</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Deck - Tivio ALT 180 - Com ROA - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>26316813</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Deck - Tivio ALT 180 - Com ROA - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>4116719</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Deck - Crédito Privado &amp; Crédito Estruturado - BTG - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>26457372</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Deck - Crédito Privado &amp; Crédito Estruturado - BTG - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>3802493</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Deck - Crédito Privado &amp; Crédito Estruturado - XP - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>26317598</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Deck - Crédito Privado &amp; Crédito Estruturado - XP - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>3976310</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
           <t>index.html</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B66" t="inlineStr">
         <is>
           <t>html</t>
         </is>
       </c>
-      <c r="C15" t="n">
+      <c r="C66" t="n">
         <v>394</v>
       </c>
     </row>

</xml_diff>

<commit_message>
AutomaTivio: deck Tivio Conecta (tabelas, barras mensais, rating, setorial, composição), slides de fundo no estilo dos posts, HGD30 pelo FIE (HGD 30), Conexão ALT 180 no cadastro, pasta saida/_Atual
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -5279,7 +5279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -5313,122 +5313,122 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>conexaoalt180</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BV Top Gestor Crédito Privado</t>
+          <t>Conexão Tivio ALT 180</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>comentário do gestor</t>
+          <t>carteira</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>não preenchido no arquivo de comentários</t>
+          <t>sem linhas na Base Carteira</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>conexaoalt180</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tivio Top Gestor HY</t>
+          <t>Conexão Tivio ALT 180</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>comentário do gestor</t>
+          <t>taxa global</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>não preenchido no arquivo de comentários</t>
+          <t>não calculado nesta edição</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>conexaoalt180</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BV Top Gestor RF Ativo</t>
+          <t>Conexão Tivio ALT 180</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>comentário do gestor</t>
+          <t>carrego</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>não preenchido no arquivo de comentários</t>
+          <t>não calculado nesta edição</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>topgestormacro</t>
+          <t>conexaoalt180</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BV Top Gestor Macro</t>
+          <t>Conexão Tivio ALT 180</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>rentabilidade</t>
+          <t>duration</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>sem cotas na dados_mensais</t>
+          <t>não calculado nesta edição</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>topgestorlongonly</t>
+          <t>conexaoalt180</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Top Gestor Ações Long Only</t>
+          <t>Conexão Tivio ALT 180</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>rentabilidade</t>
+          <t>comentário do gestor</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>sem cotas na dados_mensais</t>
+          <t>não preenchido no arquivo de comentários</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Tivio Top Manager Global</t>
+          <t>BV Top Gestor Crédito Privado</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -5445,12 +5445,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tivio RF Ativo Longo Prazo</t>
+          <t>Tivio Top Gestor HY</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -5467,12 +5467,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tivio Prev Low Vol Itaú</t>
+          <t>BV Top Gestor RF Ativo</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -5489,20 +5489,130 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>topgestormacro</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>BV Top Gestor Macro</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>rentabilidade</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>sem cotas na dados_mensais</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>topgestorlongonly</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Top Gestor Ações Long Only</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>rentabilidade</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>sem cotas na dados_mensais</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>topmanagerglobal</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Tivio Top Manager Global</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>comentário do gestor</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>não preenchido no arquivo de comentários</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ativorf</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Tivio RF Ativo Longo Prazo</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>comentário do gestor</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>não preenchido no arquivo de comentários</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>prevlowvol</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Tivio Prev Low Vol Itaú</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>comentário do gestor</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>não preenchido no arquivo de comentários</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>atuarial</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Tivio Atuarial</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>rentabilidade</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>sem cotas na dados_mensais</t>
         </is>
@@ -5602,7 +5712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K127"/>
+  <dimension ref="A1:K133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8278,17 +8388,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>hgd30</t>
+          <t>conexaoalt180</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Tivio HGD30</t>
+          <t>Conexão Tivio ALT 180</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>TIVIO HGD30 RF CP FIFE RL</t>
+          <t>CONEXÃO TIVIO ALT HY 180 RL FIM CP</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -8305,35 +8415,35 @@
         <v>46265</v>
       </c>
       <c r="G62" t="n">
-        <v>0.0108528654278528</v>
+        <v>0.01256505769580896</v>
       </c>
       <c r="H62" t="n">
         <v>0.01082559188004661</v>
       </c>
       <c r="I62" t="n">
-        <v>2.727354780618363e-05</v>
+        <v>0.001739465815762342</v>
       </c>
       <c r="J62" t="n">
-        <v>1.002519358581812</v>
+        <v>1.160680897177407</v>
       </c>
       <c r="K62" t="n">
-        <v>0.0003238255429589554</v>
+        <v>0.02084661073972982</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>hgd30</t>
+          <t>conexaoalt180</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Tivio HGD30</t>
+          <t>Conexão Tivio ALT 180</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>TIVIO HGD30 RF CP FIFE RL</t>
+          <t>CONEXÃO TIVIO ALT HY 180 RL FIM CP</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -8350,35 +8460,35 @@
         <v>46022</v>
       </c>
       <c r="G63" t="n">
-        <v>0.1071791004655822</v>
+        <v>0.1212615229042946</v>
       </c>
       <c r="H63" t="n">
         <v>0.1051127846901438</v>
       </c>
       <c r="I63" t="n">
-        <v>0.002066315775438365</v>
+        <v>0.01614873821415075</v>
       </c>
       <c r="J63" t="n">
-        <v>1.019658082330609</v>
+        <v>1.153632484019472</v>
       </c>
       <c r="K63" t="n">
-        <v>0.002520519554925826</v>
+        <v>0.01974190272509979</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>hgd30</t>
+          <t>conexaoalt180</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Tivio HGD30</t>
+          <t>Conexão Tivio ALT 180</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>TIVIO HGD30 RF CP FIFE RL</t>
+          <t>CONEXÃO TIVIO ALT HY 180 RL FIM CP</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -8395,35 +8505,35 @@
         <v>45930</v>
       </c>
       <c r="G64" t="n">
-        <v>0.146604148478189</v>
+        <v>0.1718266240927331</v>
       </c>
       <c r="H64" t="n">
         <v>0.1447903912030524</v>
       </c>
       <c r="I64" t="n">
-        <v>0.001813757275136663</v>
+        <v>0.02703623288968071</v>
       </c>
       <c r="J64" t="n">
-        <v>1.012526779298448</v>
+        <v>1.186726706551717</v>
       </c>
       <c r="K64" t="n">
-        <v>0.001590674727792951</v>
+        <v>0.02371195135192483</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>hgd30</t>
+          <t>conexaoalt180</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Tivio HGD30</t>
+          <t>Conexão Tivio ALT 180</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>TIVIO HGD30 RF CP FIFE RL</t>
+          <t>CONEXÃO TIVIO ALT HY 180 RL FIM CP</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -8437,7 +8547,7 @@
         </is>
       </c>
       <c r="F65" s="1" t="n">
-        <v>45786</v>
+        <v>45777</v>
       </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr"/>
@@ -8448,17 +8558,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>hgd30</t>
+          <t>conexaoalt180</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Tivio HGD30</t>
+          <t>Conexão Tivio ALT 180</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>TIVIO HGD30 RF CP FIFE RL</t>
+          <t>CONEXÃO TIVIO ALT HY 180 RL FIM CP</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -8472,7 +8582,7 @@
         </is>
       </c>
       <c r="F66" s="1" t="n">
-        <v>45786</v>
+        <v>45777</v>
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr"/>
@@ -8483,17 +8593,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>hgd30</t>
+          <t>conexaoalt180</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Tivio HGD30</t>
+          <t>Conexão Tivio ALT 180</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>TIVIO HGD30 RF CP FIFE RL</t>
+          <t>CONEXÃO TIVIO ALT HY 180 RL FIM CP</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -8507,38 +8617,38 @@
         </is>
       </c>
       <c r="F67" s="1" t="n">
-        <v>45786</v>
+        <v>45777</v>
       </c>
       <c r="G67" t="n">
-        <v>0.2187760000000001</v>
+        <v>0.2613932000000001</v>
       </c>
       <c r="H67" t="n">
-        <v>0.2100212531349583</v>
+        <v>0.2138611305291156</v>
       </c>
       <c r="I67" t="n">
-        <v>0.00875474686504174</v>
+        <v>0.04753206947088451</v>
       </c>
       <c r="J67" t="n">
-        <v>1.041685052033358</v>
+        <v>1.222256701595493</v>
       </c>
       <c r="K67" t="n">
-        <v>0.005174439153091015</v>
+        <v>0.02740641052062553</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>hyd60</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Tivio HYD60</t>
+          <t>Tivio HGD30</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>TIVIO HYD60 FIFE CI MULT CP RL - Expandida</t>
+          <t>TIVIO HGD30 RF CP FIFE RL</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -8555,35 +8665,35 @@
         <v>46265</v>
       </c>
       <c r="G68" t="n">
-        <v>0.01015661305298132</v>
+        <v>0.01037586029663151</v>
       </c>
       <c r="H68" t="n">
         <v>0.01082559188004661</v>
       </c>
       <c r="I68" t="n">
-        <v>-0.0006689788270652919</v>
+        <v>-0.0004497315834151028</v>
       </c>
       <c r="J68" t="n">
-        <v>0.9382039490793725</v>
+        <v>0.9584566286630448</v>
       </c>
       <c r="K68" t="n">
-        <v>-0.007912927345822274</v>
+        <v>-0.005325936059542791</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>hyd60</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Tivio HYD60</t>
+          <t>Tivio HGD30</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>TIVIO HYD60 FIFE CI MULT CP RL - Expandida</t>
+          <t>TIVIO HGD30 RF CP FIFE RL</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -8597,28 +8707,38 @@
         </is>
       </c>
       <c r="F69" s="1" t="n">
-        <v>46085</v>
-      </c>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr"/>
-      <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
+        <v>46022</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0.1024512297203906</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0.1051127846901438</v>
+      </c>
+      <c r="I69" t="n">
+        <v>-0.002661554969753288</v>
+      </c>
+      <c r="J69" t="n">
+        <v>0.9746790556676893</v>
+      </c>
+      <c r="K69" t="n">
+        <v>-0.00324418680973515</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>hyd60</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Tivio HYD60</t>
+          <t>Tivio HGD30</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>TIVIO HYD60 FIFE CI MULT CP RL - Expandida</t>
+          <t>TIVIO HGD30 RF CP FIFE RL</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -8632,28 +8752,38 @@
         </is>
       </c>
       <c r="F70" s="1" t="n">
-        <v>46085</v>
-      </c>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr"/>
+        <v>45930</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0.1400882650805524</v>
+      </c>
+      <c r="H70" t="n">
+        <v>0.1447903912030524</v>
+      </c>
+      <c r="I70" t="n">
+        <v>-0.004702126122499983</v>
+      </c>
+      <c r="J70" t="n">
+        <v>0.9675245982593846</v>
+      </c>
+      <c r="K70" t="n">
+        <v>-0.004123742695322008</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>hyd60</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Tivio HYD60</t>
+          <t>Tivio HGD30</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>TIVIO HYD60 FIFE CI MULT CP RL - Expandida</t>
+          <t>TIVIO HGD30 RF CP FIFE RL</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -8667,7 +8797,7 @@
         </is>
       </c>
       <c r="F71" s="1" t="n">
-        <v>46085</v>
+        <v>45786</v>
       </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr"/>
@@ -8678,17 +8808,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>hyd60</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Tivio HYD60</t>
+          <t>Tivio HGD30</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>TIVIO HYD60 FIFE CI MULT CP RL - Expandida</t>
+          <t>TIVIO HGD30 RF CP FIFE RL</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -8702,7 +8832,7 @@
         </is>
       </c>
       <c r="F72" s="1" t="n">
-        <v>46085</v>
+        <v>45786</v>
       </c>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr"/>
@@ -8713,17 +8843,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>hyd60</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Tivio HYD60</t>
+          <t>Tivio HGD30</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>TIVIO HYD60 FIFE CI MULT CP RL - Expandida</t>
+          <t>TIVIO HGD30 RF CP FIFE RL</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -8737,38 +8867,38 @@
         </is>
       </c>
       <c r="F73" s="1" t="n">
-        <v>46085</v>
+        <v>45786</v>
       </c>
       <c r="G73" t="n">
-        <v>0.08469909999999992</v>
+        <v>0.2083775000000001</v>
       </c>
       <c r="H73" t="n">
-        <v>0.07982471914470612</v>
+        <v>0.2100212531349583</v>
       </c>
       <c r="I73" t="n">
-        <v>0.004874380855293792</v>
+        <v>-0.001643753134958237</v>
       </c>
       <c r="J73" t="n">
-        <v>1.061063551585537</v>
+        <v>0.992173396213849</v>
       </c>
       <c r="K73" t="n">
-        <v>0.00785816559619934</v>
+        <v>-0.0009727143342039835</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>hyd60</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>BV Top Gestor Crédito Privado</t>
+          <t>Tivio HYD60</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
+          <t>TIVIO HYD60 FIFE CI MULT CP RL - Expandida</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -8785,35 +8915,35 @@
         <v>46265</v>
       </c>
       <c r="G74" t="n">
-        <v>0.005219350133194078</v>
+        <v>0.01015661305298132</v>
       </c>
       <c r="H74" t="n">
         <v>0.01082559188004661</v>
       </c>
       <c r="I74" t="n">
-        <v>-0.005606241746852536</v>
+        <v>-0.0006689788270652919</v>
       </c>
       <c r="J74" t="n">
-        <v>0.4821306946564481</v>
+        <v>0.9382039490793725</v>
       </c>
       <c r="K74" t="n">
-        <v>-0.06456129582370584</v>
+        <v>-0.007912927345822274</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>hyd60</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>BV Top Gestor Crédito Privado</t>
+          <t>Tivio HYD60</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
+          <t>TIVIO HYD60 FIFE CI MULT CP RL - Expandida</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8827,38 +8957,28 @@
         </is>
       </c>
       <c r="F75" s="1" t="n">
-        <v>46022</v>
-      </c>
-      <c r="G75" t="n">
-        <v>0.09822271466718724</v>
-      </c>
-      <c r="H75" t="n">
-        <v>0.1051127846901438</v>
-      </c>
-      <c r="I75" t="n">
-        <v>-0.006890070022956607</v>
-      </c>
-      <c r="J75" t="n">
-        <v>0.9344506946203789</v>
-      </c>
-      <c r="K75" t="n">
-        <v>-0.008392753749412729</v>
-      </c>
+        <v>46085</v>
+      </c>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>hyd60</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>BV Top Gestor Crédito Privado</t>
+          <t>Tivio HYD60</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
+          <t>TIVIO HYD60 FIFE CI MULT CP RL - Expandida</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8872,38 +8992,28 @@
         </is>
       </c>
       <c r="F76" s="1" t="n">
-        <v>45930</v>
-      </c>
-      <c r="G76" t="n">
-        <v>0.1373601954243717</v>
-      </c>
-      <c r="H76" t="n">
-        <v>0.1447903912030524</v>
-      </c>
-      <c r="I76" t="n">
-        <v>-0.007430195778680648</v>
-      </c>
-      <c r="J76" t="n">
-        <v>0.9486830878973134</v>
-      </c>
-      <c r="K76" t="n">
-        <v>-0.006516216027085298</v>
-      </c>
+        <v>46085</v>
+      </c>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>hyd60</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>BV Top Gestor Crédito Privado</t>
+          <t>Tivio HYD60</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
+          <t>TIVIO HYD60 FIFE CI MULT CP RL - Expandida</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -8917,38 +9027,28 @@
         </is>
       </c>
       <c r="F77" s="1" t="n">
-        <v>45561</v>
-      </c>
-      <c r="G77" t="n">
-        <v>0.2920431856569192</v>
-      </c>
-      <c r="H77" t="n">
-        <v>0.2980670513506256</v>
-      </c>
-      <c r="I77" t="n">
-        <v>-0.006023865693706387</v>
-      </c>
-      <c r="J77" t="n">
-        <v>0.9797902328807878</v>
-      </c>
-      <c r="K77" t="n">
-        <v>-0.002327632629077092</v>
-      </c>
+        <v>46085</v>
+      </c>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>hyd60</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>BV Top Gestor Crédito Privado</t>
+          <t>Tivio HYD60</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
+          <t>TIVIO HYD60 FIFE CI MULT CP RL - Expandida</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -8962,38 +9062,28 @@
         </is>
       </c>
       <c r="F78" s="1" t="n">
-        <v>45195</v>
-      </c>
-      <c r="G78" t="n">
-        <v>0.4695527796319496</v>
-      </c>
-      <c r="H78" t="n">
-        <v>0.4424561999402108</v>
-      </c>
-      <c r="I78" t="n">
-        <v>0.02709657969173884</v>
-      </c>
-      <c r="J78" t="n">
-        <v>1.06124127019895</v>
-      </c>
-      <c r="K78" t="n">
-        <v>0.006231139290297394</v>
-      </c>
+        <v>46085</v>
+      </c>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>hyd60</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>BV Top Gestor Crédito Privado</t>
+          <t>Tivio HYD60</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
+          <t>TIVIO HYD60 FIFE CI MULT CP RL - Expandida</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -9007,38 +9097,38 @@
         </is>
       </c>
       <c r="F79" s="1" t="n">
-        <v>44706</v>
+        <v>46085</v>
       </c>
       <c r="G79" t="n">
-        <v>0.7203075669000001</v>
+        <v>0.08469909999999992</v>
       </c>
       <c r="H79" t="n">
-        <v>0.7084789393875421</v>
+        <v>0.07982471914470612</v>
       </c>
       <c r="I79" t="n">
-        <v>0.01182862751245795</v>
+        <v>0.004874380855293792</v>
       </c>
       <c r="J79" t="n">
-        <v>1.016695806826218</v>
+        <v>1.061063551585537</v>
       </c>
       <c r="K79" t="n">
-        <v>0.001593489935187264</v>
+        <v>0.00785816559619934</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Tivio Top Gestor HY</t>
+          <t>BV Top Gestor Crédito Privado</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>TIVIO TOP GESTOR HY FIF RL</t>
+          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -9055,35 +9145,35 @@
         <v>46265</v>
       </c>
       <c r="G80" t="n">
-        <v>0.01023196421218886</v>
+        <v>0.005219350133194078</v>
       </c>
       <c r="H80" t="n">
         <v>0.01082559188004661</v>
       </c>
       <c r="I80" t="n">
-        <v>-0.0005936276678577546</v>
+        <v>-0.005606241746852536</v>
       </c>
       <c r="J80" t="n">
-        <v>0.9451644146171897</v>
+        <v>0.4821306946564481</v>
       </c>
       <c r="K80" t="n">
-        <v>-0.007024523465815835</v>
+        <v>-0.06456129582370584</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Tivio Top Gestor HY</t>
+          <t>BV Top Gestor Crédito Privado</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>TIVIO TOP GESTOR HY FIF RL</t>
+          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -9100,35 +9190,35 @@
         <v>46022</v>
       </c>
       <c r="G81" t="n">
-        <v>0.1091887763786945</v>
+        <v>0.09822271466718724</v>
       </c>
       <c r="H81" t="n">
         <v>0.1051127846901438</v>
       </c>
       <c r="I81" t="n">
-        <v>0.004075991688550662</v>
+        <v>-0.006890070022956607</v>
       </c>
       <c r="J81" t="n">
-        <v>1.038777316199605</v>
+        <v>0.9344506946203789</v>
       </c>
       <c r="K81" t="n">
-        <v>0.004973518048338343</v>
+        <v>-0.008392753749412729</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Tivio Top Gestor HY</t>
+          <t>BV Top Gestor Crédito Privado</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>TIVIO TOP GESTOR HY FIF RL</t>
+          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -9145,35 +9235,35 @@
         <v>45930</v>
       </c>
       <c r="G82" t="n">
-        <v>0.1532058020745011</v>
+        <v>0.1373601954243717</v>
       </c>
       <c r="H82" t="n">
         <v>0.1447903912030524</v>
       </c>
       <c r="I82" t="n">
-        <v>0.008415410871448703</v>
+        <v>-0.007430195778680648</v>
       </c>
       <c r="J82" t="n">
-        <v>1.058121335273188</v>
+        <v>0.9486830878973134</v>
       </c>
       <c r="K82" t="n">
-        <v>0.007380444394986974</v>
+        <v>-0.006516216027085298</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Tivio Top Gestor HY</t>
+          <t>BV Top Gestor Crédito Privado</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>TIVIO TOP GESTOR HY FIF RL</t>
+          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -9187,28 +9277,38 @@
         </is>
       </c>
       <c r="F83" s="1" t="n">
-        <v>45813</v>
-      </c>
-      <c r="G83" t="inlineStr"/>
-      <c r="H83" t="inlineStr"/>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
+        <v>45561</v>
+      </c>
+      <c r="G83" t="n">
+        <v>0.2920431856569192</v>
+      </c>
+      <c r="H83" t="n">
+        <v>0.2980670513506256</v>
+      </c>
+      <c r="I83" t="n">
+        <v>-0.006023865693706387</v>
+      </c>
+      <c r="J83" t="n">
+        <v>0.9797902328807878</v>
+      </c>
+      <c r="K83" t="n">
+        <v>-0.002327632629077092</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Tivio Top Gestor HY</t>
+          <t>BV Top Gestor Crédito Privado</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>TIVIO TOP GESTOR HY FIF RL</t>
+          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -9222,28 +9322,38 @@
         </is>
       </c>
       <c r="F84" s="1" t="n">
-        <v>45813</v>
-      </c>
-      <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr"/>
-      <c r="I84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr"/>
+        <v>45195</v>
+      </c>
+      <c r="G84" t="n">
+        <v>0.4695527796319496</v>
+      </c>
+      <c r="H84" t="n">
+        <v>0.4424561999402108</v>
+      </c>
+      <c r="I84" t="n">
+        <v>0.02709657969173884</v>
+      </c>
+      <c r="J84" t="n">
+        <v>1.06124127019895</v>
+      </c>
+      <c r="K84" t="n">
+        <v>0.006231139290297394</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Tivio Top Gestor HY</t>
+          <t>BV Top Gestor Crédito Privado</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>TIVIO TOP GESTOR HY FIF RL</t>
+          <t>BV TOP GESTOR CRED PRIV FC FIM</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -9257,38 +9367,38 @@
         </is>
       </c>
       <c r="F85" s="1" t="n">
-        <v>45813</v>
+        <v>44706</v>
       </c>
       <c r="G85" t="n">
-        <v>0.2152430848</v>
+        <v>0.7203075669000001</v>
       </c>
       <c r="H85" t="n">
-        <v>0.1976126726386125</v>
+        <v>0.7084789393875421</v>
       </c>
       <c r="I85" t="n">
-        <v>0.0176304121613875</v>
+        <v>0.01182862751245795</v>
       </c>
       <c r="J85" t="n">
-        <v>1.089217011874686</v>
+        <v>1.016695806826218</v>
       </c>
       <c r="K85" t="n">
-        <v>0.01112061570541045</v>
+        <v>0.001593489935187264</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>BV Top Gestor RF Ativo</t>
+          <t>Tivio Top Gestor HY</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
+          <t>TIVIO TOP GESTOR HY FIF RL</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -9305,35 +9415,35 @@
         <v>46265</v>
       </c>
       <c r="G86" t="n">
-        <v>0.009832721928012766</v>
+        <v>0.01023196421218886</v>
       </c>
       <c r="H86" t="n">
         <v>0.01082559188004661</v>
       </c>
       <c r="I86" t="n">
-        <v>-0.000992869952033848</v>
+        <v>-0.0005936276678577546</v>
       </c>
       <c r="J86" t="n">
-        <v>0.9082849267702513</v>
+        <v>0.9451644146171897</v>
       </c>
       <c r="K86" t="n">
-        <v>-0.01172337186485095</v>
+        <v>-0.007024523465815835</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>BV Top Gestor RF Ativo</t>
+          <t>Tivio Top Gestor HY</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
+          <t>TIVIO TOP GESTOR HY FIF RL</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -9350,35 +9460,35 @@
         <v>46022</v>
       </c>
       <c r="G87" t="n">
-        <v>0.09190461218917045</v>
+        <v>0.1091887763786945</v>
       </c>
       <c r="H87" t="n">
         <v>0.1051127846901438</v>
       </c>
       <c r="I87" t="n">
-        <v>-0.01320817250097339</v>
+        <v>0.004075991688550662</v>
       </c>
       <c r="J87" t="n">
-        <v>0.8743428542977999</v>
+        <v>1.038777316199605</v>
       </c>
       <c r="K87" t="n">
-        <v>-0.01607272996257303</v>
+        <v>0.004973518048338343</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>BV Top Gestor RF Ativo</t>
+          <t>Tivio Top Gestor HY</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
+          <t>TIVIO TOP GESTOR HY FIF RL</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -9395,35 +9505,35 @@
         <v>45930</v>
       </c>
       <c r="G88" t="n">
-        <v>0.129702412726495</v>
+        <v>0.1532058020745011</v>
       </c>
       <c r="H88" t="n">
         <v>0.1447903912030524</v>
       </c>
       <c r="I88" t="n">
-        <v>-0.01508797847655741</v>
+        <v>0.008415410871448703</v>
       </c>
       <c r="J88" t="n">
-        <v>0.8957943386215581</v>
+        <v>1.058121335273188</v>
       </c>
       <c r="K88" t="n">
-        <v>-0.01323184628895746</v>
+        <v>0.007380444394986974</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>BV Top Gestor RF Ativo</t>
+          <t>Tivio Top Gestor HY</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
+          <t>TIVIO TOP GESTOR HY FIF RL</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -9437,38 +9547,28 @@
         </is>
       </c>
       <c r="F89" s="1" t="n">
-        <v>45561</v>
-      </c>
-      <c r="G89" t="n">
-        <v>0.270242572217682</v>
-      </c>
-      <c r="H89" t="n">
-        <v>0.2980670513506256</v>
-      </c>
-      <c r="I89" t="n">
-        <v>-0.02782447913294361</v>
-      </c>
-      <c r="J89" t="n">
-        <v>0.906650268767168</v>
-      </c>
-      <c r="K89" t="n">
-        <v>-0.01079702351532119</v>
-      </c>
+        <v>45813</v>
+      </c>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>BV Top Gestor RF Ativo</t>
+          <t>Tivio Top Gestor HY</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
+          <t>TIVIO TOP GESTOR HY FIF RL</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -9482,7 +9582,7 @@
         </is>
       </c>
       <c r="F90" s="1" t="n">
-        <v>45198</v>
+        <v>45813</v>
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr"/>
@@ -9493,17 +9593,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>BV Top Gestor RF Ativo</t>
+          <t>Tivio Top Gestor HY</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
+          <t>TIVIO TOP GESTOR HY FIF RL</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -9517,43 +9617,43 @@
         </is>
       </c>
       <c r="F91" s="1" t="n">
-        <v>45198</v>
+        <v>45813</v>
       </c>
       <c r="G91" t="n">
-        <v>0.399945644</v>
+        <v>0.2152430848</v>
       </c>
       <c r="H91" t="n">
-        <v>0.4404121868646469</v>
+        <v>0.1976126726386125</v>
       </c>
       <c r="I91" t="n">
-        <v>-0.0404665428646469</v>
+        <v>0.0176304121613875</v>
       </c>
       <c r="J91" t="n">
-        <v>0.9081166596393855</v>
+        <v>1.089217011874686</v>
       </c>
       <c r="K91" t="n">
-        <v>-0.009503710662674081</v>
+        <v>0.01112061570541045</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Tivio Top Manager Global</t>
+          <t>BV Top Gestor RF Ativo</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
+          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>MSCI ACWI</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -9565,40 +9665,40 @@
         <v>46265</v>
       </c>
       <c r="G92" t="n">
-        <v>0.001361630876498987</v>
+        <v>0.009832721928012766</v>
       </c>
       <c r="H92" t="n">
-        <v>-0.01270714044827159</v>
+        <v>0.01082559188004661</v>
       </c>
       <c r="I92" t="n">
-        <v>0.01406877132477058</v>
+        <v>-0.000992869952033848</v>
       </c>
       <c r="J92" t="n">
-        <v>-0.1071547829381389</v>
+        <v>0.9082849267702513</v>
       </c>
       <c r="K92" t="n">
-        <v>0.1850574526325846</v>
+        <v>-0.01172337186485095</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Tivio Top Manager Global</t>
+          <t>BV Top Gestor RF Ativo</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
+          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>MSCI ACWI</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -9610,40 +9710,40 @@
         <v>46022</v>
       </c>
       <c r="G93" t="n">
-        <v>0.06432757633456698</v>
+        <v>0.09190461218917045</v>
       </c>
       <c r="H93" t="n">
-        <v>0.05306746240220672</v>
+        <v>0.1051127846901438</v>
       </c>
       <c r="I93" t="n">
-        <v>0.01126011393236026</v>
+        <v>-0.01320817250097339</v>
       </c>
       <c r="J93" t="n">
-        <v>1.212184894898838</v>
+        <v>0.8743428542977999</v>
       </c>
       <c r="K93" t="n">
-        <v>0.01443610338441359</v>
+        <v>-0.01607272996257303</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Tivio Top Manager Global</t>
+          <t>BV Top Gestor RF Ativo</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
+          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>MSCI ACWI</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -9655,40 +9755,40 @@
         <v>45930</v>
       </c>
       <c r="G94" t="n">
-        <v>0.1275037236060828</v>
+        <v>0.129702412726495</v>
       </c>
       <c r="H94" t="n">
-        <v>0.1224734191492385</v>
+        <v>0.1447903912030524</v>
       </c>
       <c r="I94" t="n">
-        <v>0.00503030445684427</v>
+        <v>-0.01508797847655741</v>
       </c>
       <c r="J94" t="n">
-        <v>1.041072622057809</v>
+        <v>0.8957943386215581</v>
       </c>
       <c r="K94" t="n">
-        <v>0.004499340868773238</v>
+        <v>-0.01323184628895746</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Tivio Top Manager Global</t>
+          <t>BV Top Gestor RF Ativo</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
+          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>MSCI ACWI</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -9700,40 +9800,40 @@
         <v>45561</v>
       </c>
       <c r="G95" t="n">
-        <v>0.2322960043521065</v>
+        <v>0.270242572217682</v>
       </c>
       <c r="H95" t="n">
-        <v>0.2701236930973472</v>
+        <v>0.2980670513506256</v>
       </c>
       <c r="I95" t="n">
-        <v>-0.03782768874524067</v>
+        <v>-0.02782447913294361</v>
       </c>
       <c r="J95" t="n">
-        <v>0.859961603843435</v>
+        <v>0.906650268767168</v>
       </c>
       <c r="K95" t="n">
-        <v>-0.01503350245593893</v>
+        <v>-0.01079702351532119</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Tivio Top Manager Global</t>
+          <t>BV Top Gestor RF Ativo</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
+          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>MSCI ACWI</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -9742,43 +9842,33 @@
         </is>
       </c>
       <c r="F96" s="1" t="n">
-        <v>45195</v>
-      </c>
-      <c r="G96" t="n">
-        <v>0.6834526851150575</v>
-      </c>
-      <c r="H96" t="n">
-        <v>0.8062550197741138</v>
-      </c>
-      <c r="I96" t="n">
-        <v>-0.1228023346590563</v>
-      </c>
-      <c r="J96" t="n">
-        <v>0.8476879750857719</v>
-      </c>
-      <c r="K96" t="n">
-        <v>-0.02322669426482782</v>
-      </c>
+        <v>45198</v>
+      </c>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Tivio Top Manager Global</t>
+          <t>BV Top Gestor RF Ativo</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
+          <t>BV TOP GESTOR RF ATIVO FC FI LP</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>MSCI ACWI</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -9787,43 +9877,43 @@
         </is>
       </c>
       <c r="F97" s="1" t="n">
-        <v>41978</v>
+        <v>45198</v>
       </c>
       <c r="G97" t="n">
-        <v>4.0049474242</v>
+        <v>0.399945644</v>
       </c>
       <c r="H97" t="n">
-        <v>4.3466175936699</v>
+        <v>0.4404121868646469</v>
       </c>
       <c r="I97" t="n">
-        <v>-0.3416701694699</v>
+        <v>-0.0404665428646469</v>
       </c>
       <c r="J97" t="n">
-        <v>0.9213940122159622</v>
+        <v>0.9081166596393855</v>
       </c>
       <c r="K97" t="n">
-        <v>-0.005600653521803611</v>
+        <v>-0.009503710662674081</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Tivio RF Ativo Longo Prazo</t>
+          <t>Tivio Top Manager Global</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
+          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>MSCI ACWI</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -9835,40 +9925,40 @@
         <v>46265</v>
       </c>
       <c r="G98" t="n">
-        <v>0.0155703610771285</v>
+        <v>0.001361630876498987</v>
       </c>
       <c r="H98" t="n">
-        <v>0.01082559188004661</v>
+        <v>-0.01270714044827159</v>
       </c>
       <c r="I98" t="n">
-        <v>0.004744769197081888</v>
+        <v>0.01406877132477058</v>
       </c>
       <c r="J98" t="n">
-        <v>1.43829189661466</v>
+        <v>-0.1071547829381389</v>
       </c>
       <c r="K98" t="n">
-        <v>0.05780463920320189</v>
+        <v>0.1850574526325846</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Tivio RF Ativo Longo Prazo</t>
+          <t>Tivio Top Manager Global</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
+          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>MSCI ACWI</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -9880,40 +9970,40 @@
         <v>46022</v>
       </c>
       <c r="G99" t="n">
-        <v>0.08726921494637052</v>
+        <v>0.06432757633456698</v>
       </c>
       <c r="H99" t="n">
-        <v>0.1051127846901438</v>
+        <v>0.05306746240220672</v>
       </c>
       <c r="I99" t="n">
-        <v>-0.01784356974377332</v>
+        <v>0.01126011393236026</v>
       </c>
       <c r="J99" t="n">
-        <v>0.8302435826776601</v>
+        <v>1.212184894898838</v>
       </c>
       <c r="K99" t="n">
-        <v>-0.02169748156471796</v>
+        <v>0.01443610338441359</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Tivio RF Ativo Longo Prazo</t>
+          <t>Tivio Top Manager Global</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
+          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>MSCI ACWI</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -9925,40 +10015,40 @@
         <v>45930</v>
       </c>
       <c r="G100" t="n">
-        <v>0.1254024677775691</v>
+        <v>0.1275037236060828</v>
       </c>
       <c r="H100" t="n">
-        <v>0.1447903912030524</v>
+        <v>0.1224734191492385</v>
       </c>
       <c r="I100" t="n">
-        <v>-0.01938792342548323</v>
+        <v>0.00503030445684427</v>
       </c>
       <c r="J100" t="n">
-        <v>0.866096615497821</v>
+        <v>1.041072622057809</v>
       </c>
       <c r="K100" t="n">
-        <v>-0.01700268091430945</v>
+        <v>0.004499340868773238</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Tivio RF Ativo Longo Prazo</t>
+          <t>Tivio Top Manager Global</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
+          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>MSCI ACWI</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -9970,40 +10060,40 @@
         <v>45561</v>
       </c>
       <c r="G101" t="n">
-        <v>0.2544840968352924</v>
+        <v>0.2322960043521065</v>
       </c>
       <c r="H101" t="n">
-        <v>0.2980670513506256</v>
+        <v>0.2701236930973472</v>
       </c>
       <c r="I101" t="n">
-        <v>-0.04358295451533323</v>
+        <v>-0.03782768874524067</v>
       </c>
       <c r="J101" t="n">
-        <v>0.853781374634175</v>
+        <v>0.859961603843435</v>
       </c>
       <c r="K101" t="n">
-        <v>-0.01696433769312999</v>
+        <v>-0.01503350245593893</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Tivio RF Ativo Longo Prazo</t>
+          <t>Tivio Top Manager Global</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
+          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>MSCI ACWI</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -10015,40 +10105,40 @@
         <v>45195</v>
       </c>
       <c r="G102" t="n">
-        <v>0.3777127110637792</v>
+        <v>0.6834526851150575</v>
       </c>
       <c r="H102" t="n">
-        <v>0.4424561999402108</v>
+        <v>0.8062550197741138</v>
       </c>
       <c r="I102" t="n">
-        <v>-0.06474348887643155</v>
+        <v>-0.1228023346590563</v>
       </c>
       <c r="J102" t="n">
-        <v>0.8536725468302165</v>
+        <v>0.8476879750857719</v>
       </c>
       <c r="K102" t="n">
-        <v>-0.01521096373123265</v>
+        <v>-0.02322669426482782</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Tivio RF Ativo Longo Prazo</t>
+          <t>Tivio Top Manager Global</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
+          <t>TIVIO TOP MANAG GLOBAL ALLOC FIF AÇÕES</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>MSCI ACWI</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -10057,38 +10147,38 @@
         </is>
       </c>
       <c r="F103" s="1" t="n">
-        <v>36392</v>
+        <v>41978</v>
       </c>
       <c r="G103" t="n">
-        <v>22.17376941860116</v>
+        <v>4.0049474242</v>
       </c>
       <c r="H103" t="n">
-        <v>21.93717469453623</v>
+        <v>4.3466175936699</v>
       </c>
       <c r="I103" t="n">
-        <v>0.2365947240649326</v>
+        <v>-0.3416701694699</v>
       </c>
       <c r="J103" t="n">
-        <v>1.010785104616223</v>
+        <v>0.9213940122159622</v>
       </c>
       <c r="K103" t="n">
-        <v>0.0003791455748300976</v>
+        <v>-0.005600653521803611</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Tivio Prev Low Vol Itaú</t>
+          <t>Tivio RF Ativo Longo Prazo</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
+          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -10105,35 +10195,35 @@
         <v>46265</v>
       </c>
       <c r="G104" t="n">
-        <v>0.01528942439290315</v>
+        <v>0.0155703610771285</v>
       </c>
       <c r="H104" t="n">
         <v>0.01082559188004661</v>
       </c>
       <c r="I104" t="n">
-        <v>0.004463832512856536</v>
+        <v>0.004744769197081888</v>
       </c>
       <c r="J104" t="n">
-        <v>1.412340735021069</v>
+        <v>1.43829189661466</v>
       </c>
       <c r="K104" t="n">
-        <v>0.05429853764221493</v>
+        <v>0.05780463920320189</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Tivio Prev Low Vol Itaú</t>
+          <t>Tivio RF Ativo Longo Prazo</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
+          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -10150,35 +10240,35 @@
         <v>46022</v>
       </c>
       <c r="G105" t="n">
-        <v>0.1025226903097796</v>
+        <v>0.08726921494637052</v>
       </c>
       <c r="H105" t="n">
         <v>0.1051127846901438</v>
       </c>
       <c r="I105" t="n">
-        <v>-0.002590094380364283</v>
+        <v>-0.01784356974377332</v>
       </c>
       <c r="J105" t="n">
-        <v>0.9753589024589209</v>
+        <v>0.8302435826776601</v>
       </c>
       <c r="K105" t="n">
-        <v>-0.003157118560559224</v>
+        <v>-0.02169748156471796</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Tivio Prev Low Vol Itaú</t>
+          <t>Tivio RF Ativo Longo Prazo</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
+          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -10195,35 +10285,35 @@
         <v>45930</v>
       </c>
       <c r="G106" t="n">
-        <v>0.1410909765555666</v>
+        <v>0.1254024677775691</v>
       </c>
       <c r="H106" t="n">
         <v>0.1447903912030524</v>
       </c>
       <c r="I106" t="n">
-        <v>-0.003699414647485799</v>
+        <v>-0.01938792342548323</v>
       </c>
       <c r="J106" t="n">
-        <v>0.9744498608177818</v>
+        <v>0.866096615497821</v>
       </c>
       <c r="K106" t="n">
-        <v>-0.00324437507950126</v>
+        <v>-0.01700268091430945</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Tivio Prev Low Vol Itaú</t>
+          <t>Tivio RF Ativo Longo Prazo</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
+          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -10240,35 +10330,35 @@
         <v>45561</v>
       </c>
       <c r="G107" t="n">
-        <v>0.2822773175556004</v>
+        <v>0.2544840968352924</v>
       </c>
       <c r="H107" t="n">
         <v>0.2980670513506256</v>
       </c>
       <c r="I107" t="n">
-        <v>-0.01578973379502524</v>
+        <v>-0.04358295451533323</v>
       </c>
       <c r="J107" t="n">
-        <v>0.9470262354611907</v>
+        <v>0.853781374634175</v>
       </c>
       <c r="K107" t="n">
-        <v>-0.00611271794908208</v>
+        <v>-0.01696433769312999</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Tivio Prev Low Vol Itaú</t>
+          <t>Tivio RF Ativo Longo Prazo</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
+          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -10285,35 +10375,35 @@
         <v>45195</v>
       </c>
       <c r="G108" t="n">
-        <v>0.4184670843779219</v>
+        <v>0.3777127110637792</v>
       </c>
       <c r="H108" t="n">
         <v>0.4424561999402108</v>
       </c>
       <c r="I108" t="n">
-        <v>-0.02398911556228889</v>
+        <v>-0.06474348887643155</v>
       </c>
       <c r="J108" t="n">
-        <v>0.9457819427877142</v>
+        <v>0.8536725468302165</v>
       </c>
       <c r="K108" t="n">
-        <v>-0.005581961690141801</v>
+        <v>-0.01521096373123265</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Tivio Prev Low Vol Itaú</t>
+          <t>Tivio RF Ativo Longo Prazo</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
+          <t>TIVIO RF ATIVO LONGO PRAZO FI</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -10327,38 +10417,38 @@
         </is>
       </c>
       <c r="F109" s="1" t="n">
-        <v>44917</v>
+        <v>36392</v>
       </c>
       <c r="G109" t="n">
-        <v>0.56223</v>
+        <v>22.17376941860116</v>
       </c>
       <c r="H109" t="n">
-        <v>0.5882420554079393</v>
+        <v>21.93717469453623</v>
       </c>
       <c r="I109" t="n">
-        <v>-0.02601205540793927</v>
+        <v>0.2365947240649326</v>
       </c>
       <c r="J109" t="n">
-        <v>0.9557800140795778</v>
+        <v>1.010785104616223</v>
       </c>
       <c r="K109" t="n">
-        <v>-0.004389281550695734</v>
+        <v>0.0003791455748300976</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus CDI</t>
+          <t>Tivio Prev Low Vol Itaú</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
+          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -10375,35 +10465,35 @@
         <v>46265</v>
       </c>
       <c r="G110" t="n">
-        <v>-0.001462081025388806</v>
+        <v>0.01528942439290315</v>
       </c>
       <c r="H110" t="n">
         <v>0.01082559188004661</v>
       </c>
       <c r="I110" t="n">
-        <v>-0.01228767290543542</v>
+        <v>0.004463832512856536</v>
       </c>
       <c r="J110" t="n">
-        <v>-0.1350578371685771</v>
+        <v>1.412340735021069</v>
       </c>
       <c r="K110" t="n">
-        <v>-0.1365046674965383</v>
+        <v>0.05429853764221493</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus CDI</t>
+          <t>Tivio Prev Low Vol Itaú</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
+          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -10420,35 +10510,35 @@
         <v>46022</v>
       </c>
       <c r="G111" t="n">
-        <v>0.08638432471204283</v>
+        <v>0.1025226903097796</v>
       </c>
       <c r="H111" t="n">
         <v>0.1051127846901438</v>
       </c>
       <c r="I111" t="n">
-        <v>-0.01872845997810102</v>
+        <v>-0.002590094380364283</v>
       </c>
       <c r="J111" t="n">
-        <v>0.8218250992654261</v>
+        <v>0.9753589024589209</v>
       </c>
       <c r="K111" t="n">
-        <v>-0.0227702919562276</v>
+        <v>-0.003157118560559224</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus CDI</t>
+          <t>Tivio Prev Low Vol Itaú</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
+          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -10462,28 +10552,38 @@
         </is>
       </c>
       <c r="F112" s="1" t="n">
-        <v>45950</v>
-      </c>
-      <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr"/>
-      <c r="I112" t="inlineStr"/>
-      <c r="J112" t="inlineStr"/>
-      <c r="K112" t="inlineStr"/>
+        <v>45930</v>
+      </c>
+      <c r="G112" t="n">
+        <v>0.1410909765555666</v>
+      </c>
+      <c r="H112" t="n">
+        <v>0.1447903912030524</v>
+      </c>
+      <c r="I112" t="n">
+        <v>-0.003699414647485799</v>
+      </c>
+      <c r="J112" t="n">
+        <v>0.9744498608177818</v>
+      </c>
+      <c r="K112" t="n">
+        <v>-0.00324437507950126</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus CDI</t>
+          <t>Tivio Prev Low Vol Itaú</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
+          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -10497,28 +10597,38 @@
         </is>
       </c>
       <c r="F113" s="1" t="n">
-        <v>45950</v>
-      </c>
-      <c r="G113" t="inlineStr"/>
-      <c r="H113" t="inlineStr"/>
-      <c r="I113" t="inlineStr"/>
-      <c r="J113" t="inlineStr"/>
-      <c r="K113" t="inlineStr"/>
+        <v>45561</v>
+      </c>
+      <c r="G113" t="n">
+        <v>0.2822773175556004</v>
+      </c>
+      <c r="H113" t="n">
+        <v>0.2980670513506256</v>
+      </c>
+      <c r="I113" t="n">
+        <v>-0.01578973379502524</v>
+      </c>
+      <c r="J113" t="n">
+        <v>0.9470262354611907</v>
+      </c>
+      <c r="K113" t="n">
+        <v>-0.00611271794908208</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus CDI</t>
+          <t>Tivio Prev Low Vol Itaú</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
+          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -10532,28 +10642,38 @@
         </is>
       </c>
       <c r="F114" s="1" t="n">
-        <v>45950</v>
-      </c>
-      <c r="G114" t="inlineStr"/>
-      <c r="H114" t="inlineStr"/>
-      <c r="I114" t="inlineStr"/>
-      <c r="J114" t="inlineStr"/>
-      <c r="K114" t="inlineStr"/>
+        <v>45195</v>
+      </c>
+      <c r="G114" t="n">
+        <v>0.4184670843779219</v>
+      </c>
+      <c r="H114" t="n">
+        <v>0.4424561999402108</v>
+      </c>
+      <c r="I114" t="n">
+        <v>-0.02398911556228889</v>
+      </c>
+      <c r="J114" t="n">
+        <v>0.9457819427877142</v>
+      </c>
+      <c r="K114" t="n">
+        <v>-0.005581961690141801</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus CDI</t>
+          <t>Tivio Prev Low Vol Itaú</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
+          <t>TIVIO PREV LOW VOL ITAÚ I FIF CIC MULT RL - Expandida</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -10567,43 +10687,43 @@
         </is>
       </c>
       <c r="F115" s="1" t="n">
-        <v>45950</v>
+        <v>44917</v>
       </c>
       <c r="G115" t="n">
-        <v>0.1194341999999999</v>
+        <v>0.56223</v>
       </c>
       <c r="H115" t="n">
-        <v>0.1359909271883835</v>
+        <v>0.5882420554079393</v>
       </c>
       <c r="I115" t="n">
-        <v>-0.01655672718838352</v>
+        <v>-0.02601205540793927</v>
       </c>
       <c r="J115" t="n">
-        <v>0.8782512368237032</v>
+        <v>0.9557800140795778</v>
       </c>
       <c r="K115" t="n">
-        <v>-0.0154899691480026</v>
+        <v>-0.004389281550695734</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>esplanada</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Tivio Esplanada</t>
+          <t>Tivio Infra Plus CDI</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>IMA-B 5</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -10615,40 +10735,40 @@
         <v>46265</v>
       </c>
       <c r="G116" t="n">
-        <v>0.01003070736812051</v>
+        <v>-0.001462081025388806</v>
       </c>
       <c r="H116" t="n">
-        <v>0.0200519906458918</v>
+        <v>0.01082559188004661</v>
       </c>
       <c r="I116" t="n">
-        <v>-0.0100212832777713</v>
+        <v>-0.01228767290543542</v>
       </c>
       <c r="J116" t="n">
-        <v>0.5002349913910203</v>
+        <v>-0.1350578371685771</v>
       </c>
       <c r="K116" t="n">
-        <v>-0.1117254109753738</v>
+        <v>-0.1365046674965383</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>esplanada</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Tivio Esplanada</t>
+          <t>Tivio Infra Plus CDI</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>IMA-B 5</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -10660,40 +10780,40 @@
         <v>46022</v>
       </c>
       <c r="G117" t="n">
-        <v>0.07172731728642034</v>
+        <v>0.08638432471204283</v>
       </c>
       <c r="H117" t="n">
-        <v>0.1136619152554992</v>
+        <v>0.1051127846901438</v>
       </c>
       <c r="I117" t="n">
-        <v>-0.04193459796907884</v>
+        <v>-0.01872845997810102</v>
       </c>
       <c r="J117" t="n">
-        <v>0.6310584959367033</v>
+        <v>0.8218250992654261</v>
       </c>
       <c r="K117" t="n">
-        <v>-0.05040838364525002</v>
+        <v>-0.0227702919562276</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>esplanada</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Tivio Esplanada</t>
+          <t>Tivio Infra Plus CDI</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>IMA-B 5</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -10702,43 +10822,33 @@
         </is>
       </c>
       <c r="F118" s="1" t="n">
-        <v>45930</v>
-      </c>
-      <c r="G118" t="n">
-        <v>0.09357535556093843</v>
-      </c>
-      <c r="H118" t="n">
-        <v>0.1479693332684646</v>
-      </c>
-      <c r="I118" t="n">
-        <v>-0.05439397770752619</v>
-      </c>
-      <c r="J118" t="n">
-        <v>0.6323969534360354</v>
-      </c>
-      <c r="K118" t="n">
-        <v>-0.0475669929009177</v>
-      </c>
+        <v>45950</v>
+      </c>
+      <c r="G118" t="inlineStr"/>
+      <c r="H118" t="inlineStr"/>
+      <c r="I118" t="inlineStr"/>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>esplanada</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Tivio Esplanada</t>
+          <t>Tivio Infra Plus CDI</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>IMA-B 5</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -10747,7 +10857,7 @@
         </is>
       </c>
       <c r="F119" s="1" t="n">
-        <v>45586</v>
+        <v>45950</v>
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr"/>
@@ -10758,22 +10868,22 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>esplanada</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Tivio Esplanada</t>
+          <t>Tivio Infra Plus CDI</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>IMA-B 5</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -10782,7 +10892,7 @@
         </is>
       </c>
       <c r="F120" s="1" t="n">
-        <v>45586</v>
+        <v>45950</v>
       </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="inlineStr"/>
@@ -10793,22 +10903,22 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>esplanada</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Tivio Esplanada</t>
+          <t>Tivio Infra Plus CDI</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+          <t>TIVIO INFRA PLUS CDI 30 FIF CIC RF - Expandida</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>IMA-B 5</t>
+          <t>CDI</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -10817,43 +10927,43 @@
         </is>
       </c>
       <c r="F121" s="1" t="n">
-        <v>45586</v>
+        <v>45950</v>
       </c>
       <c r="G121" t="n">
-        <v>0.2135222000000001</v>
+        <v>0.1194341999999999</v>
       </c>
       <c r="H121" t="n">
-        <v>0.2465452463189715</v>
+        <v>0.1359909271883835</v>
       </c>
       <c r="I121" t="n">
-        <v>-0.03302304631897135</v>
+        <v>-0.01655672718838352</v>
       </c>
       <c r="J121" t="n">
-        <v>0.8660568523951693</v>
+        <v>0.8782512368237032</v>
       </c>
       <c r="K121" t="n">
-        <v>-0.01382518449086667</v>
+        <v>-0.0154899691480026</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>legacy</t>
+          <t>esplanada</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Tivio Legacy Prev</t>
+          <t>Tivio Esplanada</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>IMA-B 5</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -10865,40 +10975,40 @@
         <v>46265</v>
       </c>
       <c r="G122" t="n">
-        <v>0.01025992096101835</v>
+        <v>0.01003070736812051</v>
       </c>
       <c r="H122" t="n">
-        <v>0.01082559188004661</v>
+        <v>0.0200519906458918</v>
       </c>
       <c r="I122" t="n">
-        <v>-0.0005656709190282605</v>
+        <v>-0.0100212832777713</v>
       </c>
       <c r="J122" t="n">
-        <v>0.9477468830068416</v>
+        <v>0.5002349913910203</v>
       </c>
       <c r="K122" t="n">
-        <v>-0.006694722873975767</v>
+        <v>-0.1117254109753738</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>legacy</t>
+          <t>esplanada</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Tivio Legacy Prev</t>
+          <t>Tivio Esplanada</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>IMA-B 5</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -10910,40 +11020,40 @@
         <v>46022</v>
       </c>
       <c r="G123" t="n">
-        <v>0.1002856499041807</v>
+        <v>0.07172731728642034</v>
       </c>
       <c r="H123" t="n">
-        <v>0.1051127846901438</v>
+        <v>0.1136619152554992</v>
       </c>
       <c r="I123" t="n">
-        <v>-0.004827134785963194</v>
+        <v>-0.04193459796907884</v>
       </c>
       <c r="J123" t="n">
-        <v>0.9540766158922263</v>
+        <v>0.6310584959367033</v>
       </c>
       <c r="K123" t="n">
-        <v>-0.00588181858317427</v>
+        <v>-0.05040838364525002</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>legacy</t>
+          <t>esplanada</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Tivio Legacy Prev</t>
+          <t>Tivio Esplanada</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>IMA-B 5</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -10955,40 +11065,40 @@
         <v>45930</v>
       </c>
       <c r="G124" t="n">
-        <v>0.1394310574216069</v>
+        <v>0.09357535556093843</v>
       </c>
       <c r="H124" t="n">
-        <v>0.1447903912030524</v>
+        <v>0.1479693332684646</v>
       </c>
       <c r="I124" t="n">
-        <v>-0.005359333781445486</v>
+        <v>-0.05439397770752619</v>
       </c>
       <c r="J124" t="n">
-        <v>0.9629855701271667</v>
+        <v>0.6323969534360354</v>
       </c>
       <c r="K124" t="n">
-        <v>-0.004700105358509954</v>
+        <v>-0.0475669929009177</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>legacy</t>
+          <t>esplanada</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Tivio Legacy Prev</t>
+          <t>Tivio Esplanada</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>IMA-B 5</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -10997,43 +11107,33 @@
         </is>
       </c>
       <c r="F125" s="1" t="n">
-        <v>45561</v>
-      </c>
-      <c r="G125" t="n">
-        <v>0.288834593654415</v>
-      </c>
-      <c r="H125" t="n">
-        <v>0.2980670513506256</v>
-      </c>
-      <c r="I125" t="n">
-        <v>-0.009232457696210616</v>
-      </c>
-      <c r="J125" t="n">
-        <v>0.9690255677225116</v>
-      </c>
-      <c r="K125" t="n">
-        <v>-0.00356964896216394</v>
-      </c>
+        <v>45586</v>
+      </c>
+      <c r="G125" t="inlineStr"/>
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>legacy</t>
+          <t>esplanada</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Tivio Legacy Prev</t>
+          <t>Tivio Esplanada</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>CDI</t>
+          <t>IMA-B 5</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -11042,66 +11142,326 @@
         </is>
       </c>
       <c r="F126" s="1" t="n">
-        <v>45195</v>
-      </c>
-      <c r="G126" t="n">
-        <v>0.4630786945344103</v>
-      </c>
-      <c r="H126" t="n">
-        <v>0.4424561999402108</v>
-      </c>
-      <c r="I126" t="n">
-        <v>0.02062249459419951</v>
-      </c>
-      <c r="J126" t="n">
-        <v>1.046609121076812</v>
-      </c>
-      <c r="K126" t="n">
-        <v>0.004749361817451225</v>
-      </c>
+        <v>45586</v>
+      </c>
+      <c r="G126" t="inlineStr"/>
+      <c r="H126" t="inlineStr"/>
+      <c r="I126" t="inlineStr"/>
+      <c r="J126" t="inlineStr"/>
+      <c r="K126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
+          <t>esplanada</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Tivio Esplanada</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>TIVIO ESPLANADA FIF RF INFRA RL</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>IMA-B 5</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>inicio</t>
+        </is>
+      </c>
+      <c r="F127" s="1" t="n">
+        <v>45586</v>
+      </c>
+      <c r="G127" t="n">
+        <v>0.2135222000000001</v>
+      </c>
+      <c r="H127" t="n">
+        <v>0.2465452463189715</v>
+      </c>
+      <c r="I127" t="n">
+        <v>-0.03302304631897135</v>
+      </c>
+      <c r="J127" t="n">
+        <v>0.8660568523951693</v>
+      </c>
+      <c r="K127" t="n">
+        <v>-0.01382518449086667</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
           <t>legacy</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr">
+      <c r="B128" t="inlineStr">
         <is>
           <t>Tivio Legacy Prev</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr">
+      <c r="C128" t="inlineStr">
         <is>
           <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
         </is>
       </c>
-      <c r="D127" t="inlineStr">
+      <c r="D128" t="inlineStr">
         <is>
           <t>CDI</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr">
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="F128" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="G128" t="n">
+        <v>0.01025992096101835</v>
+      </c>
+      <c r="H128" t="n">
+        <v>0.01082559188004661</v>
+      </c>
+      <c r="I128" t="n">
+        <v>-0.0005656709190282605</v>
+      </c>
+      <c r="J128" t="n">
+        <v>0.9477468830068416</v>
+      </c>
+      <c r="K128" t="n">
+        <v>-0.006694722873975767</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>legacy</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="F129" s="1" t="n">
+        <v>46022</v>
+      </c>
+      <c r="G129" t="n">
+        <v>0.1002856499041807</v>
+      </c>
+      <c r="H129" t="n">
+        <v>0.1051127846901438</v>
+      </c>
+      <c r="I129" t="n">
+        <v>-0.004827134785963194</v>
+      </c>
+      <c r="J129" t="n">
+        <v>0.9540766158922263</v>
+      </c>
+      <c r="K129" t="n">
+        <v>-0.00588181858317427</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>legacy</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>12m</t>
+        </is>
+      </c>
+      <c r="F130" s="1" t="n">
+        <v>45930</v>
+      </c>
+      <c r="G130" t="n">
+        <v>0.1394310574216069</v>
+      </c>
+      <c r="H130" t="n">
+        <v>0.1447903912030524</v>
+      </c>
+      <c r="I130" t="n">
+        <v>-0.005359333781445486</v>
+      </c>
+      <c r="J130" t="n">
+        <v>0.9629855701271667</v>
+      </c>
+      <c r="K130" t="n">
+        <v>-0.004700105358509954</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>legacy</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>24m</t>
+        </is>
+      </c>
+      <c r="F131" s="1" t="n">
+        <v>45561</v>
+      </c>
+      <c r="G131" t="n">
+        <v>0.288834593654415</v>
+      </c>
+      <c r="H131" t="n">
+        <v>0.2980670513506256</v>
+      </c>
+      <c r="I131" t="n">
+        <v>-0.009232457696210616</v>
+      </c>
+      <c r="J131" t="n">
+        <v>0.9690255677225116</v>
+      </c>
+      <c r="K131" t="n">
+        <v>-0.00356964896216394</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>legacy</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>36m</t>
+        </is>
+      </c>
+      <c r="F132" s="1" t="n">
+        <v>45195</v>
+      </c>
+      <c r="G132" t="n">
+        <v>0.4630786945344103</v>
+      </c>
+      <c r="H132" t="n">
+        <v>0.4424561999402108</v>
+      </c>
+      <c r="I132" t="n">
+        <v>0.02062249459419951</v>
+      </c>
+      <c r="J132" t="n">
+        <v>1.046609121076812</v>
+      </c>
+      <c r="K132" t="n">
+        <v>0.004749361817451225</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>legacy</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>TIVIO LEGACY PREV FIF CI RF CP RL</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
         <is>
           <t>inicio</t>
         </is>
       </c>
-      <c r="F127" s="1" t="n">
+      <c r="F133" s="1" t="n">
         <v>39674</v>
       </c>
-      <c r="G127" t="n">
+      <c r="G133" t="n">
         <v>4.4092549</v>
       </c>
-      <c r="H127" t="n">
+      <c r="H133" t="n">
         <v>4.604775473331634</v>
       </c>
-      <c r="I127" t="n">
+      <c r="I133" t="n">
         <v>-0.1955205733316348</v>
       </c>
-      <c r="J127" t="n">
+      <c r="J133" t="n">
         <v>0.957539607639073</v>
       </c>
-      <c r="K127" t="n">
+      <c r="K133" t="n">
         <v>-0.001963351321792373</v>
       </c>
     </row>
@@ -11116,7 +11476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -11482,29 +11842,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>hgd30</t>
+          <t>conexaoalt180</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Tivio HGD30</t>
+          <t>Conexão Tivio ALT 180</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>59.889.169/0001-97</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>0,30% a.a.</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>16% do que exceder 100% do CDI</t>
-        </is>
-      </c>
+          <t>60.173.255/0001-88</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>não</t>
@@ -11514,27 +11866,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>hyd60</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Tivio HYD60</t>
+          <t>Tivio HGD30</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>64.111.034/0001-36</t>
+          <t>59.889.169/0001-97</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0,50% a.a.</t>
+          <t>0,30% a.a.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>20% do que exceder 100% do CDI</t>
+          <t>16% do que exceder 100% do CDI</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -11546,27 +11898,27 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>hyd60</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BV Top Gestor Crédito Privado</t>
+          <t>Tivio HYD60</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>36.157.723/0001-46</t>
+          <t>64.111.034/0001-36</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0,25% a.a.</t>
+          <t>0,50% a.a.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Não há</t>
+          <t>20% do que exceder 100% do CDI</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -11578,22 +11930,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Tivio Top Gestor HY</t>
+          <t>BV Top Gestor Crédito Privado</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>61.026.657/0001-12</t>
+          <t>36.157.723/0001-46</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0,35% a.a.</t>
+          <t>0,25% a.a.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -11610,22 +11962,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>BV Top Gestor RF Ativo</t>
+          <t>Tivio Top Gestor HY</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>26.190.911/0001-12</t>
+          <t>61.026.657/0001-12</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0,15% a.a.</t>
+          <t>0,35% a.a.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -11642,22 +11994,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Tivio Top Manager Global</t>
+          <t>BV Top Gestor RF Ativo</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>13.614.712/0001-42</t>
+          <t>26.190.911/0001-12</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0,70% a.a.</t>
+          <t>0,15% a.a.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -11674,27 +12026,27 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Tivio RF Ativo Longo Prazo</t>
+          <t>Tivio Top Manager Global</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>00.836.263/0001-35</t>
+          <t>13.614.712/0001-42</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0,50% a.a.</t>
+          <t>0,70% a.a.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>20% do que exceder 100% do CDI</t>
+          <t>Não há</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -11706,27 +12058,27 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Tivio Prev Low Vol Itaú</t>
+          <t>Tivio RF Ativo Longo Prazo</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>45.512.215/0001-20</t>
+          <t>00.836.263/0001-35</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0,80% a.a.</t>
+          <t>0,50% a.a.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Não há</t>
+          <t>20% do que exceder 100% do CDI</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -11738,22 +12090,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>infrapluscdi</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus CDI</t>
+          <t>Tivio Prev Low Vol Itaú</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>62.791.756/0001-53</t>
+          <t>45.512.215/0001-20</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0,75% a.a.</t>
+          <t>0,80% a.a.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -11770,22 +12122,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>esplanada</t>
+          <t>infrapluscdi</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Tivio Esplanada</t>
+          <t>Tivio Infra Plus CDI</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>54.853.793/0001-10</t>
+          <t>62.791.756/0001-53</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0,475% a.a.</t>
+          <t>0,75% a.a.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -11802,30 +12154,62 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>esplanada</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Tivio Esplanada</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>54.853.793/0001-10</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>0,475% a.a.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Não há</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>legacy</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>Tivio Legacy Prev</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>09.083.848/0001-04</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>0,50% a.a.</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Não há</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>não</t>
         </is>
@@ -11842,7 +12226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -11892,114 +12276,114 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>hgd30</t>
+          <t>conexaoalt180</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>sem cotas de "BRADESCO TIVIO HGD30 PGBL/VGBL" na dados_mensais: a rentabilidade saiu do TIVIO HGD30 FIFE RESP LIMITADA FIF RENDA FIXA CRÉDITO PRIVADO (inclua a classe na planilha para usar a dela)</t>
+          <t>sem carteira na Base Carteira — alocação, carrego e duration mantidos</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>relatorio/bvp</t>
+          <t>—</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>bvp</t>
+          <t>conexaoalt180</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>logo não encontrado em assets/logos (procurei "tivio_bvp")</t>
+          <t>taxa global não encontrada na taxas_global.xlsx</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>relatorio/atuarial</t>
+          <t>relatorio/bvp</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>atuarial</t>
+          <t>bvp</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>relatório não gerado: sem dados nesta edição</t>
+          <t>logo não encontrado em assets/logos (procurei "tivio_bvp")</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>relatorio/credito_privado</t>
+          <t>relatorio/atuarial</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>bvp</t>
+          <t>atuarial</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>logo não encontrado em assets/logos (procurei "tivio_bvp")</t>
+          <t>relatório não gerado: sem dados nesta edição</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>landing/hgd30</t>
+          <t>relatorio/credito_privado</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>hgd30</t>
+          <t>bvp</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): Na atribuição de performance, a carteira de títulos bancários foi a principal re…</t>
+          <t>logo não encontrado em assets/logos (procurei "tivio_bvp")</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>landing/hyd60</t>
+          <t>landing/hgd30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>hyd60</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): - Na parcela de **crédito estruturado**, avanço na **diversificação da carteira*…</t>
+          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): Na atribuição de performance, a carteira de títulos bancários foi a principal re…</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>email/previdencia</t>
+          <t>landing/hyd60</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>hgd30</t>
+          <t>hyd60</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): Na atribuição de performance, a carteira de títulos bancários foi a principal re…</t>
+          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): - Na parcela de **crédito estruturado**, avanço na **diversificação da carteira*…</t>
         </is>
       </c>
     </row>
@@ -12011,36 +12395,36 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>hyd60</t>
+          <t>hgd30</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): - Na parcela de **crédito estruturado**, avanço na **diversificação da carteira*…</t>
+          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): Na atribuição de performance, a carteira de títulos bancários foi a principal re…</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>tivio-email-fundos-credito.html</t>
+          <t>email/previdencia</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>alt180</t>
+          <t>hyd60</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>o texto se refere a "julho" como o mês corrente — a data base é setembro</t>
+          <t>comentário: o texto antes do bloco colado (com HTML) foi ignorado (parece de outro mês): - Na parcela de **crédito estruturado**, avanço na **diversificação da carteira*…</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>tivio-email-fundos-credito.html</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -12050,7 +12434,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Mz', 'Fiagro Sr']</t>
+          <t>o texto se refere a "julho" como o mês corrente — a data base é setembro</t>
         </is>
       </c>
     </row>
@@ -12062,29 +12446,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>alt90</t>
+          <t>alt180</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Sr']</t>
+          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Mz', 'Fiagro Sr']</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>tivio-post-credito-estruturado.html</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>topgestormacro</t>
+          <t>alt90</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>sem dados — rentabilidade e PL mantidos</t>
+          <t>tipos sem nome amigável em fundos.yml (tipo_label): ['Fiagro Sr']</t>
         </is>
       </c>
     </row>
@@ -12096,7 +12480,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>topgestorlongonly</t>
+          <t>topgestormacro</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -12108,15 +12492,32 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>tivio-post-investment-solutions.html</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>topgestorlongonly</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>sem dados — rentabilidade e PL mantidos</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>tivio-central.html</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>tivio-central.html</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>card "Gerador de Relatório de Gestão · Incentivado CDI 30" removido: aponta para "Tivio Incentivado CDI 30 - Relatório de Gestão Mensal.html", que não existe nesta edição</t>
         </is>
@@ -12133,7 +12534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -12590,7 +12991,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>548567</v>
+        <v>548576</v>
       </c>
     </row>
     <row r="31">
@@ -12620,7 +13021,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2093587</v>
+        <v>2093594</v>
       </c>
     </row>
     <row r="33">
@@ -12800,7 +13201,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4829399</v>
+        <v>4829397</v>
       </c>
     </row>
     <row r="45">
@@ -12815,7 +13216,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>422853</v>
+        <v>422842</v>
       </c>
     </row>
     <row r="46">
@@ -12830,7 +13231,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>5454372</v>
+        <v>5454374</v>
       </c>
     </row>
     <row r="47">
@@ -12860,7 +13261,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>16816513</v>
+        <v>16767735</v>
       </c>
     </row>
     <row r="49">
@@ -12875,7 +13276,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>3009396</v>
+        <v>3001219</v>
       </c>
     </row>
     <row r="50">
@@ -12890,7 +13291,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>15593104</v>
+        <v>15541486</v>
       </c>
     </row>
     <row r="51">
@@ -12905,7 +13306,7 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2616247</v>
+        <v>2607970</v>
       </c>
     </row>
     <row r="52">
@@ -12920,7 +13321,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>15041374</v>
+        <v>14979429</v>
       </c>
     </row>
     <row r="53">
@@ -12935,7 +13336,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2467250</v>
+        <v>2456580</v>
       </c>
     </row>
     <row r="54">
@@ -12950,7 +13351,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>25551962</v>
+        <v>25532265</v>
       </c>
     </row>
     <row r="55">
@@ -12965,7 +13366,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2649979</v>
+        <v>2646532</v>
       </c>
     </row>
     <row r="56">
@@ -12980,7 +13381,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>23546223</v>
+        <v>23523584</v>
       </c>
     </row>
     <row r="57">
@@ -12995,7 +13396,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2643349</v>
+        <v>2640656</v>
       </c>
     </row>
     <row r="58">
@@ -13010,7 +13411,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>26316559</v>
+        <v>26287584</v>
       </c>
     </row>
     <row r="59">
@@ -13025,7 +13426,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>4115895</v>
+        <v>4111149</v>
       </c>
     </row>
     <row r="60">
@@ -13040,7 +13441,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>26316813</v>
+        <v>26287842</v>
       </c>
     </row>
     <row r="61">
@@ -13055,7 +13456,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>4116719</v>
+        <v>4111920</v>
       </c>
     </row>
     <row r="62">
@@ -13070,7 +13471,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>26457372</v>
+        <v>26408674</v>
       </c>
     </row>
     <row r="63">
@@ -13085,7 +13486,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>3802493</v>
+        <v>3794820</v>
       </c>
     </row>
     <row r="64">
@@ -13100,7 +13501,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>26317598</v>
+        <v>26255766</v>
       </c>
     </row>
     <row r="65">
@@ -13115,21 +13516,51 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>3976310</v>
+        <v>3994873</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
+          <t>Tivio Conecta - Setembro 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>87884080</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Tivio Conecta - Setembro 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>5085698</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
           <t>index.html</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B68" t="inlineStr">
         <is>
           <t>html</t>
         </is>
       </c>
-      <c r="C66" t="n">
+      <c r="C68" t="n">
         <v>394</v>
       </c>
     </row>

</xml_diff>

<commit_message>
AutomaTivio: gráfico diário dos ALT de volta; Conecta com Fundo Crédito Privado, rentabilidade maior que os cartões, Infra Plus CDI em % do CDI desde o início, painel alinhado ao logo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -13201,7 +13201,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4829397</v>
+        <v>4829395</v>
       </c>
     </row>
     <row r="45">
@@ -13231,7 +13231,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>5454374</v>
+        <v>5454373</v>
       </c>
     </row>
     <row r="47">
@@ -13261,7 +13261,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>16767735</v>
+        <v>16816509</v>
       </c>
     </row>
     <row r="49">
@@ -13276,7 +13276,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>3001219</v>
+        <v>3009396</v>
       </c>
     </row>
     <row r="50">
@@ -13291,7 +13291,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>15541486</v>
+        <v>15593110</v>
       </c>
     </row>
     <row r="51">
@@ -13306,7 +13306,7 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2607970</v>
+        <v>2616247</v>
       </c>
     </row>
     <row r="52">
@@ -13321,7 +13321,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>14979429</v>
+        <v>15041378</v>
       </c>
     </row>
     <row r="53">
@@ -13336,7 +13336,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2456580</v>
+        <v>2467250</v>
       </c>
     </row>
     <row r="54">
@@ -13351,7 +13351,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>25532265</v>
+        <v>25551962</v>
       </c>
     </row>
     <row r="55">
@@ -13366,7 +13366,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2646532</v>
+        <v>2649979</v>
       </c>
     </row>
     <row r="56">
@@ -13381,7 +13381,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>23523584</v>
+        <v>23546226</v>
       </c>
     </row>
     <row r="57">
@@ -13396,7 +13396,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2640656</v>
+        <v>2643349</v>
       </c>
     </row>
     <row r="58">
@@ -13411,7 +13411,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>26287584</v>
+        <v>26316559</v>
       </c>
     </row>
     <row r="59">
@@ -13426,7 +13426,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>4111149</v>
+        <v>4115895</v>
       </c>
     </row>
     <row r="60">
@@ -13441,7 +13441,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>26287842</v>
+        <v>26316814</v>
       </c>
     </row>
     <row r="61">
@@ -13456,7 +13456,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>4111920</v>
+        <v>4116719</v>
       </c>
     </row>
     <row r="62">
@@ -13471,7 +13471,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>26408674</v>
+        <v>26457372</v>
       </c>
     </row>
     <row r="63">
@@ -13486,7 +13486,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>3794820</v>
+        <v>3802493</v>
       </c>
     </row>
     <row r="64">
@@ -13501,7 +13501,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>26255766</v>
+        <v>26317597</v>
       </c>
     </row>
     <row r="65">
@@ -13516,7 +13516,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>3994873</v>
+        <v>3976310</v>
       </c>
     </row>
     <row r="66">
@@ -13531,7 +13531,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>87884080</v>
+        <v>87883521</v>
       </c>
     </row>
     <row r="67">
@@ -13546,7 +13546,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>5085698</v>
+        <v>5093169</v>
       </c>
     </row>
     <row r="68">

</xml_diff>

<commit_message>
AutomaTivio: Infra Plus CDI com "Desde o início" no deck
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -13201,7 +13201,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4829395</v>
+        <v>4829390</v>
       </c>
     </row>
     <row r="45">
@@ -13231,7 +13231,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>5454373</v>
+        <v>5454372</v>
       </c>
     </row>
     <row r="47">
@@ -13261,7 +13261,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>16816509</v>
+        <v>16816511</v>
       </c>
     </row>
     <row r="49">
@@ -13291,7 +13291,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>15593110</v>
+        <v>15593109</v>
       </c>
     </row>
     <row r="51">
@@ -13321,7 +13321,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>15041378</v>
+        <v>15041376</v>
       </c>
     </row>
     <row r="53">
@@ -13381,7 +13381,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>23546226</v>
+        <v>23546225</v>
       </c>
     </row>
     <row r="57">
@@ -13441,7 +13441,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>26316814</v>
+        <v>26316813</v>
       </c>
     </row>
     <row r="61">
@@ -13501,7 +13501,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>26317597</v>
+        <v>26317598</v>
       </c>
     </row>
     <row r="65">
@@ -13516,7 +13516,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>3976310</v>
+        <v>4084345</v>
       </c>
     </row>
     <row r="66">
@@ -13531,7 +13531,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>87883521</v>
+        <v>87883493</v>
       </c>
     </row>
     <row r="67">
@@ -13546,7 +13546,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>5093169</v>
+        <v>5085546</v>
       </c>
     </row>
     <row r="68">

</xml_diff>

<commit_message>
AutomaTivio: caminho acima de 260 caracteres (Chromium e PowerPoint), rentabilidade da previdência com no máximo 2 casas, relatório do que é automático
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
+++ b/AutomaTivio/saida/2026-09/conferencia_2026-09.xlsx
@@ -13021,7 +13021,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2093594</v>
+        <v>2093590</v>
       </c>
     </row>
     <row r="33">
@@ -13201,7 +13201,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4829390</v>
+        <v>4829401</v>
       </c>
     </row>
     <row r="45">
@@ -13231,7 +13231,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>5454372</v>
+        <v>5454374</v>
       </c>
     </row>
     <row r="47">
@@ -13246,7 +13246,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>554378</v>
+        <v>554363</v>
       </c>
     </row>
     <row r="48">
@@ -13261,7 +13261,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>16816511</v>
+        <v>16816509</v>
       </c>
     </row>
     <row r="49">
@@ -13291,7 +13291,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>15593109</v>
+        <v>15593104</v>
       </c>
     </row>
     <row r="51">
@@ -13321,7 +13321,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>15041376</v>
+        <v>15041378</v>
       </c>
     </row>
     <row r="53">
@@ -13351,7 +13351,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>25551962</v>
+        <v>25551961</v>
       </c>
     </row>
     <row r="55">
@@ -13411,7 +13411,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>26316559</v>
+        <v>26316562</v>
       </c>
     </row>
     <row r="59">
@@ -13471,7 +13471,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>26457372</v>
+        <v>26457371</v>
       </c>
     </row>
     <row r="63">
@@ -13501,7 +13501,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>26317598</v>
+        <v>26317596</v>
       </c>
     </row>
     <row r="65">
@@ -13516,7 +13516,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>4084345</v>
+        <v>3976310</v>
       </c>
     </row>
     <row r="66">
@@ -13531,7 +13531,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>87883493</v>
+        <v>87883512</v>
       </c>
     </row>
     <row r="67">
@@ -13546,7 +13546,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>5085546</v>
+        <v>5093171</v>
       </c>
     </row>
     <row r="68">

</xml_diff>